<commit_message>
Add Figures 2.7-2.11 to the deviation register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -10,20 +10,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Cases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contradictions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Stack" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paper Edits" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To-Do" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Diagrams" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contradictions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Stack" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paper Edits" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To-Do" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$K$154</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Use Cases'!$A$1:$F$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contradictions'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tech Stack'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Paper Edits'!$A$1:$B$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'To-Do'!$A$1:$I$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Figures'!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Activity Diagrams'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Contradictions'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tech Stack'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Paper Edits'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'To-Do'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Figures'!$A$1:$D$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +557,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Reviewed: full manuscript text incl. 4 interview transcripts; Figures 2.2-2.6. Pending: Figures 2.7-2.15 images (activity diagram text already reviewed).</t>
+          <t>Reviewed: full manuscript text incl. 4 interview transcripts; Figures 2.2-2.11. Pending: Figures 2.12-2.15 images (their text is already reviewed).</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3106,7 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>In-platform bell works; no email notifications are sent (EmailJS is only used for OTP).</t>
+          <t>In-platform bell works; no email notifications are sent (EmailJS is only used for OTP). No notification at all when an order is placed (Fig 2.10 'Send Order Submission Notification').</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -3129,7 +3131,7 @@
       </c>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>p.51</t>
+          <t>p.51; Fig 2.10</t>
         </is>
       </c>
     </row>
@@ -6353,7 +6355,7 @@
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>Approve-and-credit matches Activity 2.11 and Interview 4; fix the bug and reword REQ098.</t>
+          <t>The paper says hold everywhere (REQ095, REQ098, Fig 2.6 text, Fig 2.11 text and diagram); approve-and-credit is what the client agreed to in the Interview 4 walkthrough. Fix the bug and reword the paper (C2).</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
@@ -9431,7 +9433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11182,7 +11184,7 @@
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>(no bubble) Wholesale Exchange / Free-of-Cost</t>
+          <t>(no bubble) Free-of-Cost Distribution</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
@@ -11197,17 +11199,385 @@
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>REQ090-091</t>
+          <t>REQ091</t>
         </is>
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>Paper: has Activity 2.15 but no use case in Fig 2.2 or 2.6.</t>
+          <t>Paper: no use case in any figure (wholesale exchange is in Fig 2.7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Manage Live Chat</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>REQ108-110</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>Connected here, but not in Fig 2.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Manage Product Catalog</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>REQ068-070</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>Dosage notes missing; category rename uses native prompt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Manage Supplier Accounts</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>REQ069</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>Manage Wholesale Accounts</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>REQ085-086</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>No document expiry tracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>&lt;&lt;extend&gt;&gt; Process Wholesale Exchange Request</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>REQ090</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>&lt;&lt;include&gt;&gt; Adjust Inventory for Exchange</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>REQ090</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Manage Online Customer Accounts</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>REQ116-117</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>No order history list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>View Audit Log</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>Technical Staff (+BM)</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>REQ123-124</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>Update Product Price</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>Branch Manager</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>REQ071-072</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>Non-BM staff can set prices on new/imported products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>&lt;&lt;include&gt;&gt; Record Price Change in Audit Log</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>Branch Manager</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>REQ073</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>No reason captured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>Create Staff Account &lt;&lt;include&gt;&gt; Assign Staff Role</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>Branch Manager</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>REQ118-119</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>Shared validators not applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>Manage Staff Accounts</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>Branch Manager</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>REQ118</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>Editing an Administrator silently changes it to Branch Manager.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F59"/>
+  <autoFilter ref="A1:F71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11218,7 +11588,977 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Step / flow</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Paper shows</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>System does</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Validate credentials -&gt; role redirect</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Valid login: customer to Home, staff to Dashboard</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Same (js/auth.js:94)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Failed attempts</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Increment count; at 5, lock 2 minutes; back to Login page</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Same (js/auth.js:57)</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Device recognition + OTP</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Check if device is recognized; if not, send and validate OTP</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Change system</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>REQ005/REQ044.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Wrong OTP</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Diagram: 'No' from Validate OTP joins the failed-attempt counter (counts toward lockout). Text p.77: user is prompted to request a new OTP.</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Diagram and text disagree (C13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Steps the system has that the diagram lacks</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Not shown</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>reCAPTCHA check, rejecting attempts while locked, blocking deactivated accounts, sending unverified customers to email verification</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Add to diagram; all are in requirements (REQ003, REQ004, REQ117, REQ002).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Validate fields -&gt; duplicate email -&gt; Terms -&gt; send code</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Fields validated, then duplicate check, then Terms shown and accepted, then code sent</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Terms modal opens when the checkbox is ticked (before submit); duplicate email is caught by Firebase at account creation; code sent after</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Same outcome, different order (C14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Wrong / expired code</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Loop back to Enter Code (diagram); text p.79 adds 'request a new code'</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Retry or Resend link (js/verify-email.js)</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Add Resend to diagram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>After verification</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Go to Login</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Goes straight to the shop, already signed in</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>C10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Account activation</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Account activated only after the code is verified</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Login account is created first with emailVerified:false; unverified customers are redirected to verification on login</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Functionally equivalent; note the REQ002 bypass issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Catalog -&gt; cart -&gt; checkout</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Browse, add to cart, updated cart summary, checkout</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Same, plus choosing which cart items to check out</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Cart selection is an addition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Default address</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>If saved, pre-fill; else enter</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Same (js/checkout.js)</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>RX check position</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Diagram: RX is checked after the address and after uploading payment proof, so RX customers are still asked for a delivery address. Text p.81: RX check comes before payment and delivery is not allowed.</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>RX detected when checkout opens; address section hidden; pick-up only</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Diagram contradicts REQ023 and its own text (C15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Prescription photo upload</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Not shown in the diagram (text p.81 and REQ021 require it)</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Required on the payment page for RX orders</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>C15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Order status after submission</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Recorded as Pending Payment Verification (RX included)</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Same ('placed' = Order Pending Verification)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Diagram supports the system; REQ024 says 'Pending Prescription Verification' (C3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Order submission notification</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>System sends a notification to the customer</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Only an on-screen confirmation with the order number; no notification</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Change system</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Small: add an order-placed entry to the customer bell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Steps the system has that the diagram lacks</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Not shown</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Login required to check out, delivery schedule, store credit discount, live stock re-check before submitting</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Optional: add to diagram (delivery schedule is in Modules p.39).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Valid payment</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Confirm -&gt; notify customer -&gt; FEFO stock deduction -&gt; receipt</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Stock is deducted first; if stock ran out the order goes on an Out of Stock hold instead</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Diagram has no out-of-stock path (C19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>RX pre-order after confirmation</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Diagram: admin copies delivery details, books courier and provides a tracking link before the system checks for RX</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>RX orders skip courier booking and go straight to Ready for Pick-up</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>RX orders can't be delivered (REQ080) (C17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Prescription review</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Not shown (payment screenshot only)</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Not built (payment approval only)</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Change system</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>REQ077-079 require it (C3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Admin provides tracking link; system marks Dispatched</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Admin pastes the link and marks Dispatched in one step; customer can't see the link</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Change system</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>REQ034.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Invalid payment</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>On Hold -&gt; record reason -&gt; notify customer -&gt; re-upload -&gt; back to admin review</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Same (js/admin-online-orders.js:561; js/order-details.js)</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Resolution without re-upload</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Diagram: if the customer 'performed resolution action', the system confirms the order with no admin review</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Every resolution returns to staff (resubmission or Release Hold)</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Diagram contradicts REQ101 (C18).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Overpayment</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Treated as an invalid payment (hold)</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Approved immediately; excess added to store credit</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>C2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Expired hold</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Admin marks the order Unresolved</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Closed automatically after 7 days, with verified payment kept as credit</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Change paper</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>REQ100 says automatic; move step to System lane and add credit retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Steps the system has that the diagram lacks</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Not shown</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Fully credit-covered orders (no screenshot), Release Hold by staff</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Deviates</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Optional to add.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11295,7 +12635,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>REQ095 and REQ098 ('On Hold - Overpayment') vs Activity 2.11 and Payment Verification Module (excess recorded as unapplied value) vs Interview 4 (excess goes to customer's account for next order)</t>
+          <t>REQ095, REQ098, Fig 2.6 text and Fig 2.11 text + diagram all treat overpayment as a hold (excess recorded as unapplied value) vs Interview 4 walkthrough (enter the excess; it goes to the customer's account for the next order; client agreed)</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
@@ -11305,7 +12645,7 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Change paper: rewrite REQ098 to approve-and-credit; drop overpayment from the hold types.</t>
+          <t>Change paper: rewrite REQ098 and Fig 2.6/2.11 to approve-and-credit; drop overpayment from the hold types.</t>
         </is>
       </c>
     </row>
@@ -11322,17 +12662,17 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>REQ024, REQ077-079, Modules p.43, Conceptual Framework (dedicated RX queue, approve/reject with reason) vs Activity 2.11 (RX pre-orders 'confirmed in the same manner', verification in person)</t>
+          <t>REQ024, REQ077-079, Modules p.43, Conceptual Framework, Fig 2.10 text (dedicated RX queue, 'Pending Prescription Verification', approve/reject with reason) vs Fig 2.10 diagram (RX recorded as Pending Payment Verification) and Fig 2.11 text + diagram (RX confirmed like any order, verification in person)</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Same as Activity 2.11 (payment approval only).</t>
+          <t>Same as Fig 2.10/2.11 diagrams (payment approval only).</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Change system to match REQ077-079; fix Activity 2.11 text.</t>
+          <t>Change system to match REQ077-079; then fix Fig 2.10 and 2.11.</t>
         </is>
       </c>
     </row>
@@ -11511,7 +12851,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Activity 2.9 (after verification, redirect to login page)</t>
+          <t>Fig 2.9 text + diagram (after verification, go to Login)</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -11538,7 +12878,7 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 has no Create Purchase Order, Batch Upload, Verify Prescription, Payment Verification, Delivery, Customer Accounts, Suppliers, Notifications, Wholesale Exchange; 'Manage Live Chat' has no actor</t>
+          <t>Fig 2.2 has no Create Purchase Order, Batch Upload, Verify Prescription, Payment Verification, Delivery, Customer Accounts, Suppliers, Notifications, Wholesale Exchange (all appear in Figs 2.5-2.7); 'Manage Live Chat' has no actor in 2.2 but is linked to Technical Staff in 2.7</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -11548,7 +12888,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Change paper: add the missing bubbles or say Fig 2.2 is a summary.</t>
+          <t>Change paper: add the missing bubbles to 2.2 or say it's a summary; connect Manage Live Chat.</t>
         </is>
       </c>
     </row>
@@ -11579,13 +12919,202 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Wrong OTP at login</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.8 diagram (wrong OTP feeds the failed-attempt counter) vs Fig 2.8 text p.77 (prompted to request a new OTP)</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>No OTP yet.</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Pick one when building REQ005/044; update the other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Registration order</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.9 (validate, duplicate check, then Terms) vs system (Terms when ticking the checkbox, duplicate check at account creation)</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>See left.</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Change paper: Terms before submit; duplicate check after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>RX in the purchasing flow</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.10 diagram (RX checked after address and payment upload; no prescription upload) vs Fig 2.10 text p.81 and REQ021/023 (RX decided first, pick-up only, prescription photo required)</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Matches the text, not the diagram.</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Change paper: redraw the RX branch in Fig 2.10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Order submission notification</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.10 (system notifies customer on submission) vs REQ039 (order confirmations)</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>No notification on submission.</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Change system (small).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>RX pre-orders and couriers</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.11 diagram (courier booked and tracking link sent before the RX check) vs REQ023/080 (never delivered)</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>RX skips courier booking.</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Change paper: branch RX before the courier steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Resolving a hold</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.11 diagram (customer resolution without re-upload confirms the order automatically) vs REQ101 (admin approval confirms)</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Every resolution goes back to staff.</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Change paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Stock check at confirmation</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Fig 2.11 (notify confirmed, then FEFO deduction; no shortage path) vs REQ050</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Deducts first; shortage puts the order on an Out of Stock hold.</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Change paper: add the out-of-stock hold branch.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11919,13 +13448,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12091,76 +13620,112 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 text p.79</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>After verification the customer goes to the shop, already signed in (C10).</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 text p.83</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Prescription pre-orders need prescription approval/rejection before confirmation (C3) - after it is built.</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
+          <t>Fig 2.11 diagram + text p.82-83</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Modules FEFO p.41</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Add the 2-month Bad Order step (C7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Technical Background p.35-37; Budget p.99</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>Decision-dependent</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B18"/>
+  <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14013,54 +15578,95 @@
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>REQ039, Fig 2.10, C16</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Change system</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr"/>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
           <t>Apply all paper edits (see Paper Edits sheet)</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>Paper Edits sheet</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
       </c>
-      <c r="E44" s="11" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>Change paper</t>
         </is>
       </c>
-      <c r="F44" s="11" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H44" s="11" t="inlineStr">
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>Do after system decisions are final.</t>
         </is>
       </c>
-      <c r="I44" s="11" t="inlineStr">
+      <c r="I45" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I44"/>
-  <conditionalFormatting sqref="I2:I44">
+  <autoFilter ref="A1:I45"/>
+  <conditionalFormatting sqref="I2:I45">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14068,7 +15674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14228,10 +15834,14 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr"/>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -14246,12 +15856,12 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Text reviewed (p.76-77)</t>
+          <t>Reviewed</t>
         </is>
       </c>
     </row>
@@ -14268,12 +15878,12 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Text reviewed (p.78-79)</t>
+          <t>Reviewed</t>
         </is>
       </c>
     </row>
@@ -14290,12 +15900,12 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Text reviewed (p.80-81)</t>
+          <t>Reviewed</t>
         </is>
       </c>
     </row>
@@ -14312,12 +15922,12 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Text reviewed (p.82-83)</t>
+          <t>Reviewed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record team decisions in the register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
+          <t>DECIDED: build it with OpenAI via a Netlify Function (panel's recommended feature). Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr"/>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Orders access was added on purpose on 2026-10-01.</t>
+          <t>DECIDED: trim to POS + catalog view; Walk-in history inside POS. Orders access was added on purpose on 2026-10-01.</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr"/>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -4553,7 +4553,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: live on verification queue + customer order page only; reword REQNF005 for the rest.</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="inlineStr"/>
       <c r="J21" s="11" t="inlineStr">
         <is>
@@ -4567,7 +4571,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -4595,7 +4599,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr"/>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: Netlify (already set up).</t>
+        </is>
+      </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="11" t="inlineStr">
         <is>
@@ -4609,7 +4617,7 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -4639,13 +4647,13 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Not in the paper; client gives boss-approved discounts today.</t>
+          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr"/>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4663,7 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -4685,13 +4693,13 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -6955,7 +6963,7 @@
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
@@ -6983,11 +6991,15 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H76" s="11" t="inlineStr"/>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: leave as is; state in Limitations.</t>
+        </is>
+      </c>
       <c r="I76" s="11" t="inlineStr"/>
       <c r="J76" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -6997,7 +7009,7 @@
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
@@ -7027,13 +7039,13 @@
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>Client's current POS practice; not in the paper.</t>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
         </is>
       </c>
       <c r="I77" s="11" t="inlineStr"/>
       <c r="J77" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7055,7 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
@@ -7073,13 +7085,13 @@
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>Not in the paper; ask the client if the main office tracks collections instead.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I78" s="11" t="inlineStr"/>
       <c r="J78" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7101,7 @@
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
@@ -7119,13 +7131,13 @@
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr"/>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8217,7 +8229,7 @@
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DECIDED: build it with OpenAI via a Netlify Function (panel's recommended feature). See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr"/>
@@ -9079,7 +9091,7 @@
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,In progress,Done,Dropped"</formula1>
+      <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22126,17 +22138,17 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>Not hosted; local http-server via start-server.bat</t>
+          <t>Netlify (set up); local http-server for testing</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Netlify blocked by billing. Options: Firebase Hosting (free, HTTPS) and update the paper, or present locally and move hosting to Limitations.</t>
+          <t>DECIDED: stay on Netlify. Budget row must match the chosen plan; Netlify Functions host the OpenAI call.</t>
         </is>
       </c>
     </row>
@@ -22234,17 +22246,17 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Not integrated</t>
+          <t>Not integrated yet</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>Change system</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Needs a server-side function to keep the API key secret.</t>
+          <t>DECIDED: OpenAI through a Netlify Function so the key stays secret. Budget: add OpenAI usage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record build-to-avoid-letter decisions and Gemini for the chat (fix)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$131</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K124"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it with OpenAI via a Netlify Function (panel's recommended feature). Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr">
@@ -4899,22 +4899,22 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Objectives / evaluation (p.5-6, 21-24)</t>
+          <t>Removals (Letter) sheet</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
+          <t>Letter to the panel: OpenAI -&gt; Gemini (free), Firebase Storage -&gt; Cloudinary, DataTable -&gt; custom tables, password reset via Firebase Auth, overpayment approve-and-credit, corrections to scope/conceptual framework</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -4922,10 +4922,14 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr"/>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>One letter covers all remaining removals; send before the paper edits.</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr"/>
@@ -4941,42 +4945,38 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>REQ121</t>
+          <t>Objectives / evaluation (p.5-6, 21-24)</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
+          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Med</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: trim to POS + catalog view; Walk-in history inside POS. Orders access was added on purpose on 2026-10-01.</t>
-        </is>
-      </c>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr"/>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr"/>
@@ -4997,12 +4997,12 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>REQNF005</t>
+          <t>REQ121</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Live updates without refresh on verification queue + customer order page</t>
+          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -5022,12 +5022,12 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: live on verification queue + customer order page only; reword REQNF005 for the rest.</t>
-        </is>
-      </c>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DECIDED: trim to POS + catalog view; Walk-in history inside POS. Orders access was added on purpose on 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr"/>
@@ -5048,22 +5048,22 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>REQNF010, REQNF013</t>
+          <t>REQNF005</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
+          <t>Live updates without refresh on all order and inventory screens (staff + customer)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -5073,12 +5073,12 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: Netlify (already set up).</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>DECIDED (revised): build everywhere to avoid a removal letter.</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr"/>
@@ -5099,12 +5099,12 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
+          <t>REQNF010, REQNF013</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Discount / deduction per sale or line, with reason and audit entry</t>
+          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -5124,18 +5124,18 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
+          <t>DECIDED: Netlify (already set up).</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr"/>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5150,12 +5150,12 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
+          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
+          <t>Discount / deduction per sale or line, with reason and audit entry</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -5175,18 +5175,18 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr"/>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -5196,27 +5196,27 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Limitations (p.7)</t>
+          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
+          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -5224,7 +5224,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr"/>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+        </is>
+      </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5233,7 +5237,7 @@
       <c r="J25" s="11" t="inlineStr"/>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5257,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
+          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -5295,12 +5299,12 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Limitations (p.7)</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
+          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -5337,22 +5341,22 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
+          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
@@ -5365,11 +5369,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H28" s="11" t="inlineStr"/>
       <c r="I28" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5393,12 +5393,12 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>REQ002</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
+          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -5444,22 +5444,22 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
+          <t>REQ002</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Unrecognized-device OTP for customers and staff</t>
+          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -5467,7 +5467,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr"/>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5491,17 +5495,17 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>REQ086, REQ089, REQ091, REQ092</t>
+          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
+          <t>Unrecognized-device OTP for customers and staff</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -5514,11 +5518,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
-        </is>
-      </c>
+      <c r="H31" s="11" t="inlineStr"/>
       <c r="I31" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5542,17 +5542,17 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>REQ090, REQ114, Fig 2.15</t>
+          <t>REQ086, REQ089, REQ091, REQ092</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
+          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -5565,7 +5565,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr"/>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
+        </is>
+      </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5589,12 +5593,12 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>REQ067, C7</t>
+          <t>REQ090, REQ114, Fig 2.15</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
+          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
@@ -5636,12 +5640,12 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
+          <t>REQ067, C7</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
+          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -5651,7 +5655,7 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
@@ -5683,12 +5687,12 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>REQ084</t>
+          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>POS: RX Verified checkbox + optional notes</t>
+          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -5730,17 +5734,17 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>REQ061, C5</t>
+          <t>REQ084</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
+          <t>POS: RX Verified checkbox + optional notes</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
@@ -5777,17 +5781,17 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>REQNF025, REQNF029</t>
+          <t>REQ061, C5</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
+          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
@@ -5800,11 +5804,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H37" s="11" t="inlineStr"/>
       <c r="I37" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5828,22 +5828,22 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>REQ039, REQ042</t>
+          <t>REQNF025, REQNF029</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
+          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -5853,7 +5853,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>EmailJS free tier: 200/month.</t>
+          <t>From the first review.</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -5879,12 +5879,12 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>REQ122</t>
+          <t>REQ039, REQ042</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
+          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -5902,7 +5902,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr"/>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>EmailJS free tier: 200/month.</t>
+        </is>
+      </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5926,22 +5930,22 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>REQ014</t>
+          <t>REQ122</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Save cart to the customer's account</t>
+          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -5973,17 +5977,17 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>REQNF003, REQNF007</t>
+          <t>REQ014</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Phone/tablet and cross-browser test pass</t>
+          <t>Save cart to the customer's account</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
@@ -6020,17 +6024,17 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Interviews 2, 4</t>
+          <t>REQNF003, REQNF007</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
+          <t>Phone/tablet and cross-browser test pass</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Not verified</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
@@ -6043,11 +6047,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H42" s="11" t="inlineStr">
-        <is>
-          <t>Required column in the monthly purchases report.</t>
-        </is>
-      </c>
+      <c r="H42" s="11" t="inlineStr"/>
       <c r="I42" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6071,12 +6071,12 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Interview 4 walkthrough</t>
+          <t>Interviews 2, 4</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Supplier history: everything received from each supplier</t>
+          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>Shown to the client during the prototype walkthrough.</t>
+          <t>Required column in the monthly purchases report.</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
@@ -6122,12 +6122,12 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30; Interview 4</t>
+          <t>Interview 4 walkthrough</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>User manual + hands-on training + handover to the branch</t>
+          <t>Supplier history: everything received from each supplier</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
+          <t>Shown to the client during the prototype walkthrough.</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
@@ -6173,12 +6173,12 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
+          <t>Methodology p.30; Interview 4</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
+          <t>User manual + hands-on training + handover to the branch</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>Customer File groups every sale by customer name.</t>
+          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
@@ -6224,17 +6224,17 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Supplier sheets)</t>
+          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
+          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
+          <t>Customer File groups every sale by customer name.</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
+          <t>Report Formats sheet (Supplier sheets)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
+          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+          <t>Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
@@ -6326,17 +6326,17 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
@@ -6349,7 +6349,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H48" s="11" t="inlineStr"/>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+        </is>
+      </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6373,22 +6377,22 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>REQ085, REQ087</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Optional agreed price per wholesale buyer per product, used as default on their orders</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -6396,10 +6400,14 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr"/>
-      <c r="I49" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>Keeps per-account pricing (no letter).</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr"/>
@@ -6420,22 +6428,22 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>Production readiness</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>Cut database reads: stop loading whole collections on every page (Firestore free-plan daily read cap ~50k)</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr">
@@ -6443,7 +6451,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H50" s="11" t="inlineStr"/>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>Needed before real use with the client's ~1,000-product catalog.</t>
+        </is>
+      </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6462,17 +6474,17 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -6493,7 +6505,7 @@
       <c r="H51" s="11" t="inlineStr"/>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr"/>
@@ -6509,22 +6521,22 @@
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
@@ -6537,14 +6549,10 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H52" s="11" t="inlineStr"/>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr"/>
@@ -6560,22 +6568,22 @@
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
@@ -6588,14 +6596,10 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I53" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H53" s="11" t="inlineStr"/>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr"/>
@@ -6611,22 +6615,22 @@
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
@@ -6639,14 +6643,10 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H54" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I54" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H54" s="11" t="inlineStr"/>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr"/>
@@ -6667,12 +6667,12 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
@@ -6718,12 +6718,12 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -6746,9 +6746,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I56" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr"/>
@@ -6769,12 +6769,12 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
@@ -6820,12 +6820,12 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
@@ -6848,9 +6848,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I58" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr"/>
@@ -6871,12 +6871,12 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
@@ -6922,12 +6922,12 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -6950,9 +6950,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr"/>
@@ -6973,12 +6973,12 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
@@ -7001,9 +7001,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I61" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr"/>
@@ -7024,12 +7024,12 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -7075,12 +7075,12 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
@@ -7126,12 +7126,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -7177,12 +7177,12 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
@@ -7228,12 +7228,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -7279,12 +7279,12 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
@@ -7330,12 +7330,12 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -7381,17 +7381,17 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F69" s="11" t="inlineStr">
@@ -7404,7 +7404,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H69" s="11" t="inlineStr"/>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7428,22 +7432,22 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G70" s="11" t="inlineStr">
@@ -7451,7 +7455,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H70" s="11" t="inlineStr"/>
+      <c r="H70" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7475,17 +7483,17 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
@@ -7498,7 +7506,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H71" s="11" t="inlineStr"/>
+      <c r="H71" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7522,12 +7534,12 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -7546,9 +7558,9 @@
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr"/>
-      <c r="I72" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr"/>
@@ -7569,12 +7581,12 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
@@ -7584,7 +7596,7 @@
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
@@ -7616,12 +7628,12 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -7663,12 +7675,12 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
@@ -7687,9 +7699,9 @@
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr"/>
-      <c r="I75" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I75" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J75" s="11" t="inlineStr"/>
@@ -7705,48 +7717,44 @@
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H76" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: leave as is; state in Limitations.</t>
-        </is>
-      </c>
-      <c r="I76" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES - letter (REQ088 to Limitations)</t>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H76" s="11" t="inlineStr"/>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr"/>
       <c r="K76" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7756,48 +7764,44 @@
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F77" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G77" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H77" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="inlineStr"/>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J77" s="11" t="inlineStr"/>
       <c r="K77" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7807,48 +7811,44 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H78" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H78" s="11" t="inlineStr"/>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J78" s="11" t="inlineStr"/>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7863,22 +7863,22 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G79" s="11" t="inlineStr">
@@ -7888,18 +7888,18 @@
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7909,27 +7909,27 @@
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G80" s="11" t="inlineStr">
@@ -7937,16 +7937,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H80" s="11" t="inlineStr"/>
+      <c r="H80" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
+        </is>
+      </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr"/>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -7961,12 +7965,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
@@ -7976,7 +7980,7 @@
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
@@ -7984,16 +7988,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H81" s="11" t="inlineStr"/>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
+        </is>
+      </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr"/>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8008,17 +8016,17 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
@@ -8031,16 +8039,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H82" s="11" t="inlineStr"/>
+      <c r="H82" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+        </is>
+      </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr"/>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8050,22 +8062,22 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
@@ -8078,11 +8090,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H83" s="11" t="inlineStr">
-        <is>
-          <t>Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
-        </is>
-      </c>
+      <c r="H83" s="11" t="inlineStr"/>
       <c r="I83" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8106,17 +8114,17 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
@@ -8153,17 +8161,17 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F85" s="11" t="inlineStr">
@@ -8176,11 +8184,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H85" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H85" s="11" t="inlineStr"/>
       <c r="I85" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8204,17 +8208,17 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
@@ -8229,7 +8233,7 @@
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
@@ -8255,12 +8259,12 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
@@ -8278,11 +8282,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H87" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H87" s="11" t="inlineStr"/>
       <c r="I87" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8306,17 +8306,17 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
@@ -8329,7 +8329,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H88" s="11" t="inlineStr"/>
+      <c r="H88" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8353,17 +8357,17 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
@@ -8376,7 +8380,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H89" s="11" t="inlineStr"/>
+      <c r="H89" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8400,12 +8408,12 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -8423,7 +8431,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H90" s="11" t="inlineStr"/>
+      <c r="H90" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8447,17 +8459,17 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F91" s="11" t="inlineStr">
@@ -8494,12 +8506,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -8541,17 +8553,17 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
@@ -8564,11 +8576,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H93" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H93" s="11" t="inlineStr"/>
       <c r="I93" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8592,12 +8600,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -8615,11 +8623,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H94" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H94" s="11" t="inlineStr"/>
       <c r="I94" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8643,17 +8647,17 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F95" s="11" t="inlineStr">
@@ -8666,11 +8670,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H95" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H95" s="11" t="inlineStr"/>
       <c r="I95" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8694,17 +8694,17 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Store announcement banner (e.g. closure days)</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
@@ -8717,7 +8717,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H96" s="11" t="inlineStr"/>
+      <c r="H96" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8741,12 +8745,12 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
@@ -8764,7 +8768,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H97" s="11" t="inlineStr"/>
+      <c r="H97" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I97" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8788,17 +8796,17 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -8811,7 +8819,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H98" s="11" t="inlineStr"/>
+      <c r="H98" s="11" t="inlineStr">
+        <is>
+          <t>From the first review.</t>
+        </is>
+      </c>
       <c r="I98" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8830,22 +8842,22 @@
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F99" s="11" t="inlineStr">
@@ -8861,7 +8873,7 @@
       <c r="H99" s="11" t="inlineStr"/>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J99" s="11" t="inlineStr"/>
@@ -8877,22 +8889,22 @@
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
@@ -8907,12 +8919,12 @@
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J100" s="11" t="inlineStr"/>
@@ -8928,22 +8940,22 @@
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F101" s="11" t="inlineStr">
@@ -8958,12 +8970,12 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I101" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Keeps the Chart.js claim (no letter).</t>
+        </is>
+      </c>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J101" s="11" t="inlineStr"/>
@@ -8979,22 +8991,22 @@
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
@@ -9009,12 +9021,12 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Keeps 'price locking' (no letter).</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J102" s="11" t="inlineStr"/>
@@ -9030,22 +9042,22 @@
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F103" s="11" t="inlineStr">
@@ -9060,12 +9072,12 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Keeps the 'push notifications' claim (no letter).</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J103" s="11" t="inlineStr"/>
@@ -9081,22 +9093,22 @@
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
@@ -9109,14 +9121,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H104" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: build it with OpenAI via a Netlify Function (panel's recommended feature). See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H104" s="11" t="inlineStr"/>
       <c r="I104" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J104" s="11" t="inlineStr"/>
@@ -9132,17 +9140,17 @@
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
@@ -9163,7 +9171,7 @@
       <c r="H105" s="11" t="inlineStr"/>
       <c r="I105" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J105" s="11" t="inlineStr"/>
@@ -9179,17 +9187,17 @@
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
@@ -9208,9 +9216,9 @@
         </is>
       </c>
       <c r="H106" s="11" t="inlineStr"/>
-      <c r="I106" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I106" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J106" s="11" t="inlineStr"/>
@@ -9231,17 +9239,17 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F107" s="11" t="inlineStr">
@@ -9254,10 +9262,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H107" s="11" t="inlineStr"/>
-      <c r="I107" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H107" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I107" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J107" s="11" t="inlineStr"/>
@@ -9278,17 +9290,17 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
@@ -9301,10 +9313,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H108" s="11" t="inlineStr"/>
-      <c r="I108" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H108" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I108" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J108" s="11" t="inlineStr"/>
@@ -9325,17 +9341,17 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F109" s="11" t="inlineStr">
@@ -9348,10 +9364,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H109" s="11" t="inlineStr"/>
+      <c r="H109" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I109" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J109" s="11" t="inlineStr"/>
@@ -9372,17 +9392,17 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F110" s="11" t="inlineStr">
@@ -9395,10 +9415,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H110" s="11" t="inlineStr"/>
-      <c r="I110" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H110" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I110" s="11" t="inlineStr">
+        <is>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr"/>
@@ -9419,17 +9443,17 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F111" s="11" t="inlineStr">
@@ -9442,10 +9466,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H111" s="11" t="inlineStr"/>
-      <c r="I111" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H111" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I111" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J111" s="11" t="inlineStr"/>
@@ -9466,12 +9494,12 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -9490,9 +9518,9 @@
         </is>
       </c>
       <c r="H112" s="11" t="inlineStr"/>
-      <c r="I112" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I112" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J112" s="11" t="inlineStr"/>
@@ -9513,12 +9541,12 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -9537,9 +9565,9 @@
         </is>
       </c>
       <c r="H113" s="11" t="inlineStr"/>
-      <c r="I113" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I113" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J113" s="11" t="inlineStr"/>
@@ -9560,12 +9588,12 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
@@ -9584,9 +9612,9 @@
         </is>
       </c>
       <c r="H114" s="11" t="inlineStr"/>
-      <c r="I114" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I114" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J114" s="11" t="inlineStr"/>
@@ -9607,12 +9635,12 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
@@ -9631,9 +9659,9 @@
         </is>
       </c>
       <c r="H115" s="11" t="inlineStr"/>
-      <c r="I115" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I115" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J115" s="11" t="inlineStr"/>
@@ -9654,12 +9682,12 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
@@ -9701,12 +9729,12 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
@@ -9725,9 +9753,9 @@
         </is>
       </c>
       <c r="H117" s="11" t="inlineStr"/>
-      <c r="I117" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I117" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J117" s="11" t="inlineStr"/>
@@ -9748,12 +9776,12 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
@@ -9772,9 +9800,9 @@
         </is>
       </c>
       <c r="H118" s="11" t="inlineStr"/>
-      <c r="I118" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I118" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J118" s="11" t="inlineStr"/>
@@ -9795,12 +9823,12 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -9819,9 +9847,9 @@
         </is>
       </c>
       <c r="H119" s="11" t="inlineStr"/>
-      <c r="I119" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I119" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J119" s="11" t="inlineStr"/>
@@ -9842,12 +9870,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
@@ -9868,7 +9896,7 @@
       <c r="H120" s="11" t="inlineStr"/>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J120" s="11" t="inlineStr"/>
@@ -9889,12 +9917,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -9936,12 +9964,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -9960,9 +9988,9 @@
         </is>
       </c>
       <c r="H122" s="11" t="inlineStr"/>
-      <c r="I122" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I122" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J122" s="11" t="inlineStr"/>
@@ -9983,12 +10011,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -10030,12 +10058,12 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
@@ -10066,18 +10094,347 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="11" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>Budgetary Estimate (p.99)</t>
+        </is>
+      </c>
+      <c r="D125" s="11" t="inlineStr">
+        <is>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+        </is>
+      </c>
+      <c r="E125" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G125" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H125" s="11" t="inlineStr"/>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J125" s="11" t="inlineStr"/>
+      <c r="K125" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>Budgetary Estimate (p.99)</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+        </is>
+      </c>
+      <c r="E126" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F126" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G126" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H126" s="11" t="inlineStr"/>
+      <c r="I126" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J126" s="11" t="inlineStr"/>
+      <c r="K126" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>References (p.100)</t>
+        </is>
+      </c>
+      <c r="D127" s="11" t="inlineStr">
+        <is>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+        </is>
+      </c>
+      <c r="E127" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F127" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G127" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H127" s="11" t="inlineStr"/>
+      <c r="I127" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J127" s="11" t="inlineStr"/>
+      <c r="K127" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>References (p.10 / refs)</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+        </is>
+      </c>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F128" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G128" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H128" s="11" t="inlineStr"/>
+      <c r="I128" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J128" s="11" t="inlineStr"/>
+      <c r="K128" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>References (p.17 / refs)</t>
+        </is>
+      </c>
+      <c r="D129" s="11" t="inlineStr">
+        <is>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+        </is>
+      </c>
+      <c r="E129" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F129" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G129" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H129" s="11" t="inlineStr"/>
+      <c r="I129" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J129" s="11" t="inlineStr"/>
+      <c r="K129" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>Appendices (p.124)</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+        </is>
+      </c>
+      <c r="E130" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F130" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G130" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H130" s="11" t="inlineStr"/>
+      <c r="I130" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J130" s="11" t="inlineStr"/>
+      <c r="K130" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D131" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E131" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F131" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G131" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H131" s="11" t="inlineStr"/>
+      <c r="I131" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J131" s="11" t="inlineStr"/>
+      <c r="K131" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K124"/>
-  <conditionalFormatting sqref="K2:K124">
+  <autoFilter ref="A1:K131"/>
+  <conditionalFormatting sqref="K2:K131">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23243,7 +23600,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: OpenAI through a Netlify Function so the key stays secret. Budget: add OpenAI usage.</t>
+          <t>DECIDED: Gemini via Firebase AI Logic (free tier, no server needed); Groq as fallback. In the panel letter.</t>
         </is>
       </c>
     </row>
@@ -23899,7 +24256,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Build - no letter (S)</t>
+          <t>Building - no letter (S)</t>
         </is>
       </c>
     </row>
@@ -23926,7 +24283,7 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Build - no letter (S)</t>
+          <t>Building - no letter (S)</t>
         </is>
       </c>
     </row>
@@ -23953,7 +24310,7 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Build - no letter (M)</t>
+          <t>Building - no letter (M)</t>
         </is>
       </c>
     </row>
@@ -23980,7 +24337,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser</t>
+          <t>In letter (as a refinement the client approved)</t>
         </is>
       </c>
     </row>
@@ -24007,7 +24364,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Reconsider the decision - build (M), no letter</t>
+          <t>Building - no letter (M)</t>
         </is>
       </c>
     </row>
@@ -24034,7 +24391,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Build if time (M); otherwise letter</t>
+          <t>Building - no letter (M)</t>
         </is>
       </c>
     </row>
@@ -24061,7 +24418,7 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser (framework wording, not a requirement)</t>
+          <t>Building - no letter (S)</t>
         </is>
       </c>
     </row>
@@ -24088,7 +24445,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Build - no letter (S)</t>
+          <t>Building - no letter (S)</t>
         </is>
       </c>
     </row>
@@ -24115,7 +24472,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Build - no letter (S)</t>
+          <t>Building - no letter (S)</t>
         </is>
       </c>
     </row>
@@ -24142,7 +24499,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser - tool replacement, not a feature removal</t>
+          <t>In letter (same letter as the other tool swaps)</t>
         </is>
       </c>
     </row>
@@ -24169,7 +24526,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser - tool change</t>
+          <t>In letter</t>
         </is>
       </c>
     </row>
@@ -24196,7 +24553,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser - tool replacement</t>
+          <t>In letter</t>
         </is>
       </c>
     </row>
@@ -24223,7 +24580,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser - tool replacement (minor)</t>
+          <t>In letter</t>
         </is>
       </c>
     </row>
@@ -24250,7 +24607,7 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Ask adviser - correction of an error</t>
+          <t>In letter (correction)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: mark foundation items done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4226,7 +4226,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Title feature.</t>
+          <t>DONE e1e200b. Title feature.</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
@@ -4237,7 +4237,7 @@
       <c r="J5" s="11" t="inlineStr"/>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Client is not BIR-connected by choice and issues BIR/VAT receipts manually on request.</t>
+          <t>DONE e1e200b. Client is not BIR-connected by choice and issues BIR/VAT receipts manually on request.</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -4531,7 +4531,7 @@
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4622,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Every client report lists batch + expiry per sold line; today FEFO deducts the right batch but the sale doesn't remember which. Blocks the Reports module.</t>
+          <t>DONE e1e200b. Every client report lists batch + expiry per sold line; today FEFO deducts the right batch but the sale doesn't remember which. Blocks the Reports module.</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
@@ -4633,7 +4633,7 @@
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Replaces the separate 'receipt numbers' item; voids reference it.</t>
+          <t>DONE e1e200b. Replaces the separate 'receipt numbers' item; voids reference it.</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -4684,7 +4684,7 @@
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Credit was ₱57,534 of ₱81,181 on the sample day.</t>
+          <t>DONE e1e200b. Credit was ₱57,534 of ₱81,181 on the sample day.</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
@@ -4735,7 +4735,7 @@
       <c r="J15" s="11" t="inlineStr"/>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE e1e200b (system part; REQ098 paper wording still to do). From the first review.</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
@@ -4837,7 +4837,7 @@
       <c r="J17" s="11" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>Customer File groups every sale by customer name.</t>
+          <t>DONE e1e200b. Customer File groups every sale by customer name.</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
@@ -6260,7 +6260,7 @@
       <c r="J46" s="11" t="inlineStr"/>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6300,7 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
+          <t>DONE e1e200b: unit cost + receipt/DR no. added; pack size stays in the product name as the branch does today. Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
@@ -6311,7 +6311,7 @@
       <c r="J47" s="11" t="inlineStr"/>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+          <t>DONE e1e200b: also storefront links/filters now follow Manage Categories. Existing Firebase projects keep their current categories - add the client's in Manage Categories.. Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
@@ -6362,7 +6362,7 @@
       <c r="J48" s="11" t="inlineStr"/>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Manage Categories: add the branch's categories, move products when deleting a category
Deleting a category that still has products now asks where to move them
and moves them in the same step, so the old default categories can be
replaced. Category rename uses the app's own dialog instead of the
browser prompt (new showAppPrompt / showAppSelect helpers).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -8382,7 +8382,7 @@
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I89" s="11" t="inlineStr">
@@ -8393,7 +8393,7 @@
       <c r="J89" s="11" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show tracking link to customers; wire product search and price/stock filters
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4373,7 +4373,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>DONE customer order page shows a 'Track with Lalamove' card once dispatched.</t>
+        </is>
+      </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -4382,7 +4386,7 @@
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4475,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>DONE header search on every shop page -&gt; catalog keyword search (name, generic, brand, description); price range + availability filters.</t>
+        </is>
+      </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -4480,7 +4488,7 @@
       <c r="J10" s="11" t="inlineStr"/>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Terms & Privacy rewritten to the branch's policies; shared footer; hide unbuilt chat links
- js/legal-content.js is the one source for the sign-up pop-up and a new
  public legal.html: no refunds/exchange only, no cancellation after
  payment, 7-day holds and store credit, rider-paid delivery fees,
  prescription pick-up only, non-official receipts, AI chat limits, and
  the Data Privacy Act.
- Every page footer now comes from js/store-info.js: real About text,
  working Privacy/Terms links; the placeholder hotline, email and FDA LTO
  number are gone until the client confirms the real ones.
- Header search moved to store-info.js so it also works on the sign-in
  pages.
- Live Chat sidebar link and storefront chat buttons are hidden until the
  chat module exists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -3568,7 +3568,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Get from the client: the QR Ph image and the sales invoice format (sample reports received). Ask them: are all sales VAT-exempt (sample shows VATable 0.00), is pay-in/pay-out used, who tracks credit collections, which categories to use, may we load the real catalog for the demo?</t>
+          <t>Get from the client: the QR Ph image, the sales invoice format, and the store details for the footer (hotline, email, hours, address, FDA LTO No. - fill js/store-info.js); have them review the Terms/Privacy text. Ask them: are all sales VAT-exempt (sample shows VATable 0.00), is pay-in/pay-out used, who tracks credit collections, which categories to use, may we load the real catalog for the demo?</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Get from the client: the QR Ph image and the sales invoice format (sample reports received). Ask them: are all sales VAT-exempt (sample shows VATable 0.00), is pay-in/pay-out used, who tracks credit collections, which categories to use, may we load the real catalog for the demo?</t>
+          <t>Get from the client: the QR Ph image, the sales invoice format, and the store details for the footer (hotline, email, hours, address, FDA LTO No. - fill js/store-info.js); have them review the Terms/Privacy text. Ask them: are all sales VAT-exempt (sample shows VATable 0.00), is pay-in/pay-out used, who tracks credit collections, which categories to use, may we load the real catalog for the demo?</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Panel may read the Terms during the demo.</t>
+          <t>DONE js/legal-content.js used by the sign-up pop-up and new legal.html; written to the client's policies + Data Privacy Act. CLIENT MUST REVIEW before go-live. Panel may read the Terms during the demo.</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -4590,7 +4590,7 @@
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5861,7 +5861,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE footer rebuilt from js/store-info.js (real About text, links to legal.html; contact/LTO lines hidden until the client confirms them); chat links hidden until chat is built; payment page Terms link fixed. From the first review.</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -5872,7 +5872,7 @@
       <c r="J38" s="11" t="inlineStr"/>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price lock: Branch Manager-only prices with reason, lock toggle, rules
- Only a Branch Manager (or legacy admin) can set or change costing,
  retail and wholesale prices - in Edit Product, Add Product, batch import
  and Receive Stock's quick-add. Other staff can still add products; they
  are saved Inactive and marked 'Price pending' until priced, and staff
  get a notification listing them.
- Every price change needs a stated reason, recorded in the audit log.
- Lock/Unlock prices toggle per product for the Branch Manager.
- firestore.rules enforces the same: non-managers can't write price
  fields or activate a price-pending product.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4883,7 +4883,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr"/>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>DONE BM-only prices in the form, batch import and quick-add (others' products saved Inactive + 'Price pending'); reason required and logged; enforced in firestore.rules - PUBLISH THE RULES in the Firebase console.</t>
+        </is>
+      </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -4892,7 +4896,7 @@
       <c r="J18" s="11" t="inlineStr"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9033,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>Keeps 'price locking' (no letter).</t>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -9040,7 +9044,7 @@
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10834,7 +10838,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Terms rewritten to the branch's policies (client to review). (was: -)</t>
         </is>
       </c>
       <c r="G7" s="11" t="inlineStr">
@@ -11046,9 +11050,9 @@
           <t>Filter by category, price range, stock status</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -11058,12 +11062,12 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Category filter and price sort only; no price-range or stock-status filter.</t>
+          <t>Fixed: price range + availability filters. (was: Category filter and price sort only; no price-range or stock-status filter.)</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -11103,9 +11107,9 @@
           <t>Keyword / product-name search</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -11115,12 +11119,12 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Header search box is not wired to anything on any page.</t>
+          <t>Fixed: header search works on every page. (was: Header search box is not wired to anything on any page.)</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -12366,9 +12370,9 @@
           <t>Customer monitors delivery progress</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -12378,12 +12382,12 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Status timeline shows, but the Lalamove tracking link staff paste is never shown to the customer.</t>
+          <t>Fixed: customer sees the Lalamove tracking link. (was: Status timeline shows, but the Lalamove tracking link staff paste is never shown to the customer.)</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
@@ -14118,9 +14122,9 @@
           <t>Flag batches within 6 months; remove from sellable; wholesale free-of-cost only</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
@@ -14130,12 +14134,12 @@
       </c>
       <c r="F67" s="11" t="inlineStr">
         <is>
-          <t>The flag only runs when someone opens the Inventory page. Until then, near-expiry batches stay sellable online and at the POS. Free-of-cost distribution is not a recorded transaction type (see REQ091).</t>
+          <t>Fixed: retail stock excludes near-expiry batches by date on every load and sale; expired stock never sold. (was: The flag only runs when someone opens the Inventory page. Until then, near-expiry batches stay sellable online and at the POS. Free-of-cost distribution is not a recorded transaction type (see REQ091).)</t>
         </is>
       </c>
       <c r="G67" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H67" s="11" t="inlineStr">
@@ -14342,9 +14346,9 @@
           <t>Add, rename, remove categories</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -14354,12 +14358,12 @@
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>Rename uses the browser's native prompt(), the only native dialog left.</t>
+          <t>Fixed: rename uses the app dialog; delete can move products. (was: Rename uses the browser's native prompt(), the only native dialog left.)</t>
         </is>
       </c>
       <c r="G71" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H71" s="11" t="inlineStr">
@@ -14399,9 +14403,9 @@
           <t>Price changes restricted to Branch Manager</t>
         </is>
       </c>
-      <c r="D72" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -14411,12 +14415,12 @@
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Only editing an existing product is locked. Any staff (incl. Sales Staff) can set prices when creating or batch-importing a product, and the database rules let any staff write prices.</t>
+          <t>Fixed: BM-only prices everywhere, enforced in database rules (publish rules). (was: Only editing an existing product is locked. Any staff (incl. Sales Staff) can set prices when creating or batch-importing a product, and the database rules let any staff write prices.)</t>
         </is>
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr">
@@ -14468,7 +14472,7 @@
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Confirm step now also asks for a reason. (was: -)</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
@@ -14509,9 +14513,9 @@
           <t>Audit log: previous price, new price, timestamp</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
-        <is>
-          <t>Matches</t>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -14521,7 +14525,7 @@
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>Matches the paper, but the client asked for a reason with each change (Interview 2) and none is captured.</t>
+          <t>System now logs the reason too; paper REQ073 wording should add 'reason'. (was: Matches the paper, but the client asked for a reason with each change (Interview 2) and none is captured.)</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
@@ -15580,7 +15584,7 @@
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>Walk-in and online receipts exist; no wholesale sales invoice. Receipts show no batch numbers or expiry dates, which the Project Context (p.1) names as the old POS's main gap.</t>
+          <t>Walk-in/online receipts now carry SI No.; sales record batch + expiry per line; wholesale sales invoice still missing. (was: Walk-in and online receipts exist; no wholesale sales invoice. Receipts show no batch numbers or expiry dates, which the Project Context (p.1) names as the old POS's main gap.)</t>
         </is>
       </c>
       <c r="G93" s="11" t="inlineStr">
@@ -16118,9 +16122,9 @@
           <t>Notify customer on verification</t>
         </is>
       </c>
-      <c r="D103" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D103" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
@@ -16130,12 +16134,12 @@
       </c>
       <c r="F103" s="11" t="inlineStr">
         <is>
-          <t>Works for normal approvals; missing for overpayment approvals (see REQ098).</t>
+          <t>Fixed: overpayment approval now notifies the customer. (was: Works for normal approvals; missing for overpayment approvals (see REQ098).)</t>
         </is>
       </c>
       <c r="G103" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H103" s="11" t="inlineStr">
@@ -17120,9 +17124,9 @@
           <t>Technical Staff cannot access Staff Management or Price Management</t>
         </is>
       </c>
-      <c r="D121" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D121" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -17132,12 +17136,12 @@
       </c>
       <c r="F121" s="11" t="inlineStr">
         <is>
-          <t>Staff Management is blocked. Price: see REQ071 (Technical Staff can set prices on new products).</t>
+          <t>Fixed with REQ071. (was: Staff Management is blocked. Price: see REQ071 (Technical Staff can set prices on new products).)</t>
         </is>
       </c>
       <c r="G121" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H121" s="11" t="inlineStr">
@@ -18713,9 +18717,9 @@
           <t>Data Privacy Act 2012</t>
         </is>
       </c>
-      <c r="D150" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D150" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
@@ -18725,12 +18729,12 @@
       </c>
       <c r="F150" s="11" t="inlineStr">
         <is>
-          <t>Terms/Privacy shown at registration, but footer Privacy Policy and Terms links go nowhere.</t>
+          <t>Privacy Policy rewritten for the Data Privacy Act and linked from every footer (client to review). (was: Terms/Privacy shown at registration, but footer Privacy Policy and Terms links go nowhere.)</t>
         </is>
       </c>
       <c r="G150" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H150" s="11" t="inlineStr">
@@ -18933,9 +18937,9 @@
           <t>Clear, professional language</t>
         </is>
       </c>
-      <c r="D154" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D154" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
@@ -18945,12 +18949,12 @@
       </c>
       <c r="F154" s="11" t="inlineStr">
         <is>
-          <t>Footer says 'Amson about description sample text'.</t>
+          <t>Filler text removed from the footer. (was: Footer says 'Amson about description sample text'.)</t>
         </is>
       </c>
       <c r="G154" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H154" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register: void, RX check, receipt printing, Sales Staff access done; exports partial
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4262,7 +4262,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Client's one remaining ask (Interview 4). Build to the 4 client samples (see Report Formats sheet); Excel output must paste cleanly into the main office's own sheets (Interviews 1, 2, 4); daily sales should total by payment method to match the daily cash remittance (Interview 2).</t>
+          <t>PARTIAL aece0e7: all 6 Export buttons now produce real PDF/Excel tables of what's on screen; the client's 4 report formats are still to build. Client's one remaining ask (Interview 4). Build to the 4 client samples (see Report Formats sheet); Excel output must paste cleanly into the main office's own sheets (Interviews 1, 2, 4); daily sales should total by payment method to match the daily cash remittance (Interview 2).</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
+          <t>DONE 57f4d80: BM/Technical void completed sales from POS Today's Sales or Walk-in Orders: reason, SI No., stock restored to the same batches, exchange note + price difference, audit entry. Still open: second-person approval (client rule) and exchange as a real stock movement. Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
@@ -4794,7 +4794,7 @@
       <c r="J16" s="11" t="inlineStr"/>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: trim to POS + catalog view; Walk-in history inside POS. Orders access was added on purpose on 2026-10-01.</t>
+          <t>DONE 57f4d80: POS (with Today's Sales) + read-only catalog; lands on POS after login. Orders access was added on purpose on 2026-10-01.</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
@@ -5045,7 +5045,7 @@
       <c r="J21" s="11" t="inlineStr"/>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5722,7 +5722,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr"/>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout; 'not an official receipt' line.</t>
+        </is>
+      </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5731,7 +5735,7 @@
       <c r="J35" s="11" t="inlineStr"/>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5769,7 +5773,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr"/>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>DONE 57f4d80: checkbox + notes, required for RX items, saved on the sale.</t>
+        </is>
+      </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5778,7 +5786,7 @@
       <c r="J36" s="11" t="inlineStr"/>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15063,9 +15071,9 @@
           <t>Void with reason, restore stock, audit log, record exchange + price difference</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -15075,7 +15083,7 @@
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>No void function at all.</t>
+          <t>57f4d80: void for completed walk-in sales by BM/Technical (Admin too): reason, original SI No., stock back to the exact batches, optional exchange note + price difference, audit entry. Not yet: second-person approval; exchange item is a note, not a stock movement. (was: No void function at all.)</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
@@ -15120,9 +15128,9 @@
           <t>RX Verified checkbox + optional notes, no upload</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
@@ -15132,12 +15140,12 @@
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>Not in POS.</t>
+          <t>57f4d80: RX Verified checkbox + optional notes in POS, required when the cart has RX items. (was: Not in POS.)</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H85" s="11" t="inlineStr">
@@ -16627,9 +16635,9 @@
           <t>Export daily sales reports (from Order Processing)</t>
         </is>
       </c>
-      <c r="D112" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -16639,7 +16647,7 @@
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>Online Orders Export downloads a blank PDF. Dashboard Sales Analytics export works but is not the daily sales report the client described (per customer, items with batch + expiry).</t>
+          <t>aece0e7: Online Orders Export now gives real PDF/Excel of the listed orders. Client's daily sales format still to build. (was: Online Orders Export downloads a blank PDF. Dashboard Sales Analytics export works but is not the daily sales report the client described (per customer, items with batch + expiry).)</t>
         </is>
       </c>
       <c r="G112" s="11" t="inlineStr">
@@ -16684,9 +16692,9 @@
           <t>Export monthly inventory + purchase reports (from Inventory)</t>
         </is>
       </c>
-      <c r="D113" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -16696,7 +16704,7 @@
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>Inventory Export downloads a blank PDF.</t>
+          <t>aece0e7: Inventory Export now gives real PDF/Excel by batch (expiry, supplier, receipt/DR no., unit cost, date received). Client's monthly format still to build. (was: Inventory Export downloads a blank PDF.)</t>
         </is>
       </c>
       <c r="G113" s="11" t="inlineStr">
@@ -16863,7 +16871,7 @@
       </c>
       <c r="F116" s="11" t="inlineStr">
         <is>
-          <t>Only Sales Analytics exports (PDF + Excel). Five other Export buttons give blank PDFs (Dashboard, Inventory, Online Orders, Suppliers, Audit Log).</t>
+          <t>aece0e7: all 6 Export buttons now give real PDF or Excel. Client report formats still to build. (was: Only Sales Analytics exports (PDF + Excel). Five other Export buttons give blank PDFs (Dashboard, Inventory, Online Orders, Suppliers, Audit Log).)</t>
         </is>
       </c>
       <c r="G116" s="11" t="inlineStr">
@@ -17181,9 +17189,9 @@
           <t>Sales Staff: walk-in orders + catalog viewing only</t>
         </is>
       </c>
-      <c r="D122" s="16" t="inlineStr">
-        <is>
-          <t>Deviates</t>
+      <c r="D122" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -17193,12 +17201,12 @@
       </c>
       <c r="F122" s="11" t="inlineStr">
         <is>
-          <t>Sales Staff can also open Dashboard, Orders, Products (with editing), and Notifications. Orders access was added deliberately on 2026-10-01 for the Walk-in Orders tab.</t>
+          <t>57f4d80: Sales Staff limited to POS (with Today's Sales) + read-only catalog. (was: Sales Staff can also open Dashboard, Orders, Products (with editing), and Notifications. Orders access was added deliberately on 2026-10-01 for the Walk-in Orders tab.)</t>
         </is>
       </c>
       <c r="G122" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H122" s="11" t="inlineStr">
@@ -18460,7 +18468,7 @@
       </c>
       <c r="F145" s="11" t="inlineStr">
         <is>
-          <t>Only Sales Analytics exports.</t>
+          <t>aece0e7: every Export button offers PDF or Excel. (was: Only Sales Analytics exports.)</t>
         </is>
       </c>
       <c r="G145" s="11" t="inlineStr">
@@ -19477,9 +19485,9 @@
           <t>Technical Staff</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -19489,7 +19497,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Five blank-PDF exports.</t>
+          <t>aece0e7: exports are real PDF/Excel; client report formats still to build.</t>
         </is>
       </c>
     </row>
@@ -20517,9 +20525,9 @@
           <t>Sales/Technical</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -20529,7 +20537,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>No print button / thermal format.</t>
+          <t>57f4d80: Print button with 58mm receipt layout.</t>
         </is>
       </c>
     </row>
@@ -20549,9 +20557,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -20561,7 +20569,7 @@
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>57f4d80: void with required reason.</t>
         </is>
       </c>
     </row>
@@ -22639,24 +22647,20 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Receipt shown on screen only</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>57f4d80: Print button, 58mm layout</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
-        </is>
-      </c>
-      <c r="G41" s="11" t="inlineStr">
-        <is>
-          <t>Thermal print layout.</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -22676,22 +22680,22 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>57f4d80: void built</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>Change paper</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Build REQ083; add the void branch to the diagram.</t>
+          <t>Add the void branch to the diagram.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: prescription flow, wholesale, reconciliation, cart, dates and other fixes marked done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4326,7 +4326,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>DONE 082ec92: RX filter, Reject Prescription with reason (7-day re-upload hold), 'ready for pick-up' notice, verifier recorded + audit.</t>
+        </is>
+      </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -4335,7 +4339,7 @@
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5434,7 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE d9fc96b: locks itself after one run; SI counter now staff-only in rules (publish rules). From the first review.</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -5441,7 +5445,7 @@
       <c r="J29" s="11" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5583,7 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
+          <t>DONE 5cad255: history, sales invoice PDF, free-of-cost, LTO/permit validity. Not built: reorder from a past order. Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -5590,7 +5594,7 @@
       <c r="J32" s="11" t="inlineStr"/>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5828,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr"/>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da: others save counts; BM finalizes; variance reason required and logged.</t>
+        </is>
+      </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5833,7 +5841,7 @@
       <c r="J37" s="11" t="inlineStr"/>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6028,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr"/>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>DONE 77336f3.</t>
+        </is>
+      </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6029,7 +6041,7 @@
       <c r="J41" s="11" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6128,7 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>Required column in the monthly purchases report.</t>
+          <t>DONE e1e200b. Required column in the monthly purchases report.</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
@@ -6127,7 +6139,7 @@
       <c r="J43" s="11" t="inlineStr"/>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6581,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr"/>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+        </is>
+      </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6578,7 +6594,7 @@
       <c r="J52" s="11" t="inlineStr"/>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6632,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr"/>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>DONE footer links to legal.html on every page.</t>
+        </is>
+      </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6625,7 +6645,7 @@
       <c r="J53" s="11" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6663,7 +6683,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H54" s="11" t="inlineStr"/>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+        </is>
+      </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -6672,7 +6696,7 @@
       <c r="J54" s="11" t="inlineStr"/>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8157,7 +8181,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H84" s="11" t="inlineStr"/>
+      <c r="H84" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da.</t>
+        </is>
+      </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8166,7 +8194,7 @@
       <c r="J84" s="11" t="inlineStr"/>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8204,7 +8232,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H85" s="11" t="inlineStr"/>
+      <c r="H85" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da.</t>
+        </is>
+      </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8213,7 +8245,7 @@
       <c r="J85" s="11" t="inlineStr"/>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8253,7 +8285,7 @@
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
@@ -8264,7 +8296,7 @@
       <c r="J86" s="11" t="inlineStr"/>
       <c r="K86" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8334,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H87" s="11" t="inlineStr"/>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>DONE 847c877.</t>
+        </is>
+      </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8311,7 +8347,7 @@
       <c r="J87" s="11" t="inlineStr"/>
       <c r="K87" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8387,7 @@
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
@@ -8362,7 +8398,7 @@
       <c r="J88" s="11" t="inlineStr"/>
       <c r="K88" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8453,7 +8489,7 @@
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
@@ -8464,7 +8500,7 @@
       <c r="J90" s="11" t="inlineStr"/>
       <c r="K90" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8538,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H91" s="11" t="inlineStr"/>
+      <c r="H91" s="11" t="inlineStr">
+        <is>
+          <t>DONE 847c877.</t>
+        </is>
+      </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8511,7 +8551,7 @@
       <c r="J91" s="11" t="inlineStr"/>
       <c r="K91" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8549,7 +8589,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H92" s="11" t="inlineStr"/>
+      <c r="H92" s="11" t="inlineStr">
+        <is>
+          <t>DONE 082ec92.</t>
+        </is>
+      </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8558,7 +8602,7 @@
       <c r="J92" s="11" t="inlineStr"/>
       <c r="K92" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8596,7 +8640,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H93" s="11" t="inlineStr"/>
+      <c r="H93" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da.</t>
+        </is>
+      </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8605,7 +8653,7 @@
       <c r="J93" s="11" t="inlineStr"/>
       <c r="K93" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8643,7 +8691,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H94" s="11" t="inlineStr"/>
+      <c r="H94" s="11" t="inlineStr">
+        <is>
+          <t>DONE 77336f3.</t>
+        </is>
+      </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8652,7 +8704,7 @@
       <c r="J94" s="11" t="inlineStr"/>
       <c r="K94" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8690,7 +8742,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H95" s="11" t="inlineStr"/>
+      <c r="H95" s="11" t="inlineStr">
+        <is>
+          <t>DONE 847c877.</t>
+        </is>
+      </c>
       <c r="I95" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8699,7 +8755,7 @@
       <c r="J95" s="11" t="inlineStr"/>
       <c r="K95" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8739,7 +8795,7 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I96" s="11" t="inlineStr">
@@ -8750,7 +8806,7 @@
       <c r="J96" s="11" t="inlineStr"/>
       <c r="K96" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8790,7 +8846,7 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
@@ -8801,7 +8857,7 @@
       <c r="J97" s="11" t="inlineStr"/>
       <c r="K97" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8841,7 +8897,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE d9fc96b. From the first review.</t>
         </is>
       </c>
       <c r="I98" s="11" t="inlineStr">
@@ -8852,7 +8908,7 @@
       <c r="J98" s="11" t="inlineStr"/>
       <c r="K98" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8939,7 +8995,7 @@
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>Keeps the paper's status name (no letter).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
@@ -8950,7 +9006,7 @@
       <c r="J100" s="11" t="inlineStr"/>
       <c r="K100" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11001,9 +11057,9 @@
           <t>Catalog by category with name, price, stock availability</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -11013,12 +11069,12 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Cards show name/price and an Out of Stock badge, but not the quantity available (only on the product page).</t>
+          <t>06574da: catalog cards show the quantity in stock. (was: Cards show name/price and an Out of Stock badge, but not the quantity available (only on the product page).)</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -11225,9 +11281,9 @@
           <t>Product page: name, description, price, stock, dosage/usage notes, images</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -11237,12 +11293,12 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>No dosage/usage notes field exists anywhere.</t>
+          <t>06574da: Dosage / Usage notes field shown on the product page and quick view. (was: No dosage/usage notes field exists anywhere.)</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -11282,9 +11338,9 @@
           <t>Persistent cart per logged-in customer</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>Deviates</t>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -11294,12 +11350,12 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Cart is stored in the browser, so it follows the device, not the account.</t>
+          <t>77336f3: signed-in cart saved on the account and merged with any guest cart at sign-in. (was: Cart is stored in the browser, so it follows the device, not the account.)</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -11824,9 +11880,9 @@
           <t>Submitted as 'Pending Prescription Verification'; not prepared until staff approve the prescription</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -11836,12 +11892,12 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>RX orders use the same 'Order Pending Verification' status as normal orders; prescription approval is not a separate step.</t>
+          <t>082ec92: RX orders show 'Pending Prescription Verification' and aren't prepared until staff approve the prescription. (was: RX orders use the same 'Order Pending Verification' status as normal orders; prescription approval is not a separate step.)</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -11881,9 +11937,9 @@
           <t>Notify approved/ready for pick-up, or rejected with reason</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -11893,12 +11949,12 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Approval sends 'Payment confirmed' only; there is no rejection path at all.</t>
+          <t>082ec92: approval sends 'ready for pick-up'; rejection sends the reason. (was: Approval sends 'Payment confirmed' only; there is no rejection path at all.)</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -11938,9 +11994,9 @@
           <t>Notice: original prescription must be presented at pick-up</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -11950,12 +12006,12 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice does not mention the original prescription (only the later pick-up notification does).</t>
+          <t>082ec92: checkout and payment pages say to bring the original prescription. (was: Checkout pick-up notice does not mention the original prescription (only the later pick-up notification does).)</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -12321,9 +12377,9 @@
           <t>View/download system receipt for completed orders</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -12333,12 +12389,12 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>Receipt downloadable for any order (even unpaid); PDF shows only final total, not subtotal/credit applied.</t>
+          <t>082ec92: receipt only after verification; PDF shows subtotal and store credit applied. (was: Receipt downloadable for any order (even unpaid); PDF shows only final total, not subtotal/credit applied.)</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -12720,9 +12776,9 @@
           <t>Update name, address, contact no., profile picture</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
@@ -12732,12 +12788,12 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>No profile picture.</t>
+          <t>77336f3: profile photo upload in Account Settings. (was: No profile picture.)</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
@@ -13172,7 +13228,7 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.</t>
+          <t>57f4d80: no longer shown to Sales Staff. Still missing wholesale-order and chat notifications. (was: Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.)</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -13217,9 +13273,9 @@
           <t>Inventory list per product by batch, with supplier details</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -13229,12 +13285,12 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>Batch table has no supplier column.</t>
+          <t>06574da: batch table has a Supplier column (with receipt/DR no.). (was: Batch table has no supplier column.)</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -13861,9 +13917,9 @@
           <t>Branch Manager finalizes; variance reason in Audit Log</t>
         </is>
       </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -13873,12 +13929,12 @@
       </c>
       <c r="F62" s="11" t="inlineStr">
         <is>
-          <t>Any staff with Inventory access can finalize; no variance reason is asked or logged (only a count of adjusted batches).</t>
+          <t>06574da: only the Branch Manager finalizes; others save the count; variance reason required and logged with each batch's change. (was: Any staff with Inventory access can finalize; no variance reason is asked or logged (only a count of adjusted batches).)</t>
         </is>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
@@ -14244,9 +14300,9 @@
           <t>Create/edit/remove products incl. dosage notes, costing, retail, wholesale, image</t>
         </is>
       </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
@@ -14256,12 +14312,12 @@
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>No dosage notes field.</t>
+          <t>06574da: dosage notes field added to the product form. (was: No dosage notes field.)</t>
         </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr">
@@ -14737,9 +14793,9 @@
           <t>Dedicated RX pre-order queue with prescription + payment proof</t>
         </is>
       </c>
-      <c r="D78" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -14749,12 +14805,12 @@
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>RX orders appear in the general Payment Verification queue with the photo shown; no dedicated queue or filter.</t>
+          <t>082ec92: RX filter + RX badge in the verification queue, prescription and payment shown together. (was: RX orders appear in the general Payment Verification queue with the photo shown; no dedicated queue or filter.)</t>
         </is>
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr">
@@ -14794,9 +14850,9 @@
           <t>Approve after checking prescription: FEFO reservation, Ready for Pick-up, notify</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
@@ -14806,12 +14862,12 @@
       </c>
       <c r="F79" s="11" t="inlineStr">
         <is>
-          <t>Approving payment moves RX orders straight to Ready for Pick-up, but the notification says 'Payment confirmed', not 'Ready for pick-up'.</t>
+          <t>082ec92: approval reserves stock (FEFO), sets Ready for Pick-up and notifies 'ready for pick-up'. (was: Approving payment moves RX orders straight to Ready for Pick-up, but the notification says 'Payment confirmed', not 'Ready for pick-up'.)</t>
         </is>
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
@@ -14851,9 +14907,9 @@
           <t>Mandatory reason to reject; reason in customer notification</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D80" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
@@ -14863,12 +14919,12 @@
       </c>
       <c r="F80" s="11" t="inlineStr">
         <is>
-          <t>No reject action exists for prescriptions.</t>
+          <t>082ec92: Reject Prescription with required reason + message; customer can re-upload within 7 days. (was: No reject action exists for prescriptions.)</t>
         </is>
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr">
@@ -14961,9 +15017,9 @@
           <t>Record staff, timestamp, action per verification</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D82" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -14973,12 +15029,12 @@
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>Who approved is not stored.</t>
+          <t>082ec92: every approval/hold/rejection stores who, when and what (verification field) + audit entry for RX. (was: Who approved is not stored.)</t>
         </is>
       </c>
       <c r="G82" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H82" s="11" t="inlineStr">
@@ -15242,9 +15298,9 @@
           <t>Upload/update LTO and Business Permit</t>
         </is>
       </c>
-      <c r="D87" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
@@ -15254,12 +15310,12 @@
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>Upload works; no document expiry date or 'expired' flag (shown in Interview 4 walkthrough and Activity 2.13).</t>
+          <t>5cad255: LTO and Business Permit valid-until dates; cards flag expired/expiring; orders blocked while expired. (was: Upload works; no document expiry date or 'expired' flag (shown in Interview 4 walkthrough and Activity 2.13).)</t>
         </is>
       </c>
       <c r="G87" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H87" s="11" t="inlineStr">
@@ -15409,9 +15465,9 @@
           <t>Purchase history per wholesale account</t>
         </is>
       </c>
-      <c r="D90" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D90" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -15421,12 +15477,12 @@
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>Orders are saved (wholesaleOrders) but there is no history view.</t>
+          <t>5cad255: Purchase History per wholesale account, with invoice download. (was: Orders are saved (wholesaleOrders) but there is no history view.)</t>
         </is>
       </c>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H90" s="11" t="inlineStr">
@@ -15523,9 +15579,9 @@
           <t>Free-of-cost near-expiry distributions, zero cost, reason in audit log</t>
         </is>
       </c>
-      <c r="D92" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D92" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -15535,12 +15591,12 @@
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>A unit price of 0 is possible, but there is no free-of-cost option, reason, or dedicated audit entry.</t>
+          <t>5cad255: free-of-cost option (prices 0), required reason, own audit entry, noted on the invoice. (was: A unit price of 0 is possible, but there is no free-of-cost option, reason, or dedicated audit entry.)</t>
         </is>
       </c>
       <c r="G92" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H92" s="11" t="inlineStr">
@@ -15580,9 +15636,9 @@
           <t>Retail/walk-in receipt; wholesale sales invoice with buyer details</t>
         </is>
       </c>
-      <c r="D93" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D93" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
@@ -15592,12 +15648,12 @@
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>Walk-in/online receipts now carry SI No.; sales record batch + expiry per line; wholesale sales invoice still missing. (was: Walk-in and online receipts exist; no wholesale sales invoice. Receipts show no batch numbers or expiry dates, which the Project Context (p.1) names as the old POS's main gap.)</t>
+          <t>5cad255: wholesale sales invoice PDF with buyer details, batch and expiry per line; walk-in/online receipts carry SI No. (was: Walk-in and online receipts exist; no wholesale sales invoice. Receipts show no batch numbers or expiry dates, which the Project Context (p.1) names as the old POS's main gap.)</t>
         </is>
       </c>
       <c r="G93" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H93" s="11" t="inlineStr">
@@ -15637,9 +15693,9 @@
           <t>Receipt on payment verification, downloadable in My Orders</t>
         </is>
       </c>
-      <c r="D94" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D94" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -15649,12 +15705,12 @@
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>Available before verification too.</t>
+          <t>082ec92: receipt only downloadable once payment is verified (SI No. assigned). (was: Available before verification too.)</t>
         </is>
       </c>
       <c r="G94" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H94" s="11" t="inlineStr">
@@ -15963,9 +16019,9 @@
           <t>On Hold - Payment Not Received, reason, notify</t>
         </is>
       </c>
-      <c r="D100" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D100" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
@@ -15975,12 +16031,12 @@
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>Exists only as a reason under 'Invalid payment', not as its own hold type.</t>
+          <t>847c877: 'Payment not received' is its own hold type; customer sees 'Payment Rejected - Re-upload Needed'. (was: Exists only as a reason under 'Invalid payment', not as its own hold type.)</t>
         </is>
       </c>
       <c r="G100" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H100" s="11" t="inlineStr">
@@ -16187,9 +16243,9 @@
           <t>Compile name, address, contact, schedule, order ID; one-click copy</t>
         </is>
       </c>
-      <c r="D104" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D104" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
@@ -16199,12 +16255,12 @@
       </c>
       <c r="F104" s="11" t="inlineStr">
         <is>
-          <t>Separate copy buttons for address/name/contact/notes. Preferred schedule and order ID are not shown; no 'copy all'.</t>
+          <t>06574da: approved modal shows order no. and preferred schedule, with a Copy All button. (was: Separate copy buttons for address/name/contact/notes. Preferred schedule and order ID are not shown; no 'copy all'.)</t>
         </is>
       </c>
       <c r="G104" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H104" s="11" t="inlineStr">
@@ -16309,7 +16365,7 @@
       </c>
       <c r="F106" s="11" t="inlineStr">
         <is>
-          <t>Customer sees status, but not the tracking link. Customer confirmation sets 'Received' (a separate step after 'Delivered').</t>
+          <t>Tracking link now shown to the customer. Remaining difference is wording: customer confirmation sets 'Received' after 'Delivered' (fix in paper). (was: Customer sees status, but not the tracking link. Customer confirmation sets 'Received' (a separate step after 'Delivered').)</t>
         </is>
       </c>
       <c r="G106" s="11" t="inlineStr">
@@ -16407,9 +16463,9 @@
           <t>Optional internal delivery notes</t>
         </is>
       </c>
-      <c r="D108" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D108" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
@@ -16419,12 +16475,12 @@
       </c>
       <c r="F108" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>06574da: optional internal delivery notes saved on dispatch. (was: Not built.)</t>
         </is>
       </c>
       <c r="G108" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H108" s="11" t="inlineStr">
@@ -16912,9 +16968,9 @@
           <t>View profiles: status, registration date, order history</t>
         </is>
       </c>
-      <c r="D117" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D117" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
@@ -16924,12 +16980,12 @@
       </c>
       <c r="F117" s="11" t="inlineStr">
         <is>
-          <t>Shows total order count, not the order list.</t>
+          <t>847c877: customer profile lists their orders with status. (was: Shows total order count, not the order list.)</t>
         </is>
       </c>
       <c r="G117" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H117" s="11" t="inlineStr">
@@ -17022,9 +17078,9 @@
           <t>BM creates, modifies, revokes staff accounts</t>
         </is>
       </c>
-      <c r="D119" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D119" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -17034,12 +17090,12 @@
       </c>
       <c r="F119" s="11" t="inlineStr">
         <is>
-          <t>Works (revoke = deactivate). New staff accounts skip the shared name/email/password validators, and editing an Administrator silently changes it to Branch Manager (js/admin-staff-management.js:181).</t>
+          <t>847c877: staff form uses the shared name/email/password rules; Administrator no longer demoted on edit. (was: Works (revoke = deactivate). New staff accounts skip the shared name/email/password validators, and editing an Administrator silently changes it to Branch Manager (js/admin-staff-management.js:181).)</t>
         </is>
       </c>
       <c r="G119" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H119" s="11" t="inlineStr">
@@ -17258,7 +17314,7 @@
       </c>
       <c r="F123" s="11" t="inlineStr">
         <is>
-          <t>Logs price changes, write-offs, reconciliation, wholesale orders, account changes. Stock receiving is not logged (Fig 2.12 shows it). Voids and exchanges don't exist yet. Before/after values are free text, reasons mostly missing, IP shown as '-'.</t>
+          <t>Now also logs stock receiving, voids (reason), RX approvals/rejections, free-of-cost distributions and reconciliation variances with reason. Still free-text before/after; IP shown as '-'. (was: Logs price changes, write-offs, reconciliation, wholesale orders, account changes. Stock receiving is not logged (Fig 2.12 shows it). Voids and exchanges don't exist yet. Before/after values are free text, reasons mostly missing, IP shown as '-'.)</t>
         </is>
       </c>
       <c r="G123" s="11" t="inlineStr">
@@ -18293,9 +18349,9 @@
           <t>Modular code with documentation</t>
         </is>
       </c>
-      <c r="D142" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E142" s="11" t="inlineStr">
@@ -18305,12 +18361,12 @@
       </c>
       <c r="F142" s="11" t="inlineStr">
         <is>
-          <t>Modular, but no README or setup documentation (an error message even points to a missing README.md).</t>
+          <t>77336f3: README with setup, services, rules publishing, roles and deployment. (was: Modular, but no README or setup documentation (an error message even points to a missing README.md).)</t>
         </is>
       </c>
       <c r="G142" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H142" s="11" t="inlineStr">
@@ -18888,9 +18944,9 @@
           <t>Dates MM/DD/YYYY, 12-hour AM/PM</t>
         </is>
       </c>
-      <c r="D153" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D153" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
@@ -18900,12 +18956,12 @@
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>Several screens use 'Oct 18, 2026' or 'October 2026'; the audit log uses a 2-digit hour.</t>
+          <t>847c877: one MM/DD/YYYY + 12-hour formatter on every screen, receipt and export. (was: Several screens use 'Oct 18, 2026' or 'October 2026'; the audit log uses a 2-digit hour.)</t>
         </is>
       </c>
       <c r="G153" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H153" s="11" t="inlineStr">
@@ -19129,9 +19185,9 @@
           <t>Guest</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -19141,7 +19197,7 @@
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Search box not wired; no price/stock filters.</t>
+          <t>Header search + price/stock filters.</t>
         </is>
       </c>
     </row>
@@ -19545,9 +19601,9 @@
           <t>Technical Staff</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -19557,7 +19613,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>REQ061 says BM finalizes - see C5.</t>
+          <t>06574da: BM finalizes; variance reason logged.</t>
         </is>
       </c>
     </row>
@@ -19609,9 +19665,9 @@
           <t>Branch Manager</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -19621,7 +19677,7 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Non-BM can set prices on new products.</t>
+          <t>BM-only prices everywhere (publish rules).</t>
         </is>
       </c>
     </row>
@@ -19725,9 +19781,9 @@
           <t>Registered User</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -19737,7 +19793,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Cart is per browser, not per account.</t>
+          <t>77336f3: cart saved on the account.</t>
         </is>
       </c>
     </row>
@@ -19797,7 +19853,7 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Named 'Submit Prescription Pre-Order' in Fig 2.4.</t>
+          <t>082ec92: approve/reject built. Name still differs from Fig 2.4 ('Submit Prescription Pre-Order') - paper edit.</t>
         </is>
       </c>
     </row>
@@ -19901,9 +19957,9 @@
           <t>Guest</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -19911,7 +19967,11 @@
           <t>REQ010-011</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr"/>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Header search + price/stock filters.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -20045,9 +20105,9 @@
           <t>Registered User</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -20057,7 +20117,7 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>No separate prescription approval/rejection.</t>
+          <t>082ec92: separate prescription approval/rejection with reason.</t>
         </is>
       </c>
     </row>
@@ -20161,9 +20221,9 @@
           <t>Registered User</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -20173,7 +20233,7 @@
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>Tracking link not shown.</t>
+          <t>Tracking link shown once dispatched.</t>
         </is>
       </c>
     </row>
@@ -20373,9 +20433,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -20385,7 +20445,7 @@
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>BM finalize + reason missing.</t>
+          <t>06574da: BM finalizes; variance reason logged.</t>
         </is>
       </c>
     </row>
@@ -20673,9 +20733,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -20683,7 +20743,11 @@
           <t>REQ111-115</t>
         </is>
       </c>
-      <c r="F56" s="11" t="inlineStr"/>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>aece0e7: exports are real PDF/Excel; client report formats still to build.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -20977,9 +21041,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -20989,7 +21053,7 @@
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>No order history list.</t>
+          <t>847c877: order history listed in the profile.</t>
         </is>
       </c>
     </row>
@@ -21037,9 +21101,9 @@
           <t>Branch Manager</t>
         </is>
       </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -21049,7 +21113,7 @@
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>Non-BM staff can set prices on new/imported products.</t>
+          <t>BM-only prices everywhere (publish rules).</t>
         </is>
       </c>
     </row>
@@ -21882,17 +21946,17 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Not built (payment approval only)</t>
-        </is>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>082ec92: approve or reject (reason) before preparation; notify customer</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -21919,7 +21983,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Admin pastes the link and marks Dispatched in one step; customer can't see the link</t>
+          <t>Customer now sees the tracking link; marking Dispatched with the link is still one step</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -22170,17 +22234,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Same, except receiving is not written to the audit log</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Receiving is now written to the audit log</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -22425,17 +22489,17 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Documents viewable; no expiry tracking</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>5cad255: LTO/permit valid-until dates; expired documents block the order</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
@@ -22462,17 +22526,17 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E36" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>5cad255: Purchase History per buyer</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -22499,17 +22563,17 @@
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Near-expiry stock is used first automatically; price can be typed as 0 but there is no free-of-cost option</t>
-        </is>
-      </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>5cad255: free-of-cost option with reason and audit entry</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -22536,17 +22600,17 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Confirm + FEFO deduction + audit entry; no sales invoice</t>
-        </is>
-      </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>5cad255: sales invoice PDF with buyer, batch and expiry</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -22610,17 +22674,17 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>No RX check in POS</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>57f4d80: RX Verified checkbox + notes in POS</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Remove the 'not an official receipt' line from receipts; register: dashboard period picker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$132</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5728,7 +5728,7 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout; 'not an official receipt' line.</t>
+          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout. The 'not an official receipt' line was removed from POS and online receipts on 2026-10-21 at the team's request.</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -6511,17 +6511,17 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>Dashboard module p.40; Interview 4 (dashboard export)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>Dashboard Sales Analytics: show which dates the Today/Week/Month/Year view covers, and add a picker to choose a specific day, week, month or year (with previous/next)</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
@@ -6534,7 +6534,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr"/>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
+        </is>
+      </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6558,12 +6562,12 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -6581,11 +6585,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>DONE 06574da: system now matches (BM-only finalize).</t>
-        </is>
-      </c>
+      <c r="H52" s="11" t="inlineStr"/>
       <c r="I52" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6594,7 +6594,7 @@
       <c r="J52" s="11" t="inlineStr"/>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6609,12 +6609,12 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>DONE footer links to legal.html on every page.</t>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
@@ -6655,17 +6655,17 @@
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
@@ -6685,12 +6685,12 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+          <t>DONE footer links to legal.html on every page.</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr"/>
@@ -6706,22 +6706,22 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
@@ -6747,7 +6747,7 @@
       <c r="J55" s="11" t="inlineStr"/>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6762,12 +6762,12 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -6790,9 +6790,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I56" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr"/>
@@ -6813,12 +6813,12 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
@@ -6864,12 +6864,12 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
@@ -6892,9 +6892,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr"/>
@@ -6915,12 +6915,12 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
@@ -6966,12 +6966,12 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -6994,9 +6994,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I60" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr"/>
@@ -7017,12 +7017,12 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
@@ -7068,12 +7068,12 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -7096,9 +7096,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I62" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr"/>
@@ -7119,12 +7119,12 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
@@ -7170,12 +7170,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
@@ -7272,12 +7272,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -7323,12 +7323,12 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
@@ -7374,12 +7374,12 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -7425,12 +7425,12 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
@@ -7476,12 +7476,12 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -7527,12 +7527,12 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -7578,17 +7578,17 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
@@ -7601,7 +7601,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H72" s="11" t="inlineStr"/>
+      <c r="H72" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7625,12 +7629,12 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
@@ -7640,7 +7644,7 @@
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
@@ -7672,12 +7676,12 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -7687,7 +7691,7 @@
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
@@ -7719,12 +7723,12 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
@@ -7743,9 +7747,9 @@
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr"/>
-      <c r="I75" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J75" s="11" t="inlineStr"/>
@@ -7766,12 +7770,12 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -7790,9 +7794,9 @@
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
-      <c r="I76" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I76" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr"/>
@@ -7813,12 +7817,12 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -7865,7 +7869,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -7902,42 +7906,38 @@
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H79" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED (revised): build it to avoid a removal letter.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H79" s="11" t="inlineStr"/>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
@@ -7958,17 +7958,17 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
@@ -7983,18 +7983,18 @@
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
         </is>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr"/>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8009,12 +8009,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
         </is>
       </c>
       <c r="I81" s="11" t="inlineStr">
@@ -8060,12 +8060,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G82" s="11" t="inlineStr">
@@ -8085,7 +8085,7 @@
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I82" s="11" t="inlineStr">
@@ -8106,22 +8106,22 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
@@ -8134,16 +8134,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H83" s="11" t="inlineStr"/>
+      <c r="H83" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+        </is>
+      </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr"/>
       <c r="K83" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8153,22 +8157,22 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
@@ -8181,11 +8185,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H84" s="11" t="inlineStr">
-        <is>
-          <t>DONE 06574da.</t>
-        </is>
-      </c>
+      <c r="H84" s="11" t="inlineStr"/>
       <c r="I84" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8194,7 +8194,7 @@
       <c r="J84" s="11" t="inlineStr"/>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8209,17 +8209,17 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F85" s="11" t="inlineStr">
@@ -8260,12 +8260,12 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -8285,7 +8285,7 @@
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
@@ -8311,12 +8311,12 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="H87" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I87" s="11" t="inlineStr">
@@ -8362,17 +8362,17 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
@@ -8413,17 +8413,17 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I89" s="11" t="inlineStr">
@@ -8464,17 +8464,17 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
@@ -8489,7 +8489,7 @@
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92. From the first review.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
@@ -8515,12 +8515,12 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I91" s="11" t="inlineStr">
@@ -8566,12 +8566,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I92" s="11" t="inlineStr">
@@ -8617,12 +8617,12 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE 082ec92.</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
@@ -8668,17 +8668,17 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F94" s="11" t="inlineStr">
@@ -8693,7 +8693,7 @@
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
@@ -8719,17 +8719,17 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F95" s="11" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I95" s="11" t="inlineStr">
@@ -8770,17 +8770,17 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I96" s="11" t="inlineStr">
@@ -8821,17 +8821,17 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F97" s="11" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3. From the first review.</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
@@ -8872,17 +8872,17 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b. From the first review.</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I98" s="11" t="inlineStr">
@@ -8923,17 +8923,17 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F99" s="11" t="inlineStr">
@@ -8946,7 +8946,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H99" s="11" t="inlineStr"/>
+      <c r="H99" s="11" t="inlineStr">
+        <is>
+          <t>DONE d9fc96b. From the first review.</t>
+        </is>
+      </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8955,7 +8959,7 @@
       <c r="J99" s="11" t="inlineStr"/>
       <c r="K99" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8970,17 +8974,17 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>REQ031</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
@@ -8993,11 +8997,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H100" s="11" t="inlineStr">
-        <is>
-          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
-        </is>
-      </c>
+      <c r="H100" s="11" t="inlineStr"/>
       <c r="I100" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9006,7 +9006,7 @@
       <c r="J100" s="11" t="inlineStr"/>
       <c r="K100" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9021,17 +9021,17 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F101" s="11" t="inlineStr">
@@ -9046,7 +9046,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>Keeps the Chart.js claim (no letter).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
@@ -9057,7 +9057,7 @@
       <c r="J101" s="11" t="inlineStr"/>
       <c r="K101" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9072,12 +9072,12 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Modules p.42</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+          <t>Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -9108,7 +9108,7 @@
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9123,12 +9123,12 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework p.23</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
@@ -9148,7 +9148,7 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
@@ -9159,7 +9159,7 @@
       <c r="J103" s="11" t="inlineStr"/>
       <c r="K103" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9174,12 +9174,12 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
@@ -9197,7 +9197,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H104" s="11" t="inlineStr"/>
+      <c r="H104" s="11" t="inlineStr">
+        <is>
+          <t>Keeps the 'push notifications' claim (no letter).</t>
+        </is>
+      </c>
       <c r="I104" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9221,17 +9225,17 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F105" s="11" t="inlineStr">
@@ -9263,17 +9267,17 @@
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
@@ -9294,7 +9298,7 @@
       <c r="H106" s="11" t="inlineStr"/>
       <c r="I106" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J106" s="11" t="inlineStr"/>
@@ -9310,22 +9314,22 @@
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F107" s="11" t="inlineStr">
@@ -9338,11 +9342,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H107" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H107" s="11" t="inlineStr"/>
       <c r="I107" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -9366,12 +9366,12 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
@@ -9394,9 +9394,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I108" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I108" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J108" s="11" t="inlineStr"/>
@@ -9417,12 +9417,12 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
@@ -9445,9 +9445,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I109" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I109" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J109" s="11" t="inlineStr"/>
@@ -9468,12 +9468,12 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
@@ -9519,12 +9519,12 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
@@ -9544,12 +9544,12 @@
       </c>
       <c r="H111" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J111" s="11" t="inlineStr"/>
@@ -9570,17 +9570,17 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F112" s="11" t="inlineStr">
@@ -9593,7 +9593,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H112" s="11" t="inlineStr"/>
+      <c r="H112" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -9617,12 +9621,12 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -9641,9 +9645,9 @@
         </is>
       </c>
       <c r="H113" s="11" t="inlineStr"/>
-      <c r="I113" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I113" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J113" s="11" t="inlineStr"/>
@@ -9664,12 +9668,12 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
@@ -9711,12 +9715,12 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
@@ -9735,9 +9739,9 @@
         </is>
       </c>
       <c r="H115" s="11" t="inlineStr"/>
-      <c r="I115" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I115" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J115" s="11" t="inlineStr"/>
@@ -9758,12 +9762,12 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
@@ -9805,12 +9809,12 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
@@ -9829,9 +9833,9 @@
         </is>
       </c>
       <c r="H117" s="11" t="inlineStr"/>
-      <c r="I117" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I117" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J117" s="11" t="inlineStr"/>
@@ -9857,7 +9861,7 @@
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
@@ -9899,12 +9903,12 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -9946,12 +9950,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
@@ -9970,9 +9974,9 @@
         </is>
       </c>
       <c r="H120" s="11" t="inlineStr"/>
-      <c r="I120" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I120" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J120" s="11" t="inlineStr"/>
@@ -9993,12 +9997,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -10019,7 +10023,7 @@
       <c r="H121" s="11" t="inlineStr"/>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J121" s="11" t="inlineStr"/>
@@ -10040,12 +10044,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -10064,9 +10068,9 @@
         </is>
       </c>
       <c r="H122" s="11" t="inlineStr"/>
-      <c r="I122" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I122" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J122" s="11" t="inlineStr"/>
@@ -10087,12 +10091,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -10111,9 +10115,9 @@
         </is>
       </c>
       <c r="H123" s="11" t="inlineStr"/>
-      <c r="I123" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I123" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J123" s="11" t="inlineStr"/>
@@ -10134,12 +10138,12 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
@@ -10181,12 +10185,12 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
@@ -10233,7 +10237,7 @@
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -10275,12 +10279,12 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -10322,12 +10326,12 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -10369,12 +10373,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10416,12 +10420,12 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10463,12 +10467,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Appendices (p.124)</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10499,18 +10503,65 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="11" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E132" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F132" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G132" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H132" s="11" t="inlineStr"/>
+      <c r="I132" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J132" s="11" t="inlineStr"/>
+      <c r="K132" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K131"/>
-  <conditionalFormatting sqref="K2:K131">
+  <autoFilter ref="A1:K132"/>
+  <conditionalFormatting sqref="K2:K132">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: live chat, item voids, dashboard period picker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4098,7 +4098,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
+          <t>DONE 80b3988: widget, built-in answers, Gemini via Firebase AI Logic, daily AI limit with usage shown, staff console (reply, take over, hand back, resolve), staff alert. Enable AI Logic in the Firebase console and publish rules. Decide: build (AI needs a server function) or scope down + Limitations. Affects Objective 1, Scope, Comparative Analysis.</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr">
@@ -4139,7 +4139,7 @@
       <c r="J3" s="11" t="inlineStr"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
+          <t>DONE cb08e78: date range shown; Day/Week/Month/Year with previous/next and a date picker; exports name the period. Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
@@ -6547,7 +6547,7 @@
       <c r="J51" s="11" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9595,7 +9595,7 @@
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>DONE 80b3988: widget, built-in answers, Gemini via Firebase AI Logic, daily AI limit with usage shown, staff console (reply, take over, hand back, resolve), staff alert. Enable AI Logic in the Firebase console and publish rules. See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
@@ -9606,7 +9606,7 @@
       <c r="J112" s="11" t="inlineStr"/>
       <c r="K112" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12542,9 +12542,9 @@
           <t>Live chat for guests and customers</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -12554,12 +12554,12 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>Buttons exist but go nowhere.</t>
+          <t>80b3988: chat widget on every shop page for guests and customers. (was: Buttons exist but go nowhere.)</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -12599,9 +12599,9 @@
           <t>AI-powered responses (OpenAI) for common inquiries</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Not built. A browser-only app cannot hide an OpenAI key, so this needs a server function (e.g. Firebase Cloud Functions, Blaze plan).</t>
+          <t>80b3988: AI replies from Gemini (Firebase AI Logic, free tier) instead of OpenAI, plus built-in answers for common questions. Paper names OpenAI - in the panel letter. (was: Not built. A browser-only app cannot hide an OpenAI key, so this needs a server function (e.g. Firebase Cloud Functions, Blaze plan).)</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -12656,9 +12656,9 @@
           <t>Escalate to staff when needed</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -12668,12 +12668,12 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>80b3988: hands off to staff when asked, when the assistant is unsure, or when the daily AI limit is reached. (was: Not built.)</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -12713,9 +12713,9 @@
           <t>Notify staff of new/escalated chats</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -12725,12 +12725,12 @@
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>80b3988: waiting chats show in the staff notification bell and the Live Chat page. (was: Not built.)</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>57f4d80: no longer shown to Sales Staff. Still missing wholesale-order and chat notifications. (was: Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.)</t>
+          <t>No longer shown to Sales Staff; waiting chats now included (80b3988). Still missing wholesale-order notifications. (was: Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.)</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -15190,7 +15190,7 @@
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>57f4d80: void for completed walk-in sales by BM/Technical (Admin too): reason, original SI No., stock back to the exact batches, optional exchange note + price difference, audit entry. Not yet: second-person approval; exchange item is a note, not a stock movement. (was: No void function at all.)</t>
+          <t>57f4d80 + a771333: void the whole sale or specific items/quantities, with reason, SI No., stock back to the same batches, exchange note, audit entry. Not yet: second-person approval. (was: No void function at all.)</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
@@ -16571,9 +16571,9 @@
           <t>Staff view customer and AI conversations</t>
         </is>
       </c>
-      <c r="D109" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D109" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
@@ -16583,12 +16583,12 @@
       </c>
       <c r="F109" s="11" t="inlineStr">
         <is>
-          <t>Sidebar link goes nowhere on all 12 admin pages.</t>
+          <t>80b3988: Admin -&gt; Live Chat lists every conversation, live. (was: Sidebar link goes nowhere on all 12 admin pages.)</t>
         </is>
       </c>
       <c r="G109" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H109" s="11" t="inlineStr">
@@ -16628,9 +16628,9 @@
           <t>Staff respond to customers</t>
         </is>
       </c>
-      <c r="D110" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D110" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
@@ -16640,12 +16640,12 @@
       </c>
       <c r="F110" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>80b3988: staff reply, take over from the assistant, or hand back. (was: Not built.)</t>
         </is>
       </c>
       <c r="G110" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H110" s="11" t="inlineStr">
@@ -16685,9 +16685,9 @@
           <t>Mark threads resolved</t>
         </is>
       </c>
-      <c r="D111" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D111" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
@@ -16697,12 +16697,12 @@
       </c>
       <c r="F111" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>80b3988: Mark resolved; a new customer message reopens it. (was: Not built.)</t>
         </is>
       </c>
       <c r="G111" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H111" s="11" t="inlineStr">
@@ -17915,7 +17915,7 @@
       </c>
       <c r="F133" s="11" t="inlineStr">
         <is>
-          <t>EmailJS works; QR PH is a static image (missing, see REQ028); OpenAI not integrated.</t>
+          <t>EmailJS works; AI is Gemini via Firebase AI Logic (paper: OpenAI); QR Ph image still missing. (was: EmailJS works; QR PH is a static image (missing, see REQ028); OpenAI not integrated.)</t>
         </is>
       </c>
       <c r="G133" s="11" t="inlineStr">
@@ -19296,9 +19296,9 @@
           <t>Guest</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -19308,7 +19308,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Dead buttons.</t>
+          <t>80b3988</t>
         </is>
       </c>
     </row>
@@ -19328,9 +19328,9 @@
           <t>(no actor connected)</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -19340,7 +19340,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Paper: bubble has no actor line in the overall diagram.</t>
+          <t>80b3988: built; Fig 2.2 still needs the actor line (paper edit).</t>
         </is>
       </c>
     </row>
@@ -19924,9 +19924,9 @@
           <t>Guest</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -19934,7 +19934,11 @@
           <t>REQ035</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr"/>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>80b3988</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -20912,9 +20916,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -20924,7 +20928,7 @@
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>Connected here, but not in Fig 2.2.</t>
+          <t>80b3988</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: keep the chat paper edits open
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -9595,7 +9595,7 @@
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>DONE 80b3988: widget, built-in answers, Gemini via Firebase AI Logic, daily AI limit with usage shown, staff console (reply, take over, hand back, resolve), staff alert. Enable AI Logic in the Firebase console and publish rules. See Contradictions / Paper Edits</t>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
@@ -9606,7 +9606,7 @@
       <c r="J112" s="11" t="inlineStr"/>
       <c r="K112" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: reports, Bad Order, live updates done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4277,7 +4277,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>PARTIAL aece0e7: all 6 Export buttons now produce real PDF/Excel tables of what's on screen; the client's 4 report formats are still to build. Client's one remaining ask (Interview 4). Build to the 4 client samples (see Report Formats sheet); Excel output must paste cleanly into the main office's own sheets (Interviews 1, 2, 4); daily sales should total by payment method to match the daily cash remittance (Interview 2).</t>
+          <t>DONE bf16804: Reports page with Daily Sales, Customer File, Monthly Inventory, Supplier Purchases, Pull-Out and PO Discrepancy in the branch's formats; preview, PDF, Excel. Not yet: Return to POS / wholesale exchange report (needs the exchange feature). Discount, VAT and pay-in/pay-out columns show 0 (client: no discounts; VAT-exempt as in their sample). PARTIAL aece0e7: all 6 Export buttons now produce real PDF/Excel tables of what's on screen; the client's 4 report formats are still to build. Client's one remaining ask (Interview 4). Build to the 4 client samples (see Report Formats sheet); Excel output must paste cleanly into the main office's own sheets (Interviews 1, 2, 4); daily sales should total by payment method to match the daily cash remittance (Interview 2).</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -4288,7 +4288,7 @@
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5059,7 +5059,7 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>DECIDED (revised): build everywhere to avoid a removal letter.</t>
+          <t>DONE 21e505b: orders (staff + customer), inventory, POS today's sales, chat.</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
@@ -5100,7 +5100,7 @@
       <c r="J22" s="11" t="inlineStr"/>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr"/>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>DONE d2a957b: automatic write-off with reason, audit entry, disposal alert, Mark disposed.</t>
+        </is>
+      </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5688,7 +5692,7 @@
       <c r="J34" s="11" t="inlineStr"/>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -13805,9 +13809,9 @@
           <t>Discrepancy reports by date range, PDF/Excel</t>
         </is>
       </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
@@ -13817,12 +13821,12 @@
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>No discrepancy report export.</t>
+          <t>bf16804: Reports -&gt; Purchase Order Discrepancy Report, date range, PDF/Excel. (was: No discrepancy report export.)</t>
         </is>
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
@@ -14294,9 +14298,9 @@
           <t>Within 2 months: Bad Order, disposal alert, auto-deduct</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -14306,12 +14310,12 @@
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>No 2-month Bad Order handling.</t>
+          <t>d2a957b: within 2 months (or expired) the batch becomes Bad Order: remaining units written off automatically (write-off + audit entry), disposal alert until staff Mark disposed. (was: No 2-month Bad Order handling.)</t>
         </is>
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr">
@@ -16742,9 +16746,9 @@
           <t>Export daily sales reports (from Order Processing)</t>
         </is>
       </c>
-      <c r="D112" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D112" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -16754,12 +16758,12 @@
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: Online Orders Export now gives real PDF/Excel of the listed orders. Client's daily sales format still to build. (was: Online Orders Export downloads a blank PDF. Dashboard Sales Analytics export works but is not the daily sales report the client described (per customer, items with batch + expiry).)</t>
+          <t>bf16804: Reports -&gt; Daily Sales Report in the branch's format (sales, retail, wholesale, payment method, items sold) + Customer File; shortcut on Orders. (was: Online Orders Export downloads a blank PDF. Dashboard Sales Analytics export works but is not the daily sales report the client described (per customer, items with batch + expiry).)</t>
         </is>
       </c>
       <c r="G112" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H112" s="11" t="inlineStr">
@@ -16799,9 +16803,9 @@
           <t>Export monthly inventory + purchase reports (from Inventory)</t>
         </is>
       </c>
-      <c r="D113" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D113" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -16811,12 +16815,12 @@
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: Inventory Export now gives real PDF/Excel by batch (expiry, supplier, receipt/DR no., unit cost, date received). Client's monthly format still to build. (was: Inventory Export downloads a blank PDF.)</t>
+          <t>bf16804: Reports -&gt; Monthly Inventory (sheet per category, POS vs physical, prices, batch, expiry) + Supplier Purchases; shortcut on Inventory. (was: Inventory Export downloads a blank PDF.)</t>
         </is>
       </c>
       <c r="G113" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H113" s="11" t="inlineStr">
@@ -16856,9 +16860,9 @@
           <t>Pull-out reports by date range</t>
         </is>
       </c>
-      <c r="D114" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D114" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
@@ -16868,12 +16872,12 @@
       </c>
       <c r="F114" s="11" t="inlineStr">
         <is>
-          <t>Not built (write-offs are recorded, so data exists).</t>
+          <t>bf16804: Reports -&gt; Pull-Out Report (write-offs incl. automatic Bad Order) by date range. (was: Not built (write-offs are recorded, so data exists).)</t>
         </is>
       </c>
       <c r="G114" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H114" s="11" t="inlineStr">
@@ -16966,9 +16970,9 @@
           <t>All reports in PDF or Excel</t>
         </is>
       </c>
-      <c r="D116" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
@@ -16978,12 +16982,12 @@
       </c>
       <c r="F116" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: all 6 Export buttons now give real PDF or Excel. Client report formats still to build. (was: Only Sales Analytics exports (PDF + Excel). Five other Export buttons give blank PDFs (Dashboard, Inventory, Online Orders, Suppliers, Audit Log).)</t>
+          <t>bf16804: every report previews on screen and downloads as PDF or Excel. (was: Only Sales Analytics exports (PDF + Excel). Five other Export buttons give blank PDFs (Dashboard, Inventory, Online Orders, Suppliers, Audit Log).)</t>
         </is>
       </c>
       <c r="G116" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H116" s="11" t="inlineStr"/>
@@ -17736,9 +17740,9 @@
           <t>Inventory/order changes appear without manual refresh</t>
         </is>
       </c>
-      <c r="D130" s="16" t="inlineStr">
-        <is>
-          <t>Deviates</t>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -17748,12 +17752,12 @@
       </c>
       <c r="F130" s="11" t="inlineStr">
         <is>
-          <t>Users must reload to see new orders or stock changes.</t>
+          <t>21e505b: online orders, inventory, POS today's sales, customer order list and order page, and chat update live. Dashboard tiles refresh on load. (was: Users must reload to see new orders or stock changes.)</t>
         </is>
       </c>
       <c r="G130" s="11" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H130" s="11" t="inlineStr">
@@ -17793,9 +17797,9 @@
           <t>Reports in reasonable time</t>
         </is>
       </c>
-      <c r="D131" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D131" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -17805,7 +17809,7 @@
       </c>
       <c r="F131" s="11" t="inlineStr">
         <is>
-          <t>Reports not built yet.</t>
+          <t>Reports query only the chosen period's sales, write-offs and POs. (was: Reports not built yet.)</t>
         </is>
       </c>
       <c r="G131" s="11" t="inlineStr">
@@ -18563,9 +18567,9 @@
           <t>Data export in PDF and Excel</t>
         </is>
       </c>
-      <c r="D145" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D145" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
@@ -18575,12 +18579,12 @@
       </c>
       <c r="F145" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: every Export button offers PDF or Excel. (was: Only Sales Analytics exports.)</t>
+          <t>Every report and Export button gives PDF or Excel. (was: Only Sales Analytics exports.)</t>
         </is>
       </c>
       <c r="G145" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H145" s="11" t="inlineStr">
@@ -19592,9 +19596,9 @@
           <t>Technical Staff</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -19604,7 +19608,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: exports are real PDF/Excel; client report formats still to build.</t>
+          <t>bf16804: Reports page.</t>
         </is>
       </c>
     </row>
@@ -20428,9 +20432,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -20440,7 +20444,7 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>6-month flag yes; 2-month Bad Order missing.</t>
+          <t>6-month Wholesale Only + 2-month Bad Order (d2a957b).</t>
         </is>
       </c>
     </row>
@@ -20788,9 +20792,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D56" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -20800,7 +20804,7 @@
       </c>
       <c r="F56" s="11" t="inlineStr">
         <is>
-          <t>aece0e7: exports are real PDF/Excel; client report formats still to build.</t>
+          <t>bf16804: Reports page in the client's formats.</t>
         </is>
       </c>
     </row>
@@ -22437,17 +22441,17 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>d2a957b: built; diagram box should say 'Write off batch (Bad Order)', not FEFO deduction</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register: exchange, agreed prices, banner, void approval, notifications
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -5632,7 +5632,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr"/>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>DONE Purchase History -&gt; Exchange: return to batch, FEFO replacement, value rule, audit, exchange document; Return / Exchange report.</t>
+        </is>
+      </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5641,7 +5645,7 @@
       <c r="J33" s="11" t="inlineStr"/>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6187,7 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>Shown to the client during the prototype walkthrough.</t>
+          <t>DONE Reports -&gt; Supplier Purchases (per supplier, per month). Shown to the client during the prototype walkthrough.</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
@@ -6194,7 +6198,7 @@
       <c r="J44" s="11" t="inlineStr"/>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6442,7 @@
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>Keeps per-account pricing (no letter).</t>
+          <t>DONE saved from Process Order, listed in Edit account, default on orders. Keeps per-account pricing (no letter).</t>
         </is>
       </c>
       <c r="I49" s="12" t="inlineStr">
@@ -6449,7 +6453,7 @@
       <c r="J49" s="11" t="inlineStr"/>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6593,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr"/>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
+        </is>
+      </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6598,7 +6606,7 @@
       <c r="J52" s="11" t="inlineStr"/>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9009,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H100" s="11" t="inlineStr"/>
+      <c r="H100" s="11" t="inlineStr">
+        <is>
+          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
+        </is>
+      </c>
       <c r="I100" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9010,7 +9022,7 @@
       <c r="J100" s="11" t="inlineStr"/>
       <c r="K100" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9264,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H105" s="11" t="inlineStr"/>
+      <c r="H105" s="11" t="inlineStr">
+        <is>
+          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
+        </is>
+      </c>
       <c r="I105" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9261,7 +9277,7 @@
       <c r="J105" s="11" t="inlineStr"/>
       <c r="K105" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10134,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H123" s="11" t="inlineStr"/>
+      <c r="H123" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
       <c r="I123" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10127,7 +10147,7 @@
       <c r="J123" s="11" t="inlineStr"/>
       <c r="K123" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11055,9 +11075,9 @@
           <t>Home page with products, announcements, promotions, navigation</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -11067,12 +11087,12 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Featured products and categories exist; no announcements or promotions section.</t>
+          <t>Announcement / promotion banner on every shop page, edited in Settings by the BM or Technical Staff. (was: Featured products and categories exist; no announcements or promotions section.)</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -12786,7 +12806,7 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>In-platform bell works; no email notifications are sent (EmailJS is only used for OTP). No notification at all when an order is placed (Fig 2.10 'Send Order Submission Notification').</t>
+          <t>In-platform notifications for order placed, payment confirmed, holds, prescription results, ready for pick-up. Email notifications not built. (was: In-platform bell works; no email notifications are sent (EmailJS is only used for OTP). No notification at all when an order is placed (Fig 2.10 'Send Order Submission Notification').)</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -13271,9 +13291,9 @@
           <t>Notify BM + Technical of new orders, payments, stock, expiry, wholesale updates, chat</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
@@ -13283,12 +13303,12 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>No longer shown to Sales Staff; waiting chats now included (80b3988). Still missing wholesale-order notifications. (was: Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.)</t>
+          <t>Staff bell: orders, payments, stock, expiry, Bad Order disposal, PO discrepancies, wholesale document expiry, waiting chats. (was: Covers orders, payments, stock, expiry, PO discrepancies. No wholesale order updates or chat. Also shown to Sales Staff.)</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
@@ -15182,9 +15202,9 @@
           <t>Void with reason, restore stock, audit log, record exchange + price difference</t>
         </is>
       </c>
-      <c r="D84" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D84" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -15194,12 +15214,12 @@
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>57f4d80 + a771333: void the whole sale or specific items/quantities, with reason, SI No., stock back to the same batches, exchange note, audit entry. Not yet: second-person approval. (was: No void function at all.)</t>
+          <t>Full or item-level voids with reason, SI No., stock back to the same batches, exchange note, audit entry; Technical Staff voids need a Branch Manager's email + password approval (client rule). (was: No void function at all.)</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr">
@@ -15296,9 +15316,9 @@
           <t>Wholesale accounts with contact, business type, agreed pricing</t>
         </is>
       </c>
-      <c r="D86" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D86" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -15308,12 +15328,12 @@
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>No per-account agreed pricing; price comes from the product's wholesale price and can be edited per order.</t>
+          <t>Agreed price per buyer per product (saved from Process Order, reviewed in Edit), used as the default on their orders. (was: No per-account agreed pricing; price comes from the product's wholesale price and can be edited per order.)</t>
         </is>
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>Change paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr">
@@ -15422,7 +15442,7 @@
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POs recorded against the buyer with their agreed prices as defaults. (was: -)</t>
         </is>
       </c>
       <c r="G88" s="11" t="inlineStr">
@@ -15577,9 +15597,9 @@
           <t>Wholesale item exchanges with FEFO + audit log</t>
         </is>
       </c>
-      <c r="D91" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D91" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
@@ -15589,12 +15609,12 @@
       </c>
       <c r="F91" s="11" t="inlineStr">
         <is>
-          <t>Not built.</t>
+          <t>Wholesale exchange from Purchase History: return to the original batch, FEFO replacement, equal-or-higher value (buyer pays the difference), reason, audit entry, exchange document (EX-#####). (was: Not built.)</t>
         </is>
       </c>
       <c r="G91" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H91" s="11" t="inlineStr">
@@ -16917,9 +16937,9 @@
           <t>Wholesale exchange reports by period</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D115" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
@@ -16929,12 +16949,12 @@
       </c>
       <c r="F115" s="11" t="inlineStr">
         <is>
-          <t>Not built; depends on REQ090.</t>
+          <t>Reports -&gt; Return / Exchange Report (the branch's 'Return to POS' sheet + replacement and difference). (was: Not built; depends on REQ090.)</t>
         </is>
       </c>
       <c r="G115" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H115" s="11" t="inlineStr"/>
@@ -21044,9 +21064,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -21054,7 +21074,11 @@
           <t>REQ090</t>
         </is>
       </c>
-      <c r="F64" s="11" t="inlineStr"/>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>Purchase History -&gt; Exchange.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -21072,9 +21096,9 @@
           <t>Technical Staff (+BM)</t>
         </is>
       </c>
-      <c r="D65" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
@@ -21082,7 +21106,11 @@
           <t>REQ090</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr"/>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>Return to batch + FEFO replacement in one transaction.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
@@ -21857,17 +21885,17 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Only an on-screen confirmation with the order number; no notification</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Order-placed notice in the customer's bell</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -22840,17 +22868,17 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Built from Purchase History</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
@@ -22877,17 +22905,17 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Returned units back to their batch + FEFO replacement</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr">
@@ -22914,17 +22942,17 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E45" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Audit entry + exchange document; diagram should say 'Generate Wholesale Exchange Document'</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register: inventory chart and desktop alerts done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -9113,7 +9113,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>Keeps the Chart.js claim (no letter).</t>
+          <t>DONE Dashboard: stock in vs stock out per day/week/month/year. Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -9124,7 +9124,7 @@
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr">
@@ -9226,7 +9226,7 @@
       <c r="J104" s="11" t="inlineStr"/>
       <c r="K104" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9758,7 +9758,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H115" s="11" t="inlineStr"/>
+      <c r="H115" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
       <c r="I115" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -9767,7 +9771,7 @@
       <c r="J115" s="11" t="inlineStr"/>
       <c r="K115" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9950,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H119" s="11" t="inlineStr"/>
+      <c r="H119" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
+        </is>
+      </c>
       <c r="I119" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -9955,7 +9963,7 @@
       <c r="J119" s="11" t="inlineStr"/>
       <c r="K119" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: email notifications done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -5940,7 +5940,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>EmailJS free tier: 200/month.</t>
+          <t>DONE EmailJS order template (ID to paste in js/emailjs-config.js) + on/off toggle in Account Settings. EmailJS free tier: 200/month.</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -5951,7 +5951,7 @@
       <c r="J39" s="11" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12802,9 +12802,9 @@
           <t>In-platform and email notifications for order/payment/delivery updates</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -12814,12 +12814,12 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>In-platform notifications for order placed, payment confirmed, holds, prescription results, ready for pick-up. Email notifications not built. (was: In-platform bell works; no email notifications are sent (EmailJS is only used for OTP). No notification at all when an order is placed (Fig 2.10 'Send Order Submission Notification').)</t>
+          <t>In-platform + EmailJS email for order placed, payment confirmed, holds, prescription results, dispatched (tracking link), ready for pick-up, credit. Needs the order template ID in js/emailjs-config.js. (was: In-platform bell works; no email notifications are sent (EmailJS is only used for OTP). No notification at all when an order is placed (Fig 2.10 'Send Order Submission Notification').)</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -12969,9 +12969,9 @@
           <t>Enable/disable email notifications</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
@@ -12981,12 +12981,12 @@
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>No toggle (and no email notifications yet).</t>
+          <t>Account Settings -&gt; Notifications: email updates on/off. (was: No toggle (and no email notifications yet).)</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H43" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register and README: new-device login code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -157,9 +157,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -167,6 +164,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5534,7 +5534,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr"/>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>DONE 7ede9d4: emailed code on new browsers, customers and staff; recognized devices in Account Settings.</t>
+        </is>
+      </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5543,7 +5547,7 @@
       <c r="J31" s="11" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10916,29 +10920,29 @@
           <t>Email OTP when logging in from an unrecognized device</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>js/device-trust.js; js/auth.js</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>No device recognition or login OTP exists.</t>
+          <t>Built (7ede9d4): new browser gets an emailed 6-digit code (10 min, 5 tries, resend after 60 s); recognized devices in Account Settings. Checked in the browser, not by database rules.</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Also in Fig 2.3 (Verify OTP) and Activity 2.8; OTP + EmailJS code already exists (js/otp.js) to reuse.</t>
+          <t>Paper may add: the device check runs in the browser.</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -12350,7 +12354,7 @@
           <t>Statuses: pending payment, payment verified, confirmed, dispatched, delivered, payment rejected</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -12631,7 +12635,7 @@
           <t>AI-powered responses (OpenAI) for common inquiries</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -13079,31 +13083,27 @@
           <t>Staff OTP only on unrecognized device</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>js/device-trust.js; js/admin-header.js</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Not built (same as REQ005).</t>
+          <t>Built with REQ005 (7ede9d4); admin pages send an unconfirmed device back to login.</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
-        </is>
-      </c>
-      <c r="H45" s="11" t="inlineStr">
-        <is>
-          <t>Do together with REQ005.</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr"/>
       <c r="I45" s="11" t="inlineStr">
         <is>
           <t>Med</t>
@@ -16045,7 +16045,7 @@
           <t>On Hold - Overpayment, excess as unapplied value</t>
         </is>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D99" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -16436,7 +16436,7 @@
           <t>Reflect status to customer; customer 'Order Received' finalizes as Delivered</t>
         </is>
       </c>
-      <c r="D106" s="16" t="inlineStr">
+      <c r="D106" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -17654,7 +17654,7 @@
           <t>Works on desktop, laptop, tablet, phone</t>
         </is>
       </c>
-      <c r="D128" s="17" t="inlineStr">
+      <c r="D128" s="16" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -17711,7 +17711,7 @@
           <t>Standard operations load in reasonable time</t>
         </is>
       </c>
-      <c r="D129" s="17" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -17878,7 +17878,7 @@
           <t>Chrome, Firefox, Edge, Safari</t>
         </is>
       </c>
-      <c r="D132" s="17" t="inlineStr">
+      <c r="D132" s="16" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -18159,7 +18159,7 @@
           <t>No patient data sent to OpenAI</t>
         </is>
       </c>
-      <c r="D137" s="18" t="inlineStr">
+      <c r="D137" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -18216,7 +18216,7 @@
           <t>Hosted with uptime + recovery</t>
         </is>
       </c>
-      <c r="D138" s="15" t="inlineStr">
+      <c r="D138" s="18" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
@@ -18652,7 +18652,7 @@
           <t>Usable with basic digital literacy</t>
         </is>
       </c>
-      <c r="D146" s="17" t="inlineStr">
+      <c r="D146" s="16" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -20104,9 +20104,9 @@
           <t>Staff, Registered User</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -20116,7 +20116,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>Verify OTP not built.</t>
+          <t>Built (7ede9d4).</t>
         </is>
       </c>
     </row>
@@ -20884,7 +20884,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -20916,7 +20916,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21453,22 +21453,22 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Same (js/auth.js startDeviceVerification)</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Change system</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>REQ005/REQ044.</t>
+          <t>REQ005/REQ044, 7ede9d4.</t>
         </is>
       </c>
     </row>
@@ -21493,7 +21493,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -21530,7 +21530,7 @@
           <t>reCAPTCHA check, rejecting attempts while locked, blocking deactivated accounts, sending unverified customers to email verification</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21567,7 +21567,7 @@
           <t>Terms modal opens when the checkbox is ticked (before submit); duplicate email is caught by Firebase at account creation; code sent after</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21641,7 +21641,7 @@
           <t>Goes straight to the shop, already signed in</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21785,7 +21785,7 @@
           <t>RX detected when checkout opens; address section hidden; pick-up only</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21822,7 +21822,7 @@
           <t>Required on the payment page for RX orders</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21933,7 +21933,7 @@
           <t>Login required to check out, delivery schedule, store credit discount, live stock re-check before submitting</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -21970,7 +21970,7 @@
           <t>Stock is deducted first; if stock ran out the order goes on an Out of Stock hold instead</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22007,7 +22007,7 @@
           <t>RX orders skip courier booking and go straight to Ready for Pick-up</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22151,7 +22151,7 @@
           <t>Every resolution returns to staff (resubmission or Release Hold)</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22188,7 +22188,7 @@
           <t>Approved immediately; excess added to store credit</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22225,7 +22225,7 @@
           <t>Closed automatically after 7 days, with verified payment kept as credit</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22262,7 +22262,7 @@
           <t>Fully credit-covered orders (no screenshot), Release Hold by staff</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22369,7 +22369,7 @@
           <t>Partial stock added, PO marked Discrepancy, acknowledgment required to close</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22406,7 +22406,7 @@
           <t>Both exist (manual Receive Stock, Excel/CSV upload)</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>Deviates</t>
         </is>
@@ -22517,7 +22517,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -22990,7 +22990,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E46" s="18" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -23397,12 +23397,12 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>No OTP yet.</t>
+          <t>System follows the text: a wrong code shows tries left, Resend sends a new one; 5 wrong codes sign the person out (does not feed the password lockout).</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Pick one when building REQ005/044; update the other.</t>
+          <t>Change the Fig 2.8 diagram: 'No' from Validate OTP goes back to Enter OTP / Request new OTP, not the failed-attempt counter.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
After registering, go to the login page instead of signing straight in
Matches Fig 2.9 (after verification, go to Login). The email is filled in
and a success notice is shown. Unverified customers who verify after a
later login still go straight to the shop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -21638,22 +21638,22 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Goes straight to the shop, already signed in</t>
-        </is>
-      </c>
-      <c r="E9" s="15" t="inlineStr">
-        <is>
-          <t>Deviates</t>
+          <t>Same: after registering, the code signs them out and opens Login with the email filled in</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Matches</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Change paper</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>C10.</t>
+          <t>C10 resolved.</t>
         </is>
       </c>
     </row>
@@ -23316,12 +23316,12 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Redirects straight to the shop (already signed in).</t>
+          <t>System now matches: after registration it goes to Login.</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Change paper (minor).</t>
+          <t>No change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: security items, wholesale release and sales report batch details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$137</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4757,22 +4757,22 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>REQ083, REQ122, Fig 2.6, Fig 2.14, C4</t>
+          <t>REQNF011, REQ121</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Walk-in void: reason, original receipt no., automatic stock restore, optional exchange item + price difference, audit entry; restricted to authorized role</t>
+          <t>Database rules per staff role: Sales Staff limited to POS + read-only catalog in the rules too, not only in the page menus</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -4787,18 +4787,18 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: BM/Technical void completed sales from POS Today's Sales or Walk-in Orders: reason, SI No., stock restored to the same batches, exchange note + price difference, audit entry. Still open: second-person approval (client rule) and exchange as a real stock movement. Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
+          <t>Pages already block Sales Staff; someone with technical know-how could still write other collections directly.</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr"/>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4813,22 +4813,22 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>REQ098, REQ102, C2</t>
+          <t>REQ083, REQ122, Fig 2.6, Fig 2.14, C4</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Fix overpayment approval: clear the old hold, send 'Payment confirmed' notification; reword REQ098</t>
+          <t>Walk-in void: reason, original receipt no., automatic stock restore, optional exchange item + price difference, audit entry; restricted to authorized role</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b (system part; REQ098 paper wording still to do). From the first review.</t>
+          <t>DONE 57f4d80: BM/Technical void completed sales from POS Today's Sales or Walk-in Orders: reason, SI No., stock restored to the same batches, exchange note + price difference, audit entry. Still open: second-person approval (client rule) and exchange as a real stock movement. Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
@@ -4864,17 +4864,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>REQ071, REQ073, REQ120, REQNF011, C8</t>
+          <t>REQ098, REQ102, C2</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Price lock: only Branch Manager sets prices on create/import too; enforce in database rules; add a reason to each price change</t>
+          <t>Fix overpayment approval: clear the old hold, send 'Payment confirmed' notification; reword REQ098</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>DONE BM-only prices in the form, batch import and quick-add (others' products saved Inactive + 'Price pending'); reason required and logged; enforced in firestore.rules - PUBLISH THE RULES in the Firebase console.</t>
+          <t>DONE e1e200b (system part; REQ098 paper wording still to do). From the first review.</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
@@ -4910,22 +4910,22 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Removals (Letter) sheet</t>
+          <t>REQ071, REQ073, REQ120, REQNF011, C8</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Letter to the panel: OpenAI -&gt; Gemini (free), Firebase Storage -&gt; Cloudinary, DataTable -&gt; custom tables, password reset via Firebase Auth, overpayment approve-and-credit, corrections to scope/conceptual framework</t>
+          <t>Price lock: only Branch Manager sets prices on create/import too; enforce in database rules; add a reason to each price change</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -4940,18 +4940,18 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>One letter covers all remaining removals; send before the paper edits.</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE BM-only prices in the form, batch import and quick-add (others' products saved Inactive + 'Price pending'); reason required and logged; enforced in firestore.rules - PUBLISH THE RULES in the Firebase console.</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4966,22 +4966,22 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Objectives / evaluation (p.5-6, 21-24)</t>
+          <t>Removals (Letter) sheet</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
+          <t>Letter to the panel: OpenAI -&gt; Gemini (free), Firebase Storage -&gt; Cloudinary, DataTable -&gt; custom tables, password reset via Firebase Auth, overpayment approve-and-credit, corrections to scope/conceptual framework</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -4989,10 +4989,14 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr"/>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>One letter covers all remaining removals; send before the paper edits.</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr"/>
@@ -5008,48 +5012,44 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>REQ121</t>
+          <t>Objectives / evaluation (p.5-6, 21-24)</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
+          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>Med</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>DONE 57f4d80: POS (with Today's Sales) + read-only catalog; lands on POS after login. Orders access was added on purpose on 2026-10-01.</t>
-        </is>
-      </c>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr"/>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr"/>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5064,12 +5064,12 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>REQNF005</t>
+          <t>REQ121</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Live updates without refresh on all order and inventory screens (staff + customer)</t>
+          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -5089,12 +5089,12 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>DONE 21e505b: orders (staff + customer), inventory, POS today's sales, chat.</t>
-        </is>
-      </c>
-      <c r="I22" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE 57f4d80: POS (with Today's Sales) + read-only catalog; lands on POS after login. Orders access was added on purpose on 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr"/>
@@ -5110,27 +5110,27 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>REQNF010, REQNF013</t>
+          <t>REQNF005</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
+          <t>Live updates without refresh on all order and inventory screens (staff + customer)</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -5140,18 +5140,18 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: Netlify (already set up).</t>
-        </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>DONE 21e505b: orders (staff + customer), inventory, POS today's sales, chat.</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr"/>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5166,12 +5166,12 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
+          <t>REQNF010, REQNF013</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Discount / deduction per sale or line, with reason and audit entry</t>
+          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -5191,18 +5191,18 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
+          <t>DECIDED: Netlify (already set up).</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr"/>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5217,12 +5217,12 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
+          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
+          <t>Discount / deduction per sale or line, with reason and audit entry</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -5242,18 +5242,18 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr"/>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -5263,27 +5263,27 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Limitations (p.7)</t>
+          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
+          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -5291,7 +5291,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr"/>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+        </is>
+      </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5300,7 +5304,7 @@
       <c r="J26" s="11" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5324,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
+          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -5362,12 +5366,12 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Limitations (p.7)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
+          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -5404,22 +5408,22 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
+          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -5432,11 +5436,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>DONE d9fc96b: locks itself after one run; SI counter now staff-only in rules (publish rules). From the first review.</t>
-        </is>
-      </c>
+      <c r="H29" s="11" t="inlineStr"/>
       <c r="I29" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5445,7 +5445,7 @@
       <c r="J29" s="11" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5460,12 +5460,12 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>REQ002</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
+          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>From the first review.</t>
+          <t>DONE d9fc96b: locks itself after one run; SI counter now staff-only in rules (publish rules). From the first review.</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
@@ -5496,7 +5496,7 @@
       <c r="J30" s="11" t="inlineStr"/>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5511,22 +5511,22 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
+          <t>REQ002</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Unrecognized-device OTP for customers and staff</t>
+          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>DONE 7ede9d4: emailed code on new browsers, customers and staff; recognized devices in Account Settings.</t>
+          <t>From the first review.</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
@@ -5547,7 +5547,7 @@
       <c r="J31" s="11" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5562,17 +5562,17 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>REQ086, REQ089, REQ091, REQ092</t>
+          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
+          <t>Unrecognized-device OTP for customers and staff</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>DONE 5cad255: history, sales invoice PDF, free-of-cost, LTO/permit validity. Not built: reorder from a past order. Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
+          <t>DONE 7ede9d4: emailed code on new browsers, customers and staff; recognized devices in Account Settings.</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -5613,17 +5613,17 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>REQ090, REQ114, Fig 2.15</t>
+          <t>REQ086, REQ089, REQ091, REQ092</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
+          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>DONE Purchase History -&gt; Exchange: return to batch, FEFO replacement, value rule, audit, exchange document; Return / Exchange report.</t>
+          <t>DONE 5cad255: history, sales invoice PDF, free-of-cost, LTO/permit validity. Not built: reorder from a past order. Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
@@ -5664,12 +5664,12 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>REQ067, C7</t>
+          <t>REQ090, REQ114, Fig 2.15</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
+          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>DONE d2a957b: automatic write-off with reason, audit entry, disposal alert, Mark disposed.</t>
+          <t>DONE Purchase History -&gt; Exchange: return to batch, FEFO replacement, value rule, audit, exchange document; Return / Exchange report.</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -5715,12 +5715,12 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
+          <t>REQ067, C7</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
+          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout. The 'not an official receipt' line was removed from POS and online receipts on 2026-10-21 at the team's request.</t>
+          <t>DONE d2a957b: automatic write-off with reason, audit entry, disposal alert, Mark disposed.</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -5766,12 +5766,12 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>REQ084</t>
+          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>POS: RX Verified checkbox + optional notes</t>
+          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: checkbox + notes, required for RX items, saved on the sale.</t>
+          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout. The 'not an official receipt' line was removed from POS and online receipts on 2026-10-21 at the team's request.</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
@@ -5817,17 +5817,17 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>REQ061, C5</t>
+          <t>REQ084</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
+          <t>POS: RX Verified checkbox + optional notes</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: others save counts; BM finalizes; variance reason required and logged.</t>
+          <t>DONE 57f4d80: checkbox + notes, required for RX items, saved on the sale.</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
@@ -5868,17 +5868,17 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>REQNF025, REQNF029</t>
+          <t>REQ061, C5</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
+          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>DONE footer rebuilt from js/store-info.js (real About text, links to legal.html; contact/LTO lines hidden until the client confirms them); chat links hidden until chat is built; payment page Terms link fixed. From the first review.</t>
+          <t>DONE 06574da: others save counts; BM finalizes; variance reason required and logged.</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -5919,22 +5919,22 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>REQ039, REQ042</t>
+          <t>REQNF025, REQNF029</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
+          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>DONE EmailJS order template (ID to paste in js/emailjs-config.js) + on/off toggle in Account Settings. EmailJS free tier: 200/month.</t>
+          <t>DONE footer rebuilt from js/store-info.js (real About text, links to legal.html; contact/LTO lines hidden until the client confirms them); chat links hidden until chat is built; payment page Terms link fixed. From the first review.</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -5970,12 +5970,12 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>REQ122</t>
+          <t>REQ039, REQ042</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
+          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -5993,7 +5993,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr"/>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>DONE EmailJS order template (ID to paste in js/emailjs-config.js) + on/off toggle in Account Settings. EmailJS free tier: 200/month.</t>
+        </is>
+      </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6002,7 +6006,7 @@
       <c r="J40" s="11" t="inlineStr"/>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6017,22 +6021,22 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>REQ014</t>
+          <t>REQ122</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Save cart to the customer's account</t>
+          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -6040,11 +6044,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr">
-        <is>
-          <t>DONE 77336f3.</t>
-        </is>
-      </c>
+      <c r="H41" s="11" t="inlineStr"/>
       <c r="I41" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6053,7 +6053,7 @@
       <c r="J41" s="11" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6068,17 +6068,17 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>REQNF003, REQNF007</t>
+          <t>REQ014</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Phone/tablet and cross-browser test pass</t>
+          <t>Save cart to the customer's account</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
@@ -6091,7 +6091,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H42" s="11" t="inlineStr"/>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>DONE 77336f3.</t>
+        </is>
+      </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6100,7 +6104,7 @@
       <c r="J42" s="11" t="inlineStr"/>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6115,17 +6119,17 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Interviews 2, 4</t>
+          <t>REQNF003, REQNF007</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
+          <t>Phone/tablet and cross-browser test pass</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Not verified</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
@@ -6138,11 +6142,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
-        <is>
-          <t>DONE e1e200b. Required column in the monthly purchases report.</t>
-        </is>
-      </c>
+      <c r="H43" s="11" t="inlineStr"/>
       <c r="I43" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6151,7 +6151,7 @@
       <c r="J43" s="11" t="inlineStr"/>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6166,12 +6166,12 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Interview 4 walkthrough</t>
+          <t>Interviews 2, 4</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Supplier history: everything received from each supplier</t>
+          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>DONE Reports -&gt; Supplier Purchases (per supplier, per month). Shown to the client during the prototype walkthrough.</t>
+          <t>DONE e1e200b. Required column in the monthly purchases report.</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30; Interview 4</t>
+          <t>Interview 4 walkthrough</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>User manual + hands-on training + handover to the branch</t>
+          <t>Supplier history: everything received from each supplier</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
+          <t>DONE Reports -&gt; Supplier Purchases (per supplier, per month). Shown to the client during the prototype walkthrough.</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
@@ -6253,7 +6253,7 @@
       <c r="J45" s="11" t="inlineStr"/>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6268,12 +6268,12 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
+          <t>Methodology p.30; Interview 4</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
+          <t>User manual + hands-on training + handover to the branch</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G46" s="11" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b. Customer File groups every sale by customer name.</t>
+          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
@@ -6304,7 +6304,7 @@
       <c r="J46" s="11" t="inlineStr"/>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6319,17 +6319,17 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Supplier sheets)</t>
+          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
+          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b: unit cost + receipt/DR no. added; pack size stays in the product name as the branch does today. Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
+          <t>DONE e1e200b. Customer File groups every sale by customer name.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
@@ -6370,17 +6370,17 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
+          <t>Report Formats sheet (Supplier sheets)</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
+          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b: also storefront links/filters now follow Manage Categories. Existing Firebase projects keep their current categories - add the client's in Manage Categories.. Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+          <t>DONE e1e200b: unit cost + receipt/DR no. added; pack size stays in the product name as the branch does today. Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
@@ -6421,22 +6421,22 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087</t>
+          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Optional agreed price per wholesale buyer per product, used as default on their orders</t>
+          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -6446,12 +6446,12 @@
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>DONE saved from Process Order, listed in Edit account, default on orders. Keeps per-account pricing (no letter).</t>
-        </is>
-      </c>
-      <c r="I49" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE e1e200b: also storefront links/filters now follow Manage Categories. Existing Firebase projects keep their current categories - add the client's in Manage Categories.. Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr"/>
@@ -6472,12 +6472,12 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Production readiness</t>
+          <t>REQ085, REQ087</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Cut database reads: stop loading whole collections on every page (Firestore free-plan daily read cap ~50k)</t>
+          <t>Optional agreed price per wholesale buyer per product, used as default on their orders</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -6497,18 +6497,18 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>Needed before real use with the client's ~1,000-product catalog.</t>
-        </is>
-      </c>
-      <c r="I50" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>DONE saved from Process Order, listed in Edit account, default on orders. Keeps per-account pricing (no letter).</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr"/>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6523,22 +6523,22 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module p.40; Interview 4 (dashboard export)</t>
+          <t>Production readiness</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Dashboard Sales Analytics: show which dates the Today/Week/Month/Year view covers, and add a picker to choose a specific day, week, month or year (with previous/next)</t>
+          <t>Cut database reads: stop loading whole collections on every page (Firestore free-plan daily read cap ~50k)</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>DONE cb08e78: date range shown; Day/Week/Month/Year with previous/next and a date picker; exports name the period. Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
+          <t>Needed before real use with the client's ~1,000-product catalog.</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
@@ -6559,7 +6559,7 @@
       <c r="J51" s="11" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6574,17 +6574,17 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>Dashboard module p.40; Interview 4 (dashboard export)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>Dashboard Sales Analytics: show which dates the Today/Week/Month/Year view covers, and add a picker to choose a specific day, week, month or year (with previous/next)</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
@@ -6599,7 +6599,7 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
+          <t>DONE cb08e78: date range shown; Day/Week/Month/Year with previous/next and a date picker; exports name the period. Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
@@ -6625,17 +6625,17 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>REQ048, Notification module</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Admin notification for pending wholesale orders (Pending -&gt; Released)</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+          <t>DONE 274b8e0: wholesale orders start Pending; Mark Released in purchase history; staff notification.</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
@@ -6661,7 +6661,7 @@
       <c r="J53" s="11" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6676,17 +6676,17 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>REQ111, Sales Report module</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>Daily Sales report: batch, expiry, date received and supplier per item sold</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>DONE footer links to legal.html on every page.</t>
+          <t>DONE 274b8e0: 'Item Sold by Batch' section.</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
@@ -6712,7 +6712,7 @@
       <c r="J54" s="11" t="inlineStr"/>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6722,17 +6722,17 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
@@ -6752,12 +6752,12 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr"/>
@@ -6773,22 +6773,22 @@
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -6803,18 +6803,18 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr"/>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6824,22 +6824,22 @@
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
@@ -6854,18 +6854,18 @@
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I57" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE footer links to legal.html on every page.</t>
+        </is>
+      </c>
+      <c r="I57" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6875,22 +6875,22 @@
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
@@ -6905,18 +6905,18 @@
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I58" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr"/>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6931,12 +6931,12 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
@@ -6982,12 +6982,12 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -7010,9 +7010,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr"/>
@@ -7033,12 +7033,12 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -7112,9 +7112,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I62" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr"/>
@@ -7135,12 +7135,12 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
@@ -7186,12 +7186,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -7214,9 +7214,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr"/>
@@ -7237,12 +7237,12 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
@@ -7265,9 +7265,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I65" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I65" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr"/>
@@ -7288,12 +7288,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -7339,12 +7339,12 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
@@ -7390,12 +7390,12 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -7441,12 +7441,12 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
@@ -7492,12 +7492,12 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -7543,12 +7543,12 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -7594,12 +7594,12 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -7645,17 +7645,17 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
@@ -7668,7 +7668,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H73" s="11" t="inlineStr"/>
+      <c r="H73" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7692,22 +7696,22 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
@@ -7715,7 +7719,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H74" s="11" t="inlineStr"/>
+      <c r="H74" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7739,17 +7747,17 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
@@ -7762,7 +7770,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H75" s="11" t="inlineStr"/>
+      <c r="H75" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7786,12 +7798,12 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -7810,9 +7822,9 @@
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
-      <c r="I76" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr"/>
@@ -7833,12 +7845,12 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -7848,7 +7860,7 @@
       </c>
       <c r="F77" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G77" s="11" t="inlineStr">
@@ -7880,12 +7892,12 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -7927,12 +7939,12 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
@@ -7951,9 +7963,9 @@
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr"/>
-      <c r="I79" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
@@ -7969,42 +7981,38 @@
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H80" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED (revised): build it to avoid a removal letter.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H80" s="11" t="inlineStr"/>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr"/>
@@ -8020,48 +8028,44 @@
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H81" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H81" s="11" t="inlineStr"/>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr"/>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8071,48 +8075,44 @@
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G82" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H82" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H82" s="11" t="inlineStr"/>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr"/>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8127,22 +8127,22 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G83" s="11" t="inlineStr">
@@ -8152,18 +8152,18 @@
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
         </is>
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr"/>
       <c r="K83" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8173,27 +8173,27 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
@@ -8201,16 +8201,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H84" s="11" t="inlineStr"/>
+      <c r="H84" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
+        </is>
+      </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8225,12 +8229,12 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
@@ -8240,7 +8244,7 @@
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
@@ -8250,18 +8254,18 @@
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr"/>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8280,17 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
@@ -8301,18 +8305,18 @@
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
       <c r="K86" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8322,22 +8326,22 @@
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F87" s="11" t="inlineStr">
@@ -8350,11 +8354,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H87" s="11" t="inlineStr">
-        <is>
-          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
-        </is>
-      </c>
+      <c r="H87" s="11" t="inlineStr"/>
       <c r="I87" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8363,7 +8363,7 @@
       <c r="J87" s="11" t="inlineStr"/>
       <c r="K87" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8378,17 +8378,17 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
@@ -8429,17 +8429,17 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877. From the first review.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I89" s="11" t="inlineStr">
@@ -8480,17 +8480,17 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
@@ -8505,7 +8505,7 @@
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
@@ -8531,12 +8531,12 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I91" s="11" t="inlineStr">
@@ -8582,17 +8582,17 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F92" s="11" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I92" s="11" t="inlineStr">
@@ -8633,17 +8633,17 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
@@ -8684,12 +8684,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
@@ -8735,17 +8735,17 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F95" s="11" t="inlineStr">
@@ -8760,7 +8760,7 @@
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I95" s="11" t="inlineStr">
@@ -8786,12 +8786,12 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 082ec92.</t>
         </is>
       </c>
       <c r="I96" s="11" t="inlineStr">
@@ -8837,17 +8837,17 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F97" s="11" t="inlineStr">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
@@ -8888,12 +8888,12 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3. From the first review.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I98" s="11" t="inlineStr">
@@ -8939,17 +8939,17 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F99" s="11" t="inlineStr">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
@@ -8990,17 +8990,17 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
@@ -9041,17 +9041,17 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>REQ031</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F101" s="11" t="inlineStr">
@@ -9066,7 +9066,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
@@ -9092,17 +9092,17 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
@@ -9117,7 +9117,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>DONE Dashboard: stock in vs stock out per day/week/month/year. Keeps the Chart.js claim (no letter).</t>
+          <t>DONE d9fc96b. From the first review.</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -9143,12 +9143,12 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Modules p.42</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
@@ -9194,17 +9194,17 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework p.23</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr">
@@ -9245,12 +9245,12 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="H105" s="11" t="inlineStr">
         <is>
-          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
+          <t>DONE Dashboard: stock in vs stock out per day/week/month/year. Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I105" s="11" t="inlineStr">
@@ -9296,17 +9296,17 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F106" s="11" t="inlineStr">
@@ -9319,7 +9319,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H106" s="11" t="inlineStr"/>
+      <c r="H106" s="11" t="inlineStr">
+        <is>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+        </is>
+      </c>
       <c r="I106" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9328,7 +9332,7 @@
       <c r="J106" s="11" t="inlineStr"/>
       <c r="K106" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9338,22 +9342,22 @@
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F107" s="11" t="inlineStr">
@@ -9366,16 +9370,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H107" s="11" t="inlineStr"/>
+      <c r="H107" s="11" t="inlineStr">
+        <is>
+          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+        </is>
+      </c>
       <c r="I107" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J107" s="11" t="inlineStr"/>
       <c r="K107" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9385,22 +9393,22 @@
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
@@ -9415,18 +9423,18 @@
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
         </is>
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J108" s="11" t="inlineStr"/>
       <c r="K108" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9436,22 +9444,22 @@
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>REQ004</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F109" s="11" t="inlineStr">
@@ -9466,12 +9474,12 @@
       </c>
       <c r="H109" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I109" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
+        </is>
+      </c>
+      <c r="I109" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J109" s="11" t="inlineStr"/>
@@ -9487,22 +9495,22 @@
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F110" s="11" t="inlineStr">
@@ -9515,14 +9523,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H110" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H110" s="11" t="inlineStr"/>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr"/>
@@ -9538,22 +9542,22 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F111" s="11" t="inlineStr">
@@ -9566,14 +9570,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H111" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H111" s="11" t="inlineStr"/>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J111" s="11" t="inlineStr"/>
@@ -9594,22 +9594,22 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G112" s="11" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
@@ -9645,17 +9645,17 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F113" s="11" t="inlineStr">
@@ -9668,7 +9668,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H113" s="11" t="inlineStr"/>
+      <c r="H113" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -9692,17 +9696,17 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F114" s="11" t="inlineStr">
@@ -9715,7 +9719,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H114" s="11" t="inlineStr"/>
+      <c r="H114" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I114" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -9739,17 +9747,17 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F115" s="11" t="inlineStr">
@@ -9764,18 +9772,18 @@
       </c>
       <c r="H115" s="11" t="inlineStr">
         <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
-      <c r="I115" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I115" s="11" t="inlineStr">
+        <is>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J115" s="11" t="inlineStr"/>
       <c r="K115" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9790,17 +9798,17 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F116" s="11" t="inlineStr">
@@ -9813,10 +9821,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H116" s="11" t="inlineStr"/>
+      <c r="H116" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J116" s="11" t="inlineStr"/>
@@ -9837,17 +9849,17 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F117" s="11" t="inlineStr">
@@ -9860,7 +9872,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H117" s="11" t="inlineStr"/>
+      <c r="H117" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I117" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -9884,12 +9900,12 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
@@ -9908,9 +9924,9 @@
         </is>
       </c>
       <c r="H118" s="11" t="inlineStr"/>
-      <c r="I118" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I118" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J118" s="11" t="inlineStr"/>
@@ -9931,12 +9947,12 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -9954,11 +9970,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H119" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
-        </is>
-      </c>
+      <c r="H119" s="11" t="inlineStr"/>
       <c r="I119" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -9967,7 +9979,7 @@
       <c r="J119" s="11" t="inlineStr"/>
       <c r="K119" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9982,12 +9994,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
@@ -10005,7 +10017,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H120" s="11" t="inlineStr"/>
+      <c r="H120" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
       <c r="I120" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10014,7 +10030,7 @@
       <c r="J120" s="11" t="inlineStr"/>
       <c r="K120" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10029,12 +10045,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -10055,7 +10071,7 @@
       <c r="H121" s="11" t="inlineStr"/>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J121" s="11" t="inlineStr"/>
@@ -10076,12 +10092,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -10123,12 +10139,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -10146,11 +10162,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H123" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
+      <c r="H123" s="11" t="inlineStr"/>
       <c r="I123" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10159,7 +10171,7 @@
       <c r="J123" s="11" t="inlineStr"/>
       <c r="K123" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10174,12 +10186,12 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
@@ -10197,16 +10209,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H124" s="11" t="inlineStr"/>
-      <c r="I124" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H124" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
+        </is>
+      </c>
+      <c r="I124" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J124" s="11" t="inlineStr"/>
       <c r="K124" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10221,12 +10237,12 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
@@ -10245,9 +10261,9 @@
         </is>
       </c>
       <c r="H125" s="11" t="inlineStr"/>
-      <c r="I125" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I125" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J125" s="11" t="inlineStr"/>
@@ -10268,12 +10284,12 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -10294,7 +10310,7 @@
       <c r="H126" s="11" t="inlineStr"/>
       <c r="I126" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J126" s="11" t="inlineStr"/>
@@ -10315,12 +10331,12 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -10362,12 +10378,12 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -10385,16 +10401,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H128" s="11" t="inlineStr"/>
-      <c r="I128" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H128" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I128" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J128" s="11" t="inlineStr"/>
       <c r="K128" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10409,12 +10429,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10456,12 +10476,12 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10503,12 +10523,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10550,12 +10570,12 @@
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -10586,18 +10606,253 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="11" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C133" s="11" t="inlineStr">
+        <is>
+          <t>References (p.100)</t>
+        </is>
+      </c>
+      <c r="D133" s="11" t="inlineStr">
+        <is>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+        </is>
+      </c>
+      <c r="E133" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F133" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G133" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H133" s="11" t="inlineStr"/>
+      <c r="I133" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J133" s="11" t="inlineStr"/>
+      <c r="K133" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C134" s="11" t="inlineStr">
+        <is>
+          <t>References (p.10 / refs)</t>
+        </is>
+      </c>
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+        </is>
+      </c>
+      <c r="E134" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F134" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G134" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H134" s="11" t="inlineStr"/>
+      <c r="I134" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J134" s="11" t="inlineStr"/>
+      <c r="K134" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C135" s="11" t="inlineStr">
+        <is>
+          <t>References (p.17 / refs)</t>
+        </is>
+      </c>
+      <c r="D135" s="11" t="inlineStr">
+        <is>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+        </is>
+      </c>
+      <c r="E135" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F135" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G135" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H135" s="11" t="inlineStr"/>
+      <c r="I135" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J135" s="11" t="inlineStr"/>
+      <c r="K135" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>Appendices (p.124)</t>
+        </is>
+      </c>
+      <c r="D136" s="11" t="inlineStr">
+        <is>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+        </is>
+      </c>
+      <c r="E136" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G136" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H136" s="11" t="inlineStr"/>
+      <c r="I136" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J136" s="11" t="inlineStr"/>
+      <c r="K136" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G137" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H137" s="11" t="inlineStr"/>
+      <c r="I137" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J137" s="11" t="inlineStr"/>
+      <c r="K137" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K132"/>
-  <conditionalFormatting sqref="K2:K132">
+  <autoFilter ref="A1:K137"/>
+  <conditionalFormatting sqref="K2:K137">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register and README: system-wide bug check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$143</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4808,22 +4808,22 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>REQ083, REQ122, Fig 2.6, Fig 2.14, C4</t>
+          <t>REQ095-100, REQ098</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Walk-in void: reason, original receipt no., automatic stock restore, optional exchange item + price difference, audit entry; restricted to authorized role</t>
+          <t>Bug check: store credit could be lost or added twice on expired holds; credit redeemed on an order was lost on invalid-payment holds; two staff approving at once deducted stock twice</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -4838,18 +4838,18 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: BM/Technical void completed sales from POS Today's Sales or Walk-in Orders: reason, SI No., stock restored to the same batches, exchange note + price difference, audit entry. Still open: second-person approval (client rule) and exchange as a real stock movement. Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
+          <t>DONE f0faaad.</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4859,27 +4859,27 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>REQ098, REQ102, C2</t>
+          <t>REQNF011, REQ002, REQ098</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Fix overpayment approval: clear the old hold, send 'Payment confirmed' notification; reword REQ098</t>
+          <t>Bug check: database rules let a customer create orders with any status/hold, start with store credit, rewrite a hold when resubmitting, or reset the order counter; deactivated staff kept access</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -4889,18 +4889,18 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b (system part; REQ098 paper wording still to do). From the first review.</t>
+          <t>DONE 5d41982 (publish firestore.rules).</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4910,22 +4910,22 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>REQ071, REQ073, REQ120, REQNF011, C8</t>
+          <t>REQNF011</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Price lock: only Branch Manager sets prices on create/import too; enforce in database rules; add a reason to each price change</t>
+          <t>Bug check: customer- and staff-typed text (names, order numbers, notes) was put into admin pages as HTML</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -4940,18 +4940,18 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>DONE BM-only prices in the form, batch import and quick-add (others' products saved Inactive + 'Price pending'); reason required and logged; enforced in firestore.rules - PUBLISH THE RULES in the Firebase console.</t>
+          <t>DONE 72e7361.</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4961,27 +4961,27 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Removals (Letter) sheet</t>
+          <t>REQ083, REQ122, Fig 2.6, Fig 2.14, C4</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Letter to the panel: OpenAI -&gt; Gemini (free), Firebase Storage -&gt; Cloudinary, DataTable -&gt; custom tables, password reset via Firebase Auth, overpayment approve-and-credit, corrections to scope/conceptual framework</t>
+          <t>Walk-in void: reason, original receipt no., automatic stock restore, optional exchange item + price difference, audit entry; restricted to authorized role</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -4991,18 +4991,18 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>One letter covers all remaining removals; send before the paper edits.</t>
-        </is>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE 57f4d80: BM/Technical void completed sales from POS Today's Sales or Walk-in Orders: reason, SI No., stock restored to the same batches, exchange note + price difference, audit entry. Still open: second-person approval (client rule) and exchange as a real stock movement. Client's #1 pain point (Interview 4). Client rules: a void needs a second authorized person, not one junior staff member alone; exchange item must be equal or higher value (customer pays the difference, never refunded); restored stock must show online too.</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5012,27 +5012,27 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Objectives / evaluation (p.5-6, 21-24)</t>
+          <t>REQ098, REQ102, C2</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
+          <t>Fix overpayment approval: clear the old hold, send 'Payment confirmed' notification; reword REQ098</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -5040,7 +5040,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>DONE e1e200b (system part; REQ098 paper wording still to do). From the first review.</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -5049,7 +5053,7 @@
       <c r="J21" s="11" t="inlineStr"/>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5059,22 +5063,22 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>REQ121</t>
+          <t>REQ071, REQ073, REQ120, REQNF011, C8</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
+          <t>Price lock: only Branch Manager sets prices on create/import too; enforce in database rules; add a reason to each price change</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -5084,17 +5088,17 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: POS (with Today's Sales) + read-only catalog; lands on POS after login. Orders access was added on purpose on 2026-10-01.</t>
+          <t>DONE BM-only prices in the form, batch import and quick-add (others' products saved Inactive + 'Price pending'); reason required and logged; enforced in firestore.rules - PUBLISH THE RULES in the Firebase console.</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr"/>
@@ -5110,37 +5114,37 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>REQNF005</t>
+          <t>Removals (Letter) sheet</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Live updates without refresh on all order and inventory screens (staff + customer)</t>
+          <t>Letter to the panel: OpenAI -&gt; Gemini (free), Firebase Storage -&gt; Cloudinary, DataTable -&gt; custom tables, password reset via Firebase Auth, overpayment approve-and-credit, corrections to scope/conceptual framework</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>DONE 21e505b: orders (staff + customer), inventory, POS today's sales, chat.</t>
+          <t>One letter covers all remaining removals; send before the paper edits.</t>
         </is>
       </c>
       <c r="I23" s="12" t="inlineStr">
@@ -5151,7 +5155,7 @@
       <c r="J23" s="11" t="inlineStr"/>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5161,42 +5165,38 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>REQNF010, REQNF013</t>
+          <t>Objectives / evaluation (p.5-6, 21-24)</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
+          <t>Obj. 4 evaluates with TAM + ISO/IEC 25010, but there is no questionnaire, respondent group, sampling, scale, or statistical treatment yet. The final paper needs the instrument and a results chapter.</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Med</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: Netlify (already set up).</t>
-        </is>
-      </c>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr"/>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr"/>
@@ -5212,27 +5212,27 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
+          <t>REQ121</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Discount / deduction per sale or line, with reason and audit entry</t>
+          <t>Sales Staff access: trim to POS + catalog view, or reword REQ121</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -5242,18 +5242,18 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
+          <t>DONE 57f4d80: POS (with Today's Sales) + read-only catalog; lands on POS after login. Orders access was added on purpose on 2026-10-01.</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr"/>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5263,22 +5263,22 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
+          <t>REQNF005</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
+          <t>Live updates without refresh on all order and inventory screens (staff + customer)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -5293,18 +5293,18 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>DONE 21e505b: orders (staff + customer), inventory, POS today's sales, chat.</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5314,22 +5314,22 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Limitations (p.7)</t>
+          <t>REQNF010, REQNF013</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
+          <t>Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -5342,7 +5342,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr"/>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: Netlify (already set up).</t>
+        </is>
+      </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5361,27 +5365,27 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Limitations (p.7)</t>
+          <t>Report Formats sheet (Discount/Deductions columns); Interview 2</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
+          <t>Discount / deduction per sale or line, with reason and audit entry</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -5389,16 +5393,20 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr"/>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>Client confirmed: no discounts. Not in the paper; client gives boss-approved discounts today.</t>
+        </is>
+      </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr"/>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -5408,27 +5416,27 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Methodology p.30 ('actual client data'); Report Formats sheet</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
+          <t>Load the client's real March-end catalog (prices, batches, expiry) from their workbook via the existing upload templates</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -5436,7 +5444,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr"/>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: yes, once the client sends the catalog. Makes the demo and the TAM evaluation realistic; check confidentiality with the client first.</t>
+        </is>
+      </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5445,7 +5457,7 @@
       <c r="J29" s="11" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -5455,22 +5467,22 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Limitations (p.7)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
+          <t>'Retail item exchanges ... coordinated through live chat': if chat is cut, change this to phone/Messenger.</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -5483,11 +5495,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
-        <is>
-          <t>DONE d9fc96b: locks itself after one run; SI counter now staff-only in rules (publish rules). From the first review.</t>
-        </is>
-      </c>
+      <c r="H30" s="11" t="inlineStr"/>
       <c r="I30" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5496,7 +5504,7 @@
       <c r="J30" s="11" t="inlineStr"/>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5506,22 +5514,22 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>REQ002</t>
+          <t>Limitations (p.7)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
+          <t>Add new limitations if decided: hosting/deployment, live chat/AI, real-time refresh, OpenAI cost.</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -5534,11 +5542,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>From the first review.</t>
-        </is>
-      </c>
+      <c r="H31" s="11" t="inlineStr"/>
       <c r="I31" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5557,27 +5561,27 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Unrecognized-device OTP for customers and staff</t>
+          <t>Netlify listed for hosting with continuous integration; nothing is deployed (Netlify blocked by billing). Depends on the hosting decision.</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -5585,11 +5589,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>DONE 7ede9d4: emailed code on new browsers, customers and staff; recognized devices in Account Settings.</t>
-        </is>
-      </c>
+      <c r="H32" s="11" t="inlineStr"/>
       <c r="I32" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5598,7 +5598,7 @@
       <c r="J32" s="11" t="inlineStr"/>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5613,22 +5613,22 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>REQ086, REQ089, REQ091, REQ092</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
+          <t>Remove or lock the Migrate Credit page (re-running it re-grants spent credit)</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>DONE 5cad255: history, sales invoice PDF, free-of-cost, LTO/permit validity. Not built: reorder from a past order. Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
+          <t>DONE d9fc96b: locks itself after one run; SI counter now staff-only in rules (publish rules). From the first review.</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
@@ -5664,22 +5664,22 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>REQ090, REQ114, Fig 2.15</t>
+          <t>REQ002</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
+          <t>Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>DONE Purchase History -&gt; Exchange: return to batch, FEFO replacement, value rule, audit, exchange document; Return / Exchange report.</t>
+          <t>From the first review.</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -5700,7 +5700,7 @@
       <c r="J34" s="11" t="inlineStr"/>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5715,12 +5715,12 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>REQ067, C7</t>
+          <t>REQ005, REQ044, Fig 2.3, Fig 2.8</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
+          <t>Unrecognized-device OTP for customers and staff</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>DONE d2a957b: automatic write-off with reason, audit entry, disposal alert, Mark disposed.</t>
+          <t>DONE 7ede9d4: emailed code on new browsers, customers and staff; recognized devices in Account Settings.</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -5766,22 +5766,22 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
+          <t>REQ086, REQ089, REQ091, REQ092</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
+          <t>Wholesale: purchase history per account (with reorder from a past order), wholesale sales invoice, free-of-cost option with reason, document expiry dates</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout. The 'not an official receipt' line was removed from POS and online receipts on 2026-10-21 at the team's request.</t>
+          <t>DONE 5cad255: history, sales invoice PDF, free-of-cost, LTO/permit validity. Not built: reorder from a past order. Interview 1: free RX goods go only to medical doctors/hospitals; vitamins open to all. Interview 2: reorder what they bought weeks ago.</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
@@ -5817,12 +5817,12 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>REQ084</t>
+          <t>REQ090, REQ114, Fig 2.15</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>POS: RX Verified checkbox + optional notes</t>
+          <t>Wholesale exchange workflow (return + FEFO replacement + audit + exchange document)</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: checkbox + notes, required for RX items, saved on the sale.</t>
+          <t>DONE Purchase History -&gt; Exchange: return to batch, FEFO replacement, value rule, audit, exchange document; Return / Exchange report.</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
@@ -5868,22 +5868,22 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>REQ061, C5</t>
+          <t>REQ067, C7</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
+          <t>2-month Bad Order: auto-flag, disposal alert, auto-deduct with write-off record</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: others save counts; BM finalizes; variance reason required and logged.</t>
+          <t>DONE d2a957b: automatic write-off with reason, audit entry, disposal alert, Mark disposed.</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -5919,17 +5919,17 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>REQNF025, REQNF029</t>
+          <t>Fig 2.6 Print Transaction Receipt, Modules p.44</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
+          <t>Receipt printing (thermal 58mm print layout) for POS sales</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>DONE footer rebuilt from js/store-info.js (real About text, links to legal.html; contact/LTO lines hidden until the client confirms them); chat links hidden until chat is built; payment page Terms link fixed. From the first review.</t>
+          <t>DONE 57f4d80: Print button on every POS receipt; 58mm print layout. The 'not an official receipt' line was removed from POS and online receipts on 2026-10-21 at the team's request.</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -5970,22 +5970,22 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>REQ039, REQ042</t>
+          <t>REQ084</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
+          <t>POS: RX Verified checkbox + optional notes</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>DONE EmailJS order template (ID to paste in js/emailjs-config.js) + on/off toggle in Account Settings. EmailJS free tier: 200/month.</t>
+          <t>DONE 57f4d80: checkbox + notes, required for RX items, saved on the sale.</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
@@ -6021,12 +6021,12 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>REQ122</t>
+          <t>REQ061, C5</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
+          <t>Reconciliation: Branch Manager-only finalize + variance reason in audit log</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -6044,7 +6044,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr"/>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>DONE 06574da: others save counts; BM finalizes; variance reason required and logged.</t>
+        </is>
+      </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6053,7 +6057,7 @@
       <c r="J41" s="11" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6068,17 +6072,17 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>REQ014</t>
+          <t>REQNF025, REQNF029</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Save cart to the customer's account</t>
+          <t>Remove dead links and filler: Live Chat sidebar link, chat buttons, footer sample text, footer Privacy/Terms links</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
@@ -6093,7 +6097,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE footer rebuilt from js/store-info.js (real About text, links to legal.html; contact/LTO lines hidden until the client confirms them); chat links hidden until chat is built; payment page Terms link fixed. From the first review.</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -6119,22 +6123,22 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>REQNF003, REQNF007</t>
+          <t>REQ039, REQ042</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Phone/tablet and cross-browser test pass</t>
+          <t>Email notifications for key order events + on/off toggle in Account Settings</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>Not verified</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
@@ -6142,7 +6146,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr"/>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>DONE EmailJS order template (ID to paste in js/emailjs-config.js) + on/off toggle in Account Settings. EmailJS free tier: 200/month.</t>
+        </is>
+      </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6151,7 +6159,7 @@
       <c r="J43" s="11" t="inlineStr"/>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6166,22 +6174,22 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Interviews 2, 4</t>
+          <t>REQ122</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
+          <t>Audit log completeness: structured before/after, reasons, more events (receiving, PO, product create/delete, RX verification)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr">
@@ -6189,11 +6197,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H44" s="11" t="inlineStr">
-        <is>
-          <t>DONE e1e200b. Required column in the monthly purchases report.</t>
-        </is>
-      </c>
+      <c r="H44" s="11" t="inlineStr"/>
       <c r="I44" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6202,7 +6206,7 @@
       <c r="J44" s="11" t="inlineStr"/>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6217,17 +6221,17 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Interview 4 walkthrough</t>
+          <t>REQ014</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Supplier history: everything received from each supplier</t>
+          <t>Save cart to the customer's account</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
@@ -6242,7 +6246,7 @@
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>DONE Reports -&gt; Supplier Purchases (per supplier, per month). Shown to the client during the prototype walkthrough.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
@@ -6268,22 +6272,22 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Methodology p.30; Interview 4</t>
+          <t>REQNF003, REQNF007</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>User manual + hands-on training + handover to the branch</t>
+          <t>Phone/tablet and cross-browser test pass</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Not verified</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G46" s="11" t="inlineStr">
@@ -6291,11 +6295,7 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
-        </is>
-      </c>
+      <c r="H46" s="11" t="inlineStr"/>
       <c r="I46" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -6319,12 +6319,12 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
+          <t>Interviews 2, 4</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
+          <t>Supplier receipt / DR number field on Receive Stock and PO receiving</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b. Customer File groups every sale by customer name.</t>
+          <t>DONE e1e200b. Required column in the monthly purchases report.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
@@ -6370,17 +6370,17 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (Supplier sheets)</t>
+          <t>Interview 4 walkthrough</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
+          <t>Supplier history: everything received from each supplier</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b: unit cost + receipt/DR no. added; pack size stays in the product name as the branch does today. Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
+          <t>DONE Reports -&gt; Supplier Purchases (per supplier, per month). Shown to the client during the prototype walkthrough.</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
@@ -6421,22 +6421,22 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
+          <t>Methodology p.30; Interview 4</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
+          <t>User manual + hands-on training + handover to the branch</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Deviates</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>DONE e1e200b: also storefront links/filters now follow Manage Categories. Existing Firebase projects keep their current categories - add the client's in Manage Categories.. Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
+          <t>Client: 'kailangan pa namin gamayin, i-hands on pa namin to'.</t>
         </is>
       </c>
       <c r="I49" s="11" t="inlineStr">
@@ -6457,7 +6457,7 @@
       <c r="J49" s="11" t="inlineStr"/>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6472,22 +6472,22 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087</t>
+          <t>Report Formats sheet (Customer File shows named walk-ins, e.g. EMPLOYEE)</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Optional agreed price per wholesale buyer per product, used as default on their orders</t>
+          <t>Optional customer name on walk-in sales (default 'Walk-in')</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr">
@@ -6497,12 +6497,12 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>DONE saved from Process Order, listed in Edit account, default on orders. Keeps per-account pricing (no letter).</t>
-        </is>
-      </c>
-      <c r="I50" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE e1e200b. Customer File groups every sale by customer name.</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr"/>
@@ -6523,12 +6523,12 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Production readiness</t>
+          <t>Report Formats sheet (Supplier sheets)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Cut database reads: stop loading whole collections on every page (Firestore free-plan daily read cap ~50k)</t>
+          <t>Unit cost, supplier receipt no., brand and pack on each stock receiving entry</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Needed before real use with the client's ~1,000-product catalog.</t>
+          <t>DONE e1e200b: unit cost + receipt/DR no. added; pack size stays in the product name as the branch does today. Monthly purchases report needs cost per delivery, not just the product's current costing.</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
@@ -6559,7 +6559,7 @@
       <c r="J51" s="11" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6574,17 +6574,17 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module p.40; Interview 4 (dashboard export)</t>
+          <t>Report Formats sheet (monthly sheets); js/products-data.js:401</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Dashboard Sales Analytics: show which dates the Today/Week/Month/Year view covers, and add a picker to choose a specific day, week, month or year (with previous/next)</t>
+          <t>Match the client's categories: Generics, Branded, Drugstore (per piece), Medical Supplies, Grocery</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Deviates</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
@@ -6599,7 +6599,7 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>DONE cb08e78: date range shown; Day/Week/Month/Year with previous/next and a date picker; exports name the period. Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
+          <t>DONE e1e200b: also storefront links/filters now follow Manage Categories. Existing Firebase projects keep their current categories - add the client's in Manage Categories.. Default categories are OTC/Vitamins/Personal Care/Health &amp; Wellness; the monthly report is one sheet per client category.</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
@@ -6625,22 +6625,22 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>REQ048, Notification module</t>
+          <t>REQ085, REQ087</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Admin notification for pending wholesale orders (Pending -&gt; Released)</t>
+          <t>Optional agreed price per wholesale buyer per product, used as default on their orders</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G53" s="11" t="inlineStr">
@@ -6650,18 +6650,18 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>DONE 274b8e0: wholesale orders start Pending; Mark Released in purchase history; staff notification.</t>
-        </is>
-      </c>
-      <c r="I53" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>DONE saved from Process Order, listed in Edit account, default on orders. Keeps per-account pricing (no letter).</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6676,22 +6676,22 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>REQ111, Sales Report module</t>
+          <t>Production readiness</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Daily Sales report: batch, expiry, date received and supplier per item sold</t>
+          <t>Cut database reads: stop loading whole collections on every page (Firestore free-plan daily read cap ~50k)</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G54" s="11" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>DONE 274b8e0: 'Item Sold by Batch' section.</t>
+          <t>Needed before real use with the client's ~1,000-product catalog.</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
@@ -6727,17 +6727,17 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>Dashboard module p.40; Interview 4 (dashboard export)</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>Dashboard Sales Analytics: show which dates the Today/Week/Month/Year view covers, and add a picker to choose a specific day, week, month or year (with previous/next)</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
+          <t>DONE cb08e78: date range shown; Day/Week/Month/Year with previous/next and a date picker; exports name the period. Requested by the team 2026-10-21. Chart, totals and the export should all follow the picked period, and the export title should name it.</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
@@ -6778,17 +6778,17 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>REQ048, Notification module</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Admin notification for pending wholesale orders (Pending -&gt; Released)</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+          <t>DONE 274b8e0: wholesale orders start Pending; Mark Released in purchase history; staff notification.</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
@@ -6814,7 +6814,7 @@
       <c r="J56" s="11" t="inlineStr"/>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6829,17 +6829,17 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>REQ111, Sales Report module</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>Daily Sales report: batch, expiry, date received and supplier per item sold</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>DONE footer links to legal.html on every page.</t>
+          <t>DONE 274b8e0: 'Item Sold by Batch' section.</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
@@ -6865,7 +6865,7 @@
       <c r="J57" s="11" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6875,27 +6875,27 @@
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Various</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>Bug check: checkout, reports, inventory and wholesale fixes (RX orders always pick-up, price/availability re-check, exchanges in sales reports, write-off date, stock count variance, receiving saved all at once, invoice peso sign)</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G58" s="11" t="inlineStr">
@@ -6905,18 +6905,18 @@
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+          <t>DONE d51639d, 0e7826e.</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr"/>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -6926,22 +6926,22 @@
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F59" s="11" t="inlineStr">
@@ -6956,18 +6956,18 @@
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
         </is>
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr"/>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6977,22 +6977,22 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F60" s="11" t="inlineStr">
@@ -7007,18 +7007,18 @@
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I60" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr"/>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7028,22 +7028,22 @@
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F61" s="11" t="inlineStr">
@@ -7058,18 +7058,18 @@
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I61" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>DONE footer links to legal.html on every page.</t>
+        </is>
+      </c>
+      <c r="I61" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr"/>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7079,22 +7079,22 @@
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F62" s="11" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
@@ -7120,7 +7120,7 @@
       <c r="J62" s="11" t="inlineStr"/>
       <c r="K62" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7135,12 +7135,12 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
@@ -7186,12 +7186,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -7237,12 +7237,12 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
@@ -7288,12 +7288,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -7339,12 +7339,12 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
@@ -7390,12 +7390,12 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -7418,9 +7418,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I68" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I68" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr"/>
@@ -7441,12 +7441,12 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
@@ -7469,9 +7469,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I69" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr"/>
@@ -7492,12 +7492,12 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -7543,12 +7543,12 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -7594,12 +7594,12 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -7645,12 +7645,12 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
@@ -7696,12 +7696,12 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -7747,12 +7747,12 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
@@ -7798,17 +7798,17 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
@@ -7821,7 +7821,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H76" s="11" t="inlineStr"/>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7845,22 +7849,22 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F77" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G77" s="11" t="inlineStr">
@@ -7868,7 +7872,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H77" s="11" t="inlineStr"/>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7892,17 +7900,17 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
@@ -7915,7 +7923,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H78" s="11" t="inlineStr"/>
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -7939,17 +7951,17 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
@@ -7962,10 +7974,14 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H79" s="11" t="inlineStr"/>
-      <c r="I79" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
@@ -7986,12 +8002,12 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
@@ -8033,12 +8049,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
@@ -8048,7 +8064,7 @@
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
@@ -8080,12 +8096,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -8122,42 +8138,38 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G83" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H83" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED (revised): build it to avoid a removal letter.</t>
-        </is>
-      </c>
-      <c r="I83" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H83" s="11" t="inlineStr"/>
+      <c r="I83" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr"/>
@@ -8173,48 +8185,44 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H84" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H84" s="11" t="inlineStr"/>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8224,48 +8232,44 @@
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H85" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H85" s="11" t="inlineStr"/>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr"/>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8275,22 +8279,22 @@
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
@@ -8300,23 +8304,19 @@
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H86" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H86" s="11" t="inlineStr"/>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
       <c r="K86" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8326,27 +8326,27 @@
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G87" s="11" t="inlineStr">
@@ -8354,7 +8354,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H87" s="11" t="inlineStr"/>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
+        </is>
+      </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8378,12 +8382,12 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
@@ -8393,7 +8397,7 @@
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G88" s="11" t="inlineStr">
@@ -8403,18 +8407,18 @@
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
       <c r="K88" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8429,22 +8433,22 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G89" s="11" t="inlineStr">
@@ -8454,18 +8458,18 @@
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J89" s="11" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8480,17 +8484,17 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
@@ -8505,18 +8509,18 @@
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr"/>
       <c r="K90" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -8526,22 +8530,22 @@
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F91" s="11" t="inlineStr">
@@ -8554,11 +8558,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H91" s="11" t="inlineStr">
-        <is>
-          <t>DONE 847c877.</t>
-        </is>
-      </c>
+      <c r="H91" s="11" t="inlineStr"/>
       <c r="I91" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -8567,7 +8567,7 @@
       <c r="J91" s="11" t="inlineStr"/>
       <c r="K91" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8582,17 +8582,17 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F92" s="11" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877. From the first review.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I92" s="11" t="inlineStr">
@@ -8633,17 +8633,17 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
@@ -8684,12 +8684,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92. From the first review.</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
@@ -8735,12 +8735,12 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
@@ -8786,17 +8786,17 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I96" s="11" t="inlineStr">
@@ -8837,17 +8837,17 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F97" s="11" t="inlineStr">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
@@ -8888,17 +8888,17 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I98" s="11" t="inlineStr">
@@ -8939,12 +8939,12 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
@@ -8990,17 +8990,17 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
+          <t>DONE 082ec92.</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
@@ -9041,17 +9041,17 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F101" s="11" t="inlineStr">
@@ -9066,7 +9066,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3. From the first review.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
@@ -9092,17 +9092,17 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
@@ -9117,7 +9117,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b. From the first review.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -9143,17 +9143,17 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F103" s="11" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
@@ -9194,17 +9194,17 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>REQ031</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr">
@@ -9245,12 +9245,12 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="H105" s="11" t="inlineStr">
         <is>
-          <t>DONE Dashboard: stock in vs stock out per day/week/month/year. Keeps the Chart.js claim (no letter).</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I105" s="11" t="inlineStr">
@@ -9296,17 +9296,17 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Modules p.42</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F106" s="11" t="inlineStr">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+          <t>DONE d9fc96b. From the first review.</t>
         </is>
       </c>
       <c r="I106" s="11" t="inlineStr">
@@ -9347,12 +9347,12 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework p.23</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="H107" s="11" t="inlineStr">
         <is>
-          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
         </is>
       </c>
       <c r="I107" s="11" t="inlineStr">
@@ -9398,17 +9398,17 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I108" s="11" t="inlineStr">
@@ -9449,17 +9449,17 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>REQ004</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F109" s="11" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="H109" s="11" t="inlineStr">
         <is>
-          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
+          <t>DONE Dashboard: stock in vs stock out per day/week/month/year. Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I109" s="11" t="inlineStr">
@@ -9485,7 +9485,7 @@
       <c r="J109" s="11" t="inlineStr"/>
       <c r="K109" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9500,17 +9500,17 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F110" s="11" t="inlineStr">
@@ -9523,7 +9523,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H110" s="11" t="inlineStr"/>
+      <c r="H110" s="11" t="inlineStr">
+        <is>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+        </is>
+      </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9532,7 +9536,7 @@
       <c r="J110" s="11" t="inlineStr"/>
       <c r="K110" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9542,22 +9546,22 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F111" s="11" t="inlineStr">
@@ -9570,16 +9574,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H111" s="11" t="inlineStr"/>
+      <c r="H111" s="11" t="inlineStr">
+        <is>
+          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+        </is>
+      </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J111" s="11" t="inlineStr"/>
       <c r="K111" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9589,27 +9597,27 @@
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G112" s="11" t="inlineStr">
@@ -9619,18 +9627,18 @@
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
+          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J112" s="11" t="inlineStr"/>
       <c r="K112" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9640,22 +9648,22 @@
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>REQ004</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F113" s="11" t="inlineStr">
@@ -9670,12 +9678,12 @@
       </c>
       <c r="H113" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
         </is>
       </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J113" s="11" t="inlineStr"/>
@@ -9691,22 +9699,22 @@
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F114" s="11" t="inlineStr">
@@ -9719,14 +9727,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H114" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I114" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H114" s="11" t="inlineStr"/>
+      <c r="I114" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J114" s="11" t="inlineStr"/>
@@ -9742,22 +9746,22 @@
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F115" s="11" t="inlineStr">
@@ -9770,14 +9774,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H115" s="11" t="inlineStr">
-        <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
+      <c r="H115" s="11" t="inlineStr"/>
       <c r="I115" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J115" s="11" t="inlineStr"/>
@@ -9798,22 +9798,22 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F116" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G116" s="11" t="inlineStr">
@@ -9823,12 +9823,12 @@
       </c>
       <c r="H116" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J116" s="11" t="inlineStr"/>
@@ -9849,17 +9849,17 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F117" s="11" t="inlineStr">
@@ -9874,7 +9874,7 @@
       </c>
       <c r="H117" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>Rare; same-second exchanges on one line.</t>
         </is>
       </c>
       <c r="I117" s="11" t="inlineStr">
@@ -9900,17 +9900,17 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>REQ125</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F118" s="11" t="inlineStr">
@@ -9923,7 +9923,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H118" s="11" t="inlineStr"/>
+      <c r="H118" s="11" t="inlineStr">
+        <is>
+          <t>Needs a server function to clean up; note in the user manual.</t>
+        </is>
+      </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -9947,17 +9951,17 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F119" s="11" t="inlineStr">
@@ -9970,10 +9974,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H119" s="11" t="inlineStr"/>
-      <c r="I119" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H119" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I119" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J119" s="11" t="inlineStr"/>
@@ -9994,17 +10002,17 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F120" s="11" t="inlineStr">
@@ -10019,7 +10027,7 @@
       </c>
       <c r="H120" s="11" t="inlineStr">
         <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I120" s="12" t="inlineStr">
@@ -10030,7 +10038,7 @@
       <c r="J120" s="11" t="inlineStr"/>
       <c r="K120" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10045,17 +10053,17 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F121" s="11" t="inlineStr">
@@ -10068,10 +10076,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H121" s="11" t="inlineStr"/>
+      <c r="H121" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J121" s="11" t="inlineStr"/>
@@ -10092,17 +10104,17 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F122" s="11" t="inlineStr">
@@ -10115,10 +10127,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H122" s="11" t="inlineStr"/>
+      <c r="H122" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I122" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J122" s="11" t="inlineStr"/>
@@ -10139,17 +10155,17 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F123" s="11" t="inlineStr">
@@ -10162,10 +10178,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H123" s="11" t="inlineStr"/>
-      <c r="I123" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H123" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J123" s="11" t="inlineStr"/>
@@ -10186,12 +10206,12 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
@@ -10209,20 +10229,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H124" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
-        </is>
-      </c>
-      <c r="I124" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H124" s="11" t="inlineStr"/>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J124" s="11" t="inlineStr"/>
       <c r="K124" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10237,12 +10253,12 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
@@ -10284,12 +10300,12 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -10307,16 +10323,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H126" s="11" t="inlineStr"/>
-      <c r="I126" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="H126" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I126" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J126" s="11" t="inlineStr"/>
       <c r="K126" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10331,12 +10351,12 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -10378,12 +10398,12 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -10401,20 +10421,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H128" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I128" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H128" s="11" t="inlineStr"/>
+      <c r="I128" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J128" s="11" t="inlineStr"/>
       <c r="K128" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10429,12 +10445,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10453,9 +10469,9 @@
         </is>
       </c>
       <c r="H129" s="11" t="inlineStr"/>
-      <c r="I129" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I129" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J129" s="11" t="inlineStr"/>
@@ -10476,12 +10492,12 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10499,16 +10515,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H130" s="11" t="inlineStr"/>
-      <c r="I130" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H130" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
+        </is>
+      </c>
+      <c r="I130" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J130" s="11" t="inlineStr"/>
       <c r="K130" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10523,12 +10543,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10547,9 +10567,9 @@
         </is>
       </c>
       <c r="H131" s="11" t="inlineStr"/>
-      <c r="I131" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I131" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J131" s="11" t="inlineStr"/>
@@ -10570,12 +10590,12 @@
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -10596,7 +10616,7 @@
       <c r="H132" s="11" t="inlineStr"/>
       <c r="I132" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J132" s="11" t="inlineStr"/>
@@ -10617,12 +10637,12 @@
       </c>
       <c r="C133" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D133" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
@@ -10664,12 +10684,12 @@
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D134" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E134" s="11" t="inlineStr">
@@ -10687,16 +10707,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H134" s="11" t="inlineStr"/>
-      <c r="I134" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H134" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I134" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J134" s="11" t="inlineStr"/>
       <c r="K134" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10711,12 +10735,12 @@
       </c>
       <c r="C135" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D135" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
@@ -10758,12 +10782,12 @@
       </c>
       <c r="C136" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
@@ -10805,12 +10829,12 @@
       </c>
       <c r="C137" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D137" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E137" s="11" t="inlineStr">
@@ -10841,18 +10865,300 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="11" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>Budgetary Estimate (p.99)</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+        </is>
+      </c>
+      <c r="E138" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F138" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G138" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H138" s="11" t="inlineStr"/>
+      <c r="I138" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J138" s="11" t="inlineStr"/>
+      <c r="K138" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>References (p.100)</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr">
+        <is>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+        </is>
+      </c>
+      <c r="E139" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G139" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H139" s="11" t="inlineStr"/>
+      <c r="I139" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J139" s="11" t="inlineStr"/>
+      <c r="K139" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>References (p.10 / refs)</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+        </is>
+      </c>
+      <c r="E140" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F140" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G140" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H140" s="11" t="inlineStr"/>
+      <c r="I140" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J140" s="11" t="inlineStr"/>
+      <c r="K140" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C141" s="11" t="inlineStr">
+        <is>
+          <t>References (p.17 / refs)</t>
+        </is>
+      </c>
+      <c r="D141" s="11" t="inlineStr">
+        <is>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+        </is>
+      </c>
+      <c r="E141" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F141" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G141" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H141" s="11" t="inlineStr"/>
+      <c r="I141" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J141" s="11" t="inlineStr"/>
+      <c r="K141" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>Appendices (p.124)</t>
+        </is>
+      </c>
+      <c r="D142" s="11" t="inlineStr">
+        <is>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+        </is>
+      </c>
+      <c r="E142" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F142" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G142" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H142" s="11" t="inlineStr"/>
+      <c r="I142" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J142" s="11" t="inlineStr"/>
+      <c r="K142" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D143" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G143" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H143" s="11" t="inlineStr"/>
+      <c r="I143" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J143" s="11" t="inlineStr"/>
+      <c r="K143" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K137"/>
-  <conditionalFormatting sqref="K2:K137">
+  <autoFilter ref="A1:K143"/>
+  <conditionalFormatting sqref="K2:K143">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Remove the Inventory Movement chart from the dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$144</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9951,17 +9951,17 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F119" s="11" t="inlineStr">
@@ -9976,12 +9976,12 @@
       </c>
       <c r="H119" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I119" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
+        </is>
+      </c>
+      <c r="I119" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J119" s="11" t="inlineStr"/>
@@ -10002,12 +10002,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
@@ -10030,9 +10030,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I120" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I120" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J120" s="11" t="inlineStr"/>
@@ -10053,12 +10053,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -10081,9 +10081,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I121" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I121" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J121" s="11" t="inlineStr"/>
@@ -10104,12 +10104,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -10155,12 +10155,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -10180,12 +10180,12 @@
       </c>
       <c r="H123" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I123" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J123" s="11" t="inlineStr"/>
@@ -10206,17 +10206,17 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F124" s="11" t="inlineStr">
@@ -10229,7 +10229,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H124" s="11" t="inlineStr"/>
+      <c r="H124" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I124" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -10253,12 +10257,12 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
@@ -10277,9 +10281,9 @@
         </is>
       </c>
       <c r="H125" s="11" t="inlineStr"/>
-      <c r="I125" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J125" s="11" t="inlineStr"/>
@@ -10300,12 +10304,12 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -10323,11 +10327,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H126" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
+      <c r="H126" s="11" t="inlineStr"/>
       <c r="I126" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10336,7 +10336,7 @@
       <c r="J126" s="11" t="inlineStr"/>
       <c r="K126" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10351,12 +10351,12 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -10374,16 +10374,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H127" s="11" t="inlineStr"/>
-      <c r="I127" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H127" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I127" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J127" s="11" t="inlineStr"/>
       <c r="K127" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10398,12 +10402,12 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -10445,12 +10449,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10469,9 +10473,9 @@
         </is>
       </c>
       <c r="H129" s="11" t="inlineStr"/>
-      <c r="I129" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I129" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J129" s="11" t="inlineStr"/>
@@ -10497,7 +10501,7 @@
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10515,11 +10519,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H130" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
-        </is>
-      </c>
+      <c r="H130" s="11" t="inlineStr"/>
       <c r="I130" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10528,7 +10528,7 @@
       <c r="J130" s="11" t="inlineStr"/>
       <c r="K130" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10543,12 +10543,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10566,7 +10566,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H131" s="11" t="inlineStr"/>
+      <c r="H131" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: dashboard now has the inventory movement chart.</t>
+        </is>
+      </c>
       <c r="I131" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -10575,7 +10579,7 @@
       <c r="J131" s="11" t="inlineStr"/>
       <c r="K131" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10590,12 +10594,12 @@
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -10614,9 +10618,9 @@
         </is>
       </c>
       <c r="H132" s="11" t="inlineStr"/>
-      <c r="I132" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I132" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J132" s="11" t="inlineStr"/>
@@ -10637,12 +10641,12 @@
       </c>
       <c r="C133" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D133" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
@@ -10663,7 +10667,7 @@
       <c r="H133" s="11" t="inlineStr"/>
       <c r="I133" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J133" s="11" t="inlineStr"/>
@@ -10684,12 +10688,12 @@
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D134" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E134" s="11" t="inlineStr">
@@ -10707,20 +10711,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H134" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I134" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H134" s="11" t="inlineStr"/>
+      <c r="I134" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J134" s="11" t="inlineStr"/>
       <c r="K134" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10735,12 +10735,12 @@
       </c>
       <c r="C135" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D135" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
@@ -10758,16 +10758,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H135" s="11" t="inlineStr"/>
-      <c r="I135" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H135" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I135" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J135" s="11" t="inlineStr"/>
       <c r="K135" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10782,12 +10786,12 @@
       </c>
       <c r="C136" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
@@ -10829,12 +10833,12 @@
       </c>
       <c r="C137" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D137" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E137" s="11" t="inlineStr">
@@ -10881,7 +10885,7 @@
       </c>
       <c r="D138" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E138" s="11" t="inlineStr">
@@ -10923,12 +10927,12 @@
       </c>
       <c r="C139" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D139" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E139" s="11" t="inlineStr">
@@ -10970,12 +10974,12 @@
       </c>
       <c r="C140" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D140" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E140" s="11" t="inlineStr">
@@ -11017,12 +11021,12 @@
       </c>
       <c r="C141" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D141" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E141" s="11" t="inlineStr">
@@ -11064,12 +11068,12 @@
       </c>
       <c r="C142" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D142" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E142" s="11" t="inlineStr">
@@ -11111,12 +11115,12 @@
       </c>
       <c r="C143" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Appendices (p.124)</t>
         </is>
       </c>
       <c r="D143" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
         </is>
       </c>
       <c r="E143" s="11" t="inlineStr">
@@ -11147,18 +11151,65 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D144" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E144" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F144" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G144" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H144" s="11" t="inlineStr"/>
+      <c r="I144" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J144" s="11" t="inlineStr"/>
+      <c r="K144" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K143"/>
-  <conditionalFormatting sqref="K2:K143">
+  <autoFilter ref="A1:K144"/>
+  <conditionalFormatting sqref="K2:K144">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: items added as done now show Done; chat-dependent paper items closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4177,7 +4177,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr"/>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>DONE chat is built (80b3988); keep the tick.</t>
+        </is>
+      </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -4186,7 +4190,7 @@
       <c r="J4" s="11" t="inlineStr"/>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4853,7 @@
       <c r="J17" s="11" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4900,7 +4904,7 @@
       <c r="J18" s="11" t="inlineStr"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4955,7 @@
       <c r="J19" s="11" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5546,7 +5550,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr"/>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>DONE chat is built; keep 'coordinated through live chat'.</t>
+        </is>
+      </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -5555,7 +5563,7 @@
       <c r="J31" s="11" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6873,7 @@
       <c r="J57" s="11" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6916,7 +6924,7 @@
       <c r="J58" s="11" t="inlineStr"/>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6975,7 @@
       <c r="J59" s="11" t="inlineStr"/>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9119,7 +9127,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H102" s="11" t="inlineStr"/>
+      <c r="H102" s="11" t="inlineStr">
+        <is>
+          <t>DONE chat is built; keep the sentence.</t>
+        </is>
+      </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -9128,7 +9140,7 @@
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: chat order cards, free-plan changes, Firestore usage watch item
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K167"/>
+  <dimension ref="A1:K169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>DONE same commit as the Cloudinary/Firestore free-plan changes; reports and dashboard still read full history by design. Needed before real use with the client's ~1,000-product catalog.</t>
+          <t>DONE 6bdc6a6; reports and dashboard still read full history by design. Needed before real use with the client's ~1,000-product catalog.</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="H67" s="11" t="inlineStr">
         <is>
-          <t>DONE resized delivery URLs (f_auto,q_auto,w_), photos shrunk before upload by kind; shop catalog cached 5 min in the browser, staff bell cached 2 min with status-filtered order/PO reads, Inventory and Orders read once via their live listeners. Keeps Cloudinary and Firestore on the free plans as visits grow. Offered, not built yet.</t>
+          <t>DONE 6bdc6a6: resized delivery URLs (f_auto,q_auto,w_), photos shrunk before upload by kind; shop catalog cached 5 min in the browser, staff bell cached 2 min with status-filtered order/PO reads, Inventory and Orders read once via their live listeners. Keeps Cloudinary and Firestore on the free plans as visits grow. Offered, not built yet.</t>
         </is>
       </c>
       <c r="I67" s="11" t="inlineStr">
@@ -7398,17 +7398,17 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>Live chat module, Online order tracking</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>Live chat order cards: products with photos, progress tracker with dates, delivery or pick-up, what happens next, Track rider; live status; Gemini routes order questions the word list misses</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
-          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
+          <t>DONE d16bd76. Several orders show as short cards with Show details; follow-up buttons fit the status.</t>
         </is>
       </c>
       <c r="I68" s="11" t="inlineStr">
@@ -7449,12 +7449,12 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
         </is>
       </c>
       <c r="I69" s="11" t="inlineStr">
@@ -7500,12 +7500,12 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>DONE footer links to legal.html on every page.</t>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
@@ -7546,17 +7546,17 @@
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -7576,12 +7576,12 @@
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+          <t>DONE footer links to legal.html on every page.</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr"/>
@@ -7597,22 +7597,22 @@
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>REQ001 registration, Scope and Limitations</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Phone number verification by SMS code: on hold (every SMS costs money; Amson doesn't want to spend)</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>Paper: state in Limitations (number format checked, not ownership) and in Recommendations (SMS OTP).</t>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
@@ -7638,7 +7638,7 @@
       <c r="J72" s="11" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7653,17 +7653,17 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Chapter 3 evaluation (Objective 4)</t>
+          <t>REQ001 registration, Scope and Limitations</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Evaluation survey questionnaires: Branch Manager, Technical Staff, Sales Staff and User forms, mapped to TAM + ISO/IEC 25010</t>
+          <t>Phone number verification by SMS code: on hold (every SMS costs money; Amson doesn't want to spend)</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>DONE Claude Docs, 2026-10-22. In Claude Docs ('Survey Questionnaires (Admin and User)'); maintainability covered by the developers' testing (no IT expert form).</t>
+          <t>Paper: state in Limitations (number format checked, not ownership) and in Recommendations (SMS OTP).</t>
         </is>
       </c>
       <c r="I73" s="11" t="inlineStr">
@@ -7689,7 +7689,7 @@
       <c r="J73" s="11" t="inlineStr"/>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -7704,17 +7704,17 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Chapter 3 evaluation (Objective 4)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>Evaluation survey questionnaires: Branch Manager, Technical Staff, Sales Staff and User forms, mapped to TAM + ISO/IEC 25010</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE Claude Docs, 2026-10-22. In Claude Docs ('Survey Questionnaires (Admin and User)'); maintainability covered by the developers' testing (no IT expert form).</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
@@ -7740,7 +7740,7 @@
       <c r="J74" s="11" t="inlineStr"/>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7755,12 +7755,12 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
@@ -7783,9 +7783,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I75" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J75" s="11" t="inlineStr"/>
@@ -7806,12 +7806,12 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -7857,12 +7857,12 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -7885,9 +7885,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I77" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J77" s="11" t="inlineStr"/>
@@ -7908,12 +7908,12 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -7959,12 +7959,12 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
@@ -7987,9 +7987,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I79" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
@@ -8010,12 +8010,12 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
@@ -8061,12 +8061,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
@@ -8089,9 +8089,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I81" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I81" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr"/>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -8163,12 +8163,12 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
@@ -8214,12 +8214,12 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -8265,12 +8265,12 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
@@ -8316,12 +8316,12 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -8367,12 +8367,12 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
@@ -8418,12 +8418,12 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
@@ -8520,12 +8520,12 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -8571,17 +8571,17 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F91" s="11" t="inlineStr">
@@ -8594,7 +8594,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H91" s="11" t="inlineStr"/>
+      <c r="H91" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -8618,12 +8622,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -8633,7 +8637,7 @@
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G92" s="11" t="inlineStr">
@@ -8665,12 +8669,12 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
@@ -8680,7 +8684,7 @@
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G93" s="11" t="inlineStr">
@@ -8712,12 +8716,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -8736,9 +8740,9 @@
         </is>
       </c>
       <c r="H94" s="11" t="inlineStr"/>
-      <c r="I94" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I94" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J94" s="11" t="inlineStr"/>
@@ -8759,12 +8763,12 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
@@ -8783,9 +8787,9 @@
         </is>
       </c>
       <c r="H95" s="11" t="inlineStr"/>
-      <c r="I95" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J95" s="11" t="inlineStr"/>
@@ -8806,12 +8810,12 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
@@ -8858,7 +8862,7 @@
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
@@ -8895,42 +8899,38 @@
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G98" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H98" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED (revised): build it to avoid a removal letter.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H98" s="11" t="inlineStr"/>
       <c r="I98" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J98" s="11" t="inlineStr"/>
@@ -8951,17 +8951,17 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F99" s="11" t="inlineStr">
@@ -8976,18 +8976,18 @@
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J99" s="11" t="inlineStr"/>
       <c r="K99" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9002,12 +9002,12 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
@@ -9053,12 +9053,12 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
@@ -9068,7 +9068,7 @@
       </c>
       <c r="F101" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G101" s="11" t="inlineStr">
@@ -9078,7 +9078,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
@@ -9099,22 +9099,22 @@
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
@@ -9129,18 +9129,18 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>DONE chat is built; keep the sentence.</t>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -9150,22 +9150,22 @@
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F103" s="11" t="inlineStr">
@@ -9180,7 +9180,7 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE chat is built; keep the sentence.</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
@@ -9206,17 +9206,17 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
@@ -9257,12 +9257,12 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="H105" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I105" s="11" t="inlineStr">
@@ -9308,12 +9308,12 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I106" s="11" t="inlineStr">
@@ -9359,17 +9359,17 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F107" s="11" t="inlineStr">
@@ -9384,7 +9384,7 @@
       </c>
       <c r="H107" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I107" s="11" t="inlineStr">
@@ -9410,17 +9410,17 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I108" s="11" t="inlineStr">
@@ -9461,17 +9461,17 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F109" s="11" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="H109" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92. From the first review.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I109" s="11" t="inlineStr">
@@ -9512,12 +9512,12 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
@@ -9537,7 +9537,7 @@
       </c>
       <c r="H110" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I110" s="11" t="inlineStr">
@@ -9563,12 +9563,12 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="H111" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I111" s="11" t="inlineStr">
@@ -9614,12 +9614,12 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE 082ec92.</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
@@ -9665,17 +9665,17 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F113" s="11" t="inlineStr">
@@ -9690,7 +9690,7 @@
       </c>
       <c r="H113" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I113" s="11" t="inlineStr">
@@ -9716,17 +9716,17 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F114" s="11" t="inlineStr">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="H114" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I114" s="11" t="inlineStr">
@@ -9767,17 +9767,17 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F115" s="11" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="H115" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I115" s="11" t="inlineStr">
@@ -9818,17 +9818,17 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F116" s="11" t="inlineStr">
@@ -9843,7 +9843,7 @@
       </c>
       <c r="H116" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3. From the first review.</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I116" s="11" t="inlineStr">
@@ -9869,17 +9869,17 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F117" s="11" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="H117" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b. From the first review.</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I117" s="11" t="inlineStr">
@@ -9920,17 +9920,17 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F118" s="11" t="inlineStr">
@@ -9945,7 +9945,7 @@
       </c>
       <c r="H118" s="11" t="inlineStr">
         <is>
-          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
+          <t>DONE d9fc96b. From the first review.</t>
         </is>
       </c>
       <c r="I118" s="11" t="inlineStr">
@@ -9971,17 +9971,17 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>REQ031</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F119" s="11" t="inlineStr">
@@ -9996,7 +9996,7 @@
       </c>
       <c r="H119" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
+          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
         </is>
       </c>
       <c r="I119" s="11" t="inlineStr">
@@ -10022,17 +10022,17 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F120" s="11" t="inlineStr">
@@ -10047,18 +10047,18 @@
       </c>
       <c r="H120" s="11" t="inlineStr">
         <is>
-          <t>Built (stock in vs out), then removed at the team's request 2026-10-21 - see the Removals sheet. Keeps the Chart.js claim (no letter).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J120" s="11" t="inlineStr"/>
       <c r="K120" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10073,12 +10073,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Modules p.42</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -10098,18 +10098,18 @@
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+          <t>Built (stock in vs out), then removed at the team's request 2026-10-21 - see the Removals sheet. Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J121" s="11" t="inlineStr"/>
       <c r="K121" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -10124,12 +10124,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework p.23</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="H122" s="11" t="inlineStr">
         <is>
-          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
         </is>
       </c>
       <c r="I122" s="11" t="inlineStr">
@@ -10175,12 +10175,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="H123" s="11" t="inlineStr">
         <is>
-          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
+          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
         </is>
       </c>
       <c r="I123" s="11" t="inlineStr">
@@ -10226,17 +10226,17 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>REQ004</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F124" s="11" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="H124" s="11" t="inlineStr">
         <is>
-          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
+          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
         </is>
       </c>
       <c r="I124" s="11" t="inlineStr">
@@ -10262,7 +10262,7 @@
       <c r="J124" s="11" t="inlineStr"/>
       <c r="K124" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10277,17 +10277,17 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Inventory module</t>
+          <t>REQ004</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>Inventory list: drop the 'Never received' placeholder rows</t>
+          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F125" s="11" t="inlineStr">
@@ -10302,7 +10302,7 @@
       </c>
       <c r="H125" s="11" t="inlineStr">
         <is>
-          <t>DONE 66b8b2e. Products never stocked no longer show as empty batch rows.</t>
+          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
         </is>
       </c>
       <c r="I125" s="11" t="inlineStr">
@@ -10313,7 +10313,7 @@
       <c r="J125" s="11" t="inlineStr"/>
       <c r="K125" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10328,12 +10328,12 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>REQ001 registration validation</t>
+          <t>Inventory module</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Name fields allow periods and dashes (Ma. Clara, Juan P. Cruz, Jr., Anne-Marie)</t>
+          <t>Inventory list: drop the 'Never received' placeholder rows</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -10353,7 +10353,7 @@
       </c>
       <c r="H126" s="11" t="inlineStr">
         <is>
-          <t>DONE 010449e, 8ce4aa0. Same rule on register, account settings, staff and admin settings.</t>
+          <t>DONE 66b8b2e. Products never stocked no longer show as empty batch rows.</t>
         </is>
       </c>
       <c r="I126" s="11" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>Checkout module, REQ019</t>
+          <t>REQ001 registration validation</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Checkout: Same Day Delivery wording and a notice that the Lalamove fee is paid to the rider</t>
+          <t>Name fields allow periods and dashes (Ma. Clara, Juan P. Cruz, Jr., Anne-Marie)</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="H127" s="11" t="inlineStr">
         <is>
-          <t>DONE 010449e.</t>
+          <t>DONE 010449e, 8ce4aa0. Same rule on register, account settings, staff and admin settings.</t>
         </is>
       </c>
       <c r="I127" s="11" t="inlineStr">
@@ -10430,12 +10430,12 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>EmailJS (Technical Background)</t>
+          <t>Checkout module, REQ019</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>Settings: Email Test button that shows EmailJS's reply</t>
+          <t>Checkout: Same Day Delivery wording and a notice that the Lalamove fee is paid to the rider</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="H128" s="11" t="inlineStr">
         <is>
-          <t>DONE 4eca895. Found the order template was missing To Email {{to_email}} - set it in the EmailJS dashboard before go-live.</t>
+          <t>DONE 010449e.</t>
         </is>
       </c>
       <c r="I128" s="11" t="inlineStr">
@@ -10481,12 +10481,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Shopping cart module</t>
+          <t>EmailJS (Technical Background)</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>Cart page: 'You May Also Like' product suggestions under the cart items</t>
+          <t>Settings: Email Test button that shows EmailJS's reply</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="H129" s="11" t="inlineStr">
         <is>
-          <t>DONE 1581610. Team request 2026-10-21 (like Shopee).</t>
+          <t>DONE 4eca895. Found the order template was missing To Email {{to_email}} - set it in the EmailJS dashboard before go-live.</t>
         </is>
       </c>
       <c r="I129" s="11" t="inlineStr">
@@ -10532,12 +10532,12 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>Notification module</t>
+          <t>Shopping cart module</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>Notifications: filter by Orders / Stock / Live Chat, newest first, mark read per filter</t>
+          <t>Cart page: 'You May Also Like' product suggestions under the cart items</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10557,7 +10557,7 @@
       </c>
       <c r="H130" s="11" t="inlineStr">
         <is>
-          <t>DONE 1581610. Team request 2026-10-21.</t>
+          <t>DONE 1581610. Team request 2026-10-21 (like Shopee).</t>
         </is>
       </c>
       <c r="I130" s="11" t="inlineStr">
@@ -10583,12 +10583,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>Inventory module</t>
+          <t>Notification module</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>Inventory: 'Quantity' renamed to 'Available Inventory' (table and export)</t>
+          <t>Notifications: filter by Orders / Stock / Live Chat, newest first, mark read per filter</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10634,12 +10634,12 @@
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>All PDF exports</t>
+          <t>Inventory module</t>
         </is>
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>PDFs printed the peso sign as a broken character - now 'PHP'</t>
+          <t>Inventory: 'Quantity' renamed to 'Available Inventory' (table and export)</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -10659,7 +10659,7 @@
       </c>
       <c r="H132" s="11" t="inlineStr">
         <is>
-          <t>DONE a3f410b. jsPDF's built-in fonts have no peso sign.</t>
+          <t>DONE 1581610. Team request 2026-10-21.</t>
         </is>
       </c>
       <c r="I132" s="11" t="inlineStr">
@@ -10685,12 +10685,12 @@
       </c>
       <c r="C133" s="11" t="inlineStr">
         <is>
-          <t>Online order module</t>
+          <t>All PDF exports</t>
         </is>
       </c>
       <c r="D133" s="11" t="inlineStr">
         <is>
-          <t>Online Orders: Reference No. and SI No. columns (searchable); order date and time shown in Payment Verification</t>
+          <t>PDFs printed the peso sign as a broken character - now 'PHP'</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="H133" s="11" t="inlineStr">
         <is>
-          <t>DONE 2a52561, 8d5a42e. Team request 2026-10-21.</t>
+          <t>DONE a3f410b. jsPDF's built-in fonts have no peso sign.</t>
         </is>
       </c>
       <c r="I133" s="11" t="inlineStr">
@@ -10736,12 +10736,12 @@
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module, Reports module</t>
+          <t>Online order module</t>
         </is>
       </c>
       <c r="D134" s="11" t="inlineStr">
         <is>
-          <t>Reports moved out of the Orders tab: all reports open from the dashboard Reports panel</t>
+          <t>Online Orders: Reference No. and SI No. columns (searchable); order date and time shown in Payment Verification</t>
         </is>
       </c>
       <c r="E134" s="11" t="inlineStr">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="H134" s="11" t="inlineStr">
         <is>
-          <t>DONE 2a52561. Team request 2026-10-21. Paper: if the Orders module text mentions an export there, point it to Reports.</t>
+          <t>DONE 2a52561, 8d5a42e. Team request 2026-10-21.</t>
         </is>
       </c>
       <c r="I134" s="11" t="inlineStr">
@@ -10787,12 +10787,12 @@
       </c>
       <c r="C135" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module, sequential SI</t>
+          <t>Dashboard module, Reports module</t>
         </is>
       </c>
       <c r="D135" s="11" t="inlineStr">
         <is>
-          <t>Dashboard: Find a Sale by SI No. (walk-in, online and wholesale)</t>
+          <t>Reports moved out of the Orders tab: all reports open from the dashboard Reports panel</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="H135" s="11" t="inlineStr">
         <is>
-          <t>DONE 8d5a42e. Every sale gets an SI No.; online orders keep their order/reference numbers too.</t>
+          <t>DONE 2a52561. Team request 2026-10-21. Paper: if the Orders module text mentions an export there, point it to Reports.</t>
         </is>
       </c>
       <c r="I135" s="11" t="inlineStr">
@@ -10838,12 +10838,12 @@
       </c>
       <c r="C136" s="11" t="inlineStr">
         <is>
-          <t>Go-live</t>
+          <t>Dashboard module, sequential SI</t>
         </is>
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>Temporary Clear Test Data page (Branch Manager / Administrator) and its delete rule; both switch off 2026-11-15</t>
+          <t>Dashboard: Find a Sale by SI No. (walk-in, online and wholesale)</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="H136" s="11" t="inlineStr">
         <is>
-          <t>DONE 77fdd25, 112ce91 (publish firestore.rules to use it). Remove the page, its Settings card and the TEMPORARY rule block after go-live; not part of the paper.</t>
+          <t>DONE 8d5a42e. Every sale gets an SI No.; online orders keep their order/reference numbers too.</t>
         </is>
       </c>
       <c r="I136" s="11" t="inlineStr">
@@ -10889,17 +10889,17 @@
       </c>
       <c r="C137" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>Go-live</t>
         </is>
       </c>
       <c r="D137" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Temporary Clear Test Data page (Branch Manager / Administrator) and its delete rule; both switch off 2026-11-15</t>
         </is>
       </c>
       <c r="E137" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F137" s="11" t="inlineStr">
@@ -10912,7 +10912,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H137" s="11" t="inlineStr"/>
+      <c r="H137" s="11" t="inlineStr">
+        <is>
+          <t>DONE 77fdd25, 112ce91 (publish firestore.rules to use it). Remove the page, its Settings card and the TEMPORARY rule block after go-live; not part of the paper.</t>
+        </is>
+      </c>
       <c r="I137" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -10921,7 +10925,7 @@
       <c r="J137" s="11" t="inlineStr"/>
       <c r="K137" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10931,22 +10935,22 @@
       </c>
       <c r="B138" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C138" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>Tech Stack (free plans), REQNF013</t>
         </is>
       </c>
       <c r="D138" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>Watch Firestore usage after go-live: Dashboard and Reports still read the full sales history on each visit</t>
         </is>
       </c>
       <c r="E138" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F138" s="11" t="inlineStr">
@@ -10959,10 +10963,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H138" s="11" t="inlineStr"/>
+      <c r="H138" s="11" t="inlineStr">
+        <is>
+          <t>Fine at one branch's volume; if the 50,000 reads/day limit gets close, limit them to the chosen period.</t>
+        </is>
+      </c>
       <c r="I138" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J138" s="11" t="inlineStr"/>
@@ -10978,27 +10986,27 @@
       </c>
       <c r="B139" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C139" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D139" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E139" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F139" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G139" s="11" t="inlineStr">
@@ -11006,14 +11014,10 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H139" s="11" t="inlineStr">
-        <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
-        </is>
-      </c>
+      <c r="H139" s="11" t="inlineStr"/>
       <c r="I139" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J139" s="11" t="inlineStr"/>
@@ -11029,22 +11033,22 @@
       </c>
       <c r="B140" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C140" s="11" t="inlineStr">
         <is>
-          <t>REQ090</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D140" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E140" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F140" s="11" t="inlineStr">
@@ -11057,11 +11061,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H140" s="11" t="inlineStr">
-        <is>
-          <t>Rare; same-second exchanges on one line.</t>
-        </is>
-      </c>
+      <c r="H140" s="11" t="inlineStr"/>
       <c r="I140" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -11085,12 +11085,12 @@
       </c>
       <c r="C141" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D141" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E141" s="11" t="inlineStr">
@@ -11100,7 +11100,7 @@
       </c>
       <c r="F141" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G141" s="11" t="inlineStr">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="H141" s="11" t="inlineStr">
         <is>
-          <t>Needs a server function to clean up; note in the user manual.</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I141" s="11" t="inlineStr">
@@ -11136,17 +11136,17 @@
       </c>
       <c r="C142" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D142" s="11" t="inlineStr">
         <is>
-          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E142" s="11" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F142" s="11" t="inlineStr">
@@ -11161,12 +11161,12 @@
       </c>
       <c r="H142" s="11" t="inlineStr">
         <is>
-          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
-        </is>
-      </c>
-      <c r="I142" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Rare; same-second exchanges on one line.</t>
+        </is>
+      </c>
+      <c r="I142" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J142" s="11" t="inlineStr"/>
@@ -11187,17 +11187,17 @@
       </c>
       <c r="C143" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D143" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E143" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F143" s="11" t="inlineStr">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="H143" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Needs a server function to clean up; note in the user manual.</t>
         </is>
       </c>
       <c r="I143" s="11" t="inlineStr">
@@ -11238,17 +11238,17 @@
       </c>
       <c r="C144" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D144" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E144" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F144" s="11" t="inlineStr">
@@ -11263,7 +11263,7 @@
       </c>
       <c r="H144" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
         </is>
       </c>
       <c r="I144" s="12" t="inlineStr">
@@ -11289,12 +11289,12 @@
       </c>
       <c r="C145" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D145" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="I145" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J145" s="11" t="inlineStr"/>
@@ -11340,12 +11340,12 @@
       </c>
       <c r="C146" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D146" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
@@ -11368,9 +11368,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I146" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I146" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J146" s="11" t="inlineStr"/>
@@ -11391,12 +11391,12 @@
       </c>
       <c r="C147" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D147" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>The client also sells medical supplies and grocery items (monthly report); the paper only mentions OTC/prescription medicines. Mention them, or exclude them on purpose.</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
@@ -11416,12 +11416,12 @@
       </c>
       <c r="H147" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I147" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J147" s="11" t="inlineStr"/>
@@ -11442,17 +11442,17 @@
       </c>
       <c r="C148" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D148" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
@@ -11465,10 +11465,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H148" s="11" t="inlineStr"/>
+      <c r="H148" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I148" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J148" s="11" t="inlineStr"/>
@@ -11489,17 +11493,17 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D149" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F149" s="11" t="inlineStr">
@@ -11512,10 +11516,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H149" s="11" t="inlineStr"/>
-      <c r="I149" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H149" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I149" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J149" s="11" t="inlineStr"/>
@@ -11536,12 +11544,12 @@
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
@@ -11559,20 +11567,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H150" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
-      <c r="I150" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H150" s="11" t="inlineStr"/>
+      <c r="I150" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J150" s="11" t="inlineStr"/>
       <c r="K150" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -11587,12 +11591,12 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D151" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
@@ -11611,9 +11615,9 @@
         </is>
       </c>
       <c r="H151" s="11" t="inlineStr"/>
-      <c r="I151" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I151" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J151" s="11" t="inlineStr"/>
@@ -11634,12 +11638,12 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
@@ -11657,16 +11661,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H152" s="11" t="inlineStr"/>
-      <c r="I152" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H152" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I152" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J152" s="11" t="inlineStr"/>
       <c r="K152" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11681,12 +11689,12 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D153" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
@@ -11705,9 +11713,9 @@
         </is>
       </c>
       <c r="H153" s="11" t="inlineStr"/>
-      <c r="I153" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I153" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J153" s="11" t="inlineStr"/>
@@ -11728,12 +11736,12 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
@@ -11752,9 +11760,9 @@
         </is>
       </c>
       <c r="H154" s="11" t="inlineStr"/>
-      <c r="I154" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I154" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J154" s="11" t="inlineStr"/>
@@ -11775,12 +11783,12 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D155" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
@@ -11822,12 +11830,12 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
@@ -11846,9 +11854,9 @@
         </is>
       </c>
       <c r="H156" s="11" t="inlineStr"/>
-      <c r="I156" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I156" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr"/>
@@ -11869,12 +11877,12 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D157" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
@@ -11893,9 +11901,9 @@
         </is>
       </c>
       <c r="H157" s="11" t="inlineStr"/>
-      <c r="I157" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I157" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J157" s="11" t="inlineStr"/>
@@ -11916,12 +11924,12 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
@@ -11939,20 +11947,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H158" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I158" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H158" s="11" t="inlineStr"/>
+      <c r="I158" s="11" t="inlineStr">
+        <is>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J158" s="11" t="inlineStr"/>
       <c r="K158" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -11967,12 +11971,12 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D159" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
@@ -12014,12 +12018,12 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
@@ -12037,16 +12041,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H160" s="11" t="inlineStr"/>
-      <c r="I160" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H160" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I160" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J160" s="11" t="inlineStr"/>
       <c r="K160" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12061,12 +12069,12 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D161" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
@@ -12108,12 +12116,12 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
@@ -12155,12 +12163,12 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D163" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
@@ -12202,12 +12210,12 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -12249,12 +12257,12 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D165" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
@@ -12296,12 +12304,12 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -12343,12 +12351,12 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D167" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
@@ -12379,18 +12387,112 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C168" s="11" t="inlineStr">
+        <is>
+          <t>Appendices (p.124)</t>
+        </is>
+      </c>
+      <c r="D168" s="11" t="inlineStr">
+        <is>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+        </is>
+      </c>
+      <c r="E168" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F168" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G168" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H168" s="11" t="inlineStr"/>
+      <c r="I168" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J168" s="11" t="inlineStr"/>
+      <c r="K168" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C169" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D169" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E169" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F169" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G169" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H169" s="11" t="inlineStr"/>
+      <c r="I169" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J169" s="11" t="inlineStr"/>
+      <c r="K169" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K167"/>
-  <conditionalFormatting sqref="K2:K167">
+  <autoFilter ref="A1:K169"/>
+  <conditionalFormatting sqref="K2:K169">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19573,7 +19675,7 @@
       </c>
       <c r="F130" s="11" t="inlineStr">
         <is>
-          <t>21e505b: online orders, inventory, POS today's sales, customer order list and order page, and chat update live. Dashboard tiles refresh on load. (was: Users must reload to see new orders or stock changes.)</t>
+          <t>21e505b: online orders, inventory, POS today's sales, customer order list and order page, chat and chat order cards update live. Dashboard tiles refresh on load; the shop catalog refreshes every 5 minutes (checkout re-checks stock live). (was: Users must reload to see new orders or stock changes.)</t>
         </is>
       </c>
       <c r="G130" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register: full catalog POS-only, 50 demo products online; description and photo sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4081,7 +4081,7 @@
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>Rebuilt 2026-10-23: 42 price-0 lines (free goods / not priced) and 2 unpriced lines left out and listed. Tested through the importer. Upload as the Branch Manager, each file once. Not committed (client data).</t>
+          <t>Every product is in the POS; only the 50 demo products are also in the online store (the other 1,080 upload as POS-only). Rebuilt 2026-10-23: 42 price-0 lines (free goods / not priced) and 2 unpriced lines left out and listed. Tested through the importer. Upload as the Branch Manager, each file once. Not committed (client data).</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Picked from Amson's April 15 sales and everyday pharmacy needs (fever, cough/colds, allergy, stomach, vitamins, skin, maintenance medicines, supplies). Descriptions are label-level, no doses - pharmacist to read them. 'Demo photos' checklist in the read-me.</t>
+          <t>Picked from Amson's April 15 sales and everyday pharmacy needs (fever, cough/colds, allergy, stomach, vitamins, skin, maintenance medicines, supplies). Descriptions follow each medicine's standard approved use, no doses - the pharmacist checks them against the package insert of the box on the shelf (official wording; some also on the Philippine FDA verification portal). Photos: take them of Amson's own boxes (most of these local brands have no official images online). 'Demo photos' checklist in the read-me.</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Register: bulk photo upload (item 157)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$179</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K178"/>
+  <dimension ref="A1:K179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Picked from Amson's April 15 sales and everyday pharmacy needs (fever, cough/colds, allergy, stomach, vitamins, skin, maintenance medicines, supplies). Descriptions follow each medicine's standard approved use, no doses - the pharmacist checks them against the package insert of the box on the shelf (official wording; some also on the Philippine FDA verification portal). Photos: take them of Amson's own boxes (most of these local brands have no official images online). 'Demo photos' checklist in the read-me.</t>
+          <t>Picked from Amson's April 15 sales and everyday pharmacy needs (fever, cough/colds, allergy, stomach, vitamins, skin, maintenance medicines, supplies). Descriptions follow each medicine's standard approved use, no doses - the pharmacist checks them against the package insert of the box on the shelf (official wording; some also on the Philippine FDA verification portal). Photos: take them of Amson's own boxes (most of these local brands have no official images online), name each file after its product and add them all at once with Products &gt; Upload Photos (item 157). 'Demo photos' checklist in the read-me.</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
@@ -11450,17 +11450,17 @@
       </c>
       <c r="C148" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ064 batch upload, Product Management module</t>
         </is>
       </c>
       <c r="D148" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Bulk photo upload (Products &gt; Upload Photos): pick many photos at once, each matched to a product by its file name (brand, strength, form, or SKU), staff check/change every match, then all are shrunk, uploaded to Cloudinary and saved together; audit-logged</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
@@ -11473,7 +11473,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H148" s="11" t="inlineStr"/>
+      <c r="H148" s="11" t="inlineStr">
+        <is>
+          <t>DONE 17d8caa. Branch Manager and Technical Staff (not Sales Staff). Ambiguous names (e.g. 'cetirizine.jpg' when there's a tablet and a syrup) are left for staff to choose; two photos for one product are blocked. Paper (optional): one sentence under REQ064 / Product Management.</t>
+        </is>
+      </c>
       <c r="I148" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -11482,7 +11486,7 @@
       <c r="J148" s="11" t="inlineStr"/>
       <c r="K148" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11492,17 +11496,17 @@
       </c>
       <c r="B149" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D149" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
@@ -11523,7 +11527,7 @@
       <c r="H149" s="11" t="inlineStr"/>
       <c r="I149" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J149" s="11" t="inlineStr"/>
@@ -11539,27 +11543,27 @@
       </c>
       <c r="B150" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F150" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G150" s="11" t="inlineStr">
@@ -11567,11 +11571,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H150" s="11" t="inlineStr">
-        <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
-        </is>
-      </c>
+      <c r="H150" s="11" t="inlineStr"/>
       <c r="I150" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -11595,12 +11595,12 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>REQ090</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D151" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="F151" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G151" s="11" t="inlineStr">
@@ -11620,7 +11620,7 @@
       </c>
       <c r="H151" s="11" t="inlineStr">
         <is>
-          <t>Rare; same-second exchanges on one line.</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I151" s="11" t="inlineStr">
@@ -11646,12 +11646,12 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Needs a server function to clean up; note in the user manual.</t>
+          <t>Rare; same-second exchanges on one line.</t>
         </is>
       </c>
       <c r="I152" s="11" t="inlineStr">
@@ -11697,17 +11697,17 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D153" s="11" t="inlineStr">
         <is>
-          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
@@ -11722,12 +11722,12 @@
       </c>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
-        </is>
-      </c>
-      <c r="I153" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Needs a server function to clean up; note in the user manual.</t>
+        </is>
+      </c>
+      <c r="I153" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J153" s="11" t="inlineStr"/>
@@ -11748,17 +11748,17 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
@@ -11773,12 +11773,12 @@
       </c>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I154" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
+        </is>
+      </c>
+      <c r="I154" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J154" s="11" t="inlineStr"/>
@@ -11799,12 +11799,12 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D155" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
@@ -11827,9 +11827,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I155" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I155" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J155" s="11" t="inlineStr"/>
@@ -11850,12 +11850,12 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
@@ -11878,9 +11878,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I156" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I156" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr"/>
@@ -11901,12 +11901,12 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D157" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
@@ -11952,12 +11952,12 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
@@ -11977,12 +11977,12 @@
       </c>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I158" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J158" s="11" t="inlineStr"/>
@@ -12003,17 +12003,17 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D159" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F159" s="11" t="inlineStr">
@@ -12026,7 +12026,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H159" s="11" t="inlineStr"/>
+      <c r="H159" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I159" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -12050,12 +12054,12 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
@@ -12074,9 +12078,9 @@
         </is>
       </c>
       <c r="H160" s="11" t="inlineStr"/>
-      <c r="I160" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I160" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J160" s="11" t="inlineStr"/>
@@ -12097,12 +12101,12 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D161" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
@@ -12120,11 +12124,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H161" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
+      <c r="H161" s="11" t="inlineStr"/>
       <c r="I161" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -12133,7 +12133,7 @@
       <c r="J161" s="11" t="inlineStr"/>
       <c r="K161" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12148,12 +12148,12 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
@@ -12171,16 +12171,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H162" s="11" t="inlineStr"/>
-      <c r="I162" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H162" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I162" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J162" s="11" t="inlineStr"/>
       <c r="K162" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12195,12 +12199,12 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D163" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
@@ -12242,12 +12246,12 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -12266,9 +12270,9 @@
         </is>
       </c>
       <c r="H164" s="11" t="inlineStr"/>
-      <c r="I164" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I164" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J164" s="11" t="inlineStr"/>
@@ -12294,7 +12298,7 @@
       </c>
       <c r="D165" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
@@ -12336,12 +12340,12 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -12383,12 +12387,12 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D167" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
@@ -12407,9 +12411,9 @@
         </is>
       </c>
       <c r="H167" s="11" t="inlineStr"/>
-      <c r="I167" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I167" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J167" s="11" t="inlineStr"/>
@@ -12430,12 +12434,12 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D168" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
@@ -12456,7 +12460,7 @@
       <c r="H168" s="11" t="inlineStr"/>
       <c r="I168" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J168" s="11" t="inlineStr"/>
@@ -12477,12 +12481,12 @@
       </c>
       <c r="C169" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D169" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
@@ -12500,20 +12504,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H169" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I169" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H169" s="11" t="inlineStr"/>
+      <c r="I169" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J169" s="11" t="inlineStr"/>
       <c r="K169" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12528,12 +12528,12 @@
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
@@ -12551,16 +12551,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H170" s="11" t="inlineStr"/>
-      <c r="I170" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H170" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I170" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J170" s="11" t="inlineStr"/>
       <c r="K170" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12575,12 +12579,12 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D171" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
@@ -12622,12 +12626,12 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
@@ -12674,7 +12678,7 @@
       </c>
       <c r="D173" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
@@ -12716,12 +12720,12 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
@@ -12763,12 +12767,12 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D175" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
@@ -12810,12 +12814,12 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
@@ -12857,12 +12861,12 @@
       </c>
       <c r="C177" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D177" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
@@ -12904,12 +12908,12 @@
       </c>
       <c r="C178" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Appendices (p.124)</t>
         </is>
       </c>
       <c r="D178" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
@@ -12940,18 +12944,65 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C179" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D179" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E179" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F179" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G179" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H179" s="11" t="inlineStr"/>
+      <c r="I179" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J179" s="11" t="inlineStr"/>
+      <c r="K179" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K178"/>
-  <conditionalFormatting sqref="K2:K178">
+  <autoFilter ref="A1:K179"/>
+  <conditionalFormatting sqref="K2:K179">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: Products page upload UI (item 158)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K179"/>
+  <dimension ref="A1:K180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11501,17 +11501,17 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ064 batch upload, Product Management module, REQNF usability</t>
         </is>
       </c>
       <c r="D149" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Products page UI: Upload Photos is a two-step modal (choose/drop photos with naming tips, then check matches with filters and a searchable product picker); progress and result pop-ups for photo saving and batch import (import result offers Add photos, failed rows kept for retry); batch import audit-logged</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F149" s="11" t="inlineStr">
@@ -11524,7 +11524,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H149" s="11" t="inlineStr"/>
+      <c r="H149" s="11" t="inlineStr">
+        <is>
+          <t>DONE 93635fd. Client/team feedback 2026-10-23: it was hard to tell when an import had finished.</t>
+        </is>
+      </c>
       <c r="I149" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -11533,7 +11537,7 @@
       <c r="J149" s="11" t="inlineStr"/>
       <c r="K149" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11543,17 +11547,17 @@
       </c>
       <c r="B150" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
@@ -11574,7 +11578,7 @@
       <c r="H150" s="11" t="inlineStr"/>
       <c r="I150" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J150" s="11" t="inlineStr"/>
@@ -11590,27 +11594,27 @@
       </c>
       <c r="B151" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D151" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G151" s="11" t="inlineStr">
@@ -11618,11 +11622,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H151" s="11" t="inlineStr">
-        <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
-        </is>
-      </c>
+      <c r="H151" s="11" t="inlineStr"/>
       <c r="I151" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -11646,12 +11646,12 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>REQ090</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
@@ -11661,7 +11661,7 @@
       </c>
       <c r="F152" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G152" s="11" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Rare; same-second exchanges on one line.</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I152" s="11" t="inlineStr">
@@ -11697,12 +11697,12 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D153" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Needs a server function to clean up; note in the user manual.</t>
+          <t>Rare; same-second exchanges on one line.</t>
         </is>
       </c>
       <c r="I153" s="11" t="inlineStr">
@@ -11748,17 +11748,17 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
@@ -11773,12 +11773,12 @@
       </c>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
-        </is>
-      </c>
-      <c r="I154" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Needs a server function to clean up; note in the user manual.</t>
+        </is>
+      </c>
+      <c r="I154" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J154" s="11" t="inlineStr"/>
@@ -11799,17 +11799,17 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D155" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F155" s="11" t="inlineStr">
@@ -11824,12 +11824,12 @@
       </c>
       <c r="H155" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I155" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
+        </is>
+      </c>
+      <c r="I155" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J155" s="11" t="inlineStr"/>
@@ -11850,12 +11850,12 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
@@ -11878,9 +11878,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I156" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I156" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr"/>
@@ -11901,12 +11901,12 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D157" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
@@ -11929,9 +11929,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I157" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I157" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J157" s="11" t="inlineStr"/>
@@ -11952,12 +11952,12 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
@@ -12003,12 +12003,12 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D159" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
@@ -12028,12 +12028,12 @@
       </c>
       <c r="H159" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I159" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J159" s="11" t="inlineStr"/>
@@ -12054,17 +12054,17 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F160" s="11" t="inlineStr">
@@ -12077,7 +12077,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H160" s="11" t="inlineStr"/>
+      <c r="H160" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I160" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -12101,12 +12105,12 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D161" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
@@ -12125,9 +12129,9 @@
         </is>
       </c>
       <c r="H161" s="11" t="inlineStr"/>
-      <c r="I161" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I161" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J161" s="11" t="inlineStr"/>
@@ -12148,12 +12152,12 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
@@ -12171,11 +12175,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H162" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
+      <c r="H162" s="11" t="inlineStr"/>
       <c r="I162" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -12184,7 +12184,7 @@
       <c r="J162" s="11" t="inlineStr"/>
       <c r="K162" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12199,12 +12199,12 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D163" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
@@ -12222,16 +12222,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H163" s="11" t="inlineStr"/>
-      <c r="I163" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H163" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I163" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J163" s="11" t="inlineStr"/>
       <c r="K163" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12246,12 +12250,12 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -12293,12 +12297,12 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D165" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
@@ -12317,9 +12321,9 @@
         </is>
       </c>
       <c r="H165" s="11" t="inlineStr"/>
-      <c r="I165" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I165" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J165" s="11" t="inlineStr"/>
@@ -12345,7 +12349,7 @@
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -12387,12 +12391,12 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D167" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
@@ -12434,12 +12438,12 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D168" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
@@ -12458,9 +12462,9 @@
         </is>
       </c>
       <c r="H168" s="11" t="inlineStr"/>
-      <c r="I168" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I168" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J168" s="11" t="inlineStr"/>
@@ -12481,12 +12485,12 @@
       </c>
       <c r="C169" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D169" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
@@ -12507,7 +12511,7 @@
       <c r="H169" s="11" t="inlineStr"/>
       <c r="I169" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J169" s="11" t="inlineStr"/>
@@ -12528,12 +12532,12 @@
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
@@ -12551,20 +12555,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H170" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I170" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H170" s="11" t="inlineStr"/>
+      <c r="I170" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J170" s="11" t="inlineStr"/>
       <c r="K170" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12579,12 +12579,12 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D171" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
@@ -12602,16 +12602,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H171" s="11" t="inlineStr"/>
-      <c r="I171" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H171" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I171" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J171" s="11" t="inlineStr"/>
       <c r="K171" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12626,12 +12630,12 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
@@ -12673,12 +12677,12 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D173" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
@@ -12725,7 +12729,7 @@
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
@@ -12767,12 +12771,12 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D175" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
@@ -12814,12 +12818,12 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
@@ -12861,12 +12865,12 @@
       </c>
       <c r="C177" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D177" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
@@ -12908,12 +12912,12 @@
       </c>
       <c r="C178" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D178" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
@@ -12955,12 +12959,12 @@
       </c>
       <c r="C179" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Appendices (p.124)</t>
         </is>
       </c>
       <c r="D179" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
         </is>
       </c>
       <c r="E179" s="11" t="inlineStr">
@@ -12991,18 +12995,65 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="11" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C180" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D180" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E180" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F180" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G180" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H180" s="11" t="inlineStr"/>
+      <c r="I180" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J180" s="11" t="inlineStr"/>
+      <c r="K180" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K179"/>
-  <conditionalFormatting sqref="K2:K179">
+  <autoFilter ref="A1:K180"/>
+  <conditionalFormatting sqref="K2:K180">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: mark the 2026-10-22 review fixes done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -7729,7 +7729,7 @@
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>Publish firestore.rules again.</t>
+          <t>DONE ed64de3 (publish firestore.rules). Publish firestore.rules again.</t>
         </is>
       </c>
       <c r="I74" s="12" t="inlineStr">
@@ -7740,7 +7740,7 @@
       <c r="J74" s="11" t="inlineStr"/>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: no duplicate products (159), Stock Count rename and paper wording (160)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K180"/>
+  <dimension ref="A1:K182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7755,17 +7755,17 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Project Context (p.1)</t>
+          <t>REQ064 batch upload, Product Management module</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
+          <t>No duplicate products: batch import skips rows already in the catalog or repeated in the file (with 'Remove duplicates'); Add/Edit Product refuses an existing name; product codes (MED-) can never repeat</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="H75" s="11" t="inlineStr">
         <is>
-          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
+          <t>DONE f7fb34c. Client request 2026-10-24. Names compared ignoring capitals, spaces and punctuation.</t>
         </is>
       </c>
       <c r="I75" s="11" t="inlineStr">
@@ -7806,12 +7806,12 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.24)</t>
+          <t>Project Context (p.1)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
+          <t>Says the old POS couldn't print batch numbers, expiration dates or supplier details on receipts. The new receipts don't show them either; add batch/expiry to receipts and reports, or soften the sentence.</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da: system now matches (BM-only finalize).</t>
+          <t>DONE Wholesale sales invoices, the Customer File report and Return/Exchange report carry batch + expiry per line; no paper change needed.</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
@@ -7857,12 +7857,12 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Output) (p.27)</t>
+          <t>Theoretical Framework (p.24)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
+          <t>'Only authorized branch managers can ... override automated inventory counts': needs the REQ061 fix (Branch Manager-only reconciliation finalize).</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
@@ -7882,7 +7882,7 @@
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>DONE footer links to legal.html on every page.</t>
+          <t>DONE 06574da: system now matches (BM-only finalize).</t>
         </is>
       </c>
       <c r="I77" s="11" t="inlineStr">
@@ -7903,17 +7903,17 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Modules: Staff roles (p.45-46)</t>
+          <t>Conceptual Framework (Output) (p.27)</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
+          <t>'Terms and Conditions remain available throughout the session': footer Privacy/Terms links are dead. Link them to the existing legal text.</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -7933,12 +7933,12 @@
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
+          <t>DONE footer links to legal.html on every page.</t>
         </is>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J78" s="11" t="inlineStr"/>
@@ -7954,22 +7954,22 @@
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>REQ001 registration, Scope and Limitations</t>
+          <t>Modules: Staff roles (p.45-46)</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>Phone number verification by SMS code: on hold (every SMS costs money; Amson doesn't want to spend)</t>
+          <t>Lists 'void authorization' for Branch Manager and Technical Staff: needs the void feature. 'Sales Staff: product catalog viewing only': see REQ121 decision.</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
@@ -7984,7 +7984,7 @@
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>Paper: state in Limitations (number format checked, not ownership) and in Recommendations (SMS OTP).</t>
+          <t>DONE 57f4d80: void built for BM/Technical; Sales Staff POS-only.</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
@@ -7995,7 +7995,7 @@
       <c r="J79" s="11" t="inlineStr"/>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8010,17 +8010,17 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Chapter 3 evaluation (Objective 4)</t>
+          <t>REQ001 registration, Scope and Limitations</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Evaluation survey questionnaires: Branch Manager, Technical Staff, Sales Staff and User forms, mapped to TAM + ISO/IEC 25010</t>
+          <t>Phone number verification by SMS code: on hold (every SMS costs money; Amson doesn't want to spend)</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>DONE Claude Docs, 2026-10-22. In Claude Docs ('Survey Questionnaires (Admin and User)'); maintainability covered by the developers' testing (no IT expert form).</t>
+          <t>Paper: state in Limitations (number format checked, not ownership) and in Recommendations (SMS OTP).</t>
         </is>
       </c>
       <c r="I80" s="11" t="inlineStr">
@@ -8046,7 +8046,7 @@
       <c r="J80" s="11" t="inlineStr"/>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -8061,17 +8061,17 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>REQ007 / Technical Background p.35-36</t>
+          <t>Chapter 3 evaluation (Objective 4)</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
+          <t>Evaluation survey questionnaires: Branch Manager, Technical Staff, Sales Staff and User forms, mapped to TAM + ISO/IEC 25010</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F81" s="11" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>DONE Claude Docs, 2026-10-22. In Claude Docs ('Survey Questionnaires (Admin and User)'); maintainability covered by the developers' testing (no IT expert form).</t>
         </is>
       </c>
       <c r="I81" s="11" t="inlineStr">
@@ -8097,7 +8097,7 @@
       <c r="J81" s="11" t="inlineStr"/>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>REQ008 p.47; Modules p.38</t>
+          <t>REQ007 / Technical Background p.35-36</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
+          <t>Password reset link is sent by Firebase Authentication, not EmailJS.</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -8140,9 +8140,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I82" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr"/>
@@ -8163,12 +8163,12 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>REQ031 p.50</t>
+          <t>REQ008 p.47; Modules p.38</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
+          <t>Drop 'promotions' unless you plan them; keep 'announcements' (banner to be built).</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
@@ -8214,12 +8214,12 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>REQ073 p.55</t>
+          <t>REQ031 p.50</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
+          <t>Replace status list with: Pending Verification, Payment Confirmed, Dispatched / Ready for Pick-up, Delivered, Received / Picked Up, On Hold (with type), Closed (Unresolved).</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -8242,9 +8242,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I84" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I84" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
@@ -8265,12 +8265,12 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
+          <t>REQ073 p.55</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
+          <t>Add 'and the stated reason' (client requirement, Interview 2) - after the reason field is built.</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
@@ -8316,12 +8316,12 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>REQ085, REQ087 p.57; Modules p.44</t>
+          <t>REQ083 p.56; Fig 2.6 text p.73; Fig 2.14 text p.89</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Default wholesale price per product, adjustable per order (C9).</t>
+          <t>Void applies to completed transactions, referencing the original receipt number (C4).</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -8344,9 +8344,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I86" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
@@ -8367,12 +8367,12 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
+          <t>REQ085, REQ087 p.57; Modules p.44</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
+          <t>Default wholesale price per product, adjustable per order (C9).</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
@@ -8418,12 +8418,12 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
+          <t>REQ095, REQ098 p.58-59; Fig 2.6 text p.74; Fig 2.11 text p.83</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
+          <t>Overpayment is approved and the excess is added to the customer's store credit; three hold types plus overpayment-approval (C2).</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
@@ -8446,9 +8446,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I88" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I88" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>REQ121 p.61</t>
+          <t>REQ105 p.60; Fig 2.4 text p.71; Modules p.39-40</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
+          <t>Delivered is set by staff (or automatically after 3 days); the customer's confirmation marks it Received (C1).</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
@@ -8520,12 +8520,12 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 text p.67</t>
+          <t>REQ121 p.61</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
+          <t>Only if you keep Sales Staff access to Walk-in Orders history: add it to REQ121.</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -8571,12 +8571,12 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 diagram</t>
+          <t>Fig 2.2 text p.67</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
+          <t>Audit log is available to Technical Staff and Branch Manager (C6).</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
@@ -8622,12 +8622,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.5 text p.72</t>
+          <t>Fig 2.2 diagram</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
+          <t>Connect 'Manage Live Chat' to Technical Staff; add missing bubbles or label as summary (C11); one name for the pre-order use case (C12).</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -8673,12 +8673,12 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.2 / 2.7 diagrams</t>
+          <t>Fig 2.5 text p.72</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
+          <t>Technical Staff opens/counts; Branch Manager finalizes (C5).</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
@@ -8724,12 +8724,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.8 diagram + text p.76-77</t>
+          <t>Fig 2.2 / 2.7 diagrams</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
+          <t>Overpayment, free-of-cost distribution: no bubble anywhere; add 'Record Free-of-Cost Distribution' under Manage Wholesale Accounts if REQ091 stays.</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -8775,12 +8775,12 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.9 diagram + text p.78-79</t>
+          <t>Fig 2.8 diagram + text p.76-77</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
+          <t>Add reCAPTCHA, locked-account check, deactivated-account check, unverified-email redirect; make the wrong-OTP path match the text (C13).</t>
         </is>
       </c>
       <c r="E95" s="11" t="inlineStr">
@@ -8826,12 +8826,12 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.10 diagram</t>
+          <t>Fig 2.9 diagram + text p.78-79</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
+          <t>Terms accepted before submit, duplicate email caught at account creation (C14); add Resend Code; end at the shop, signed in (C10).</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
@@ -8877,12 +8877,12 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Fig 2.11 diagram + text p.82-83</t>
+          <t>Fig 2.10 diagram</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
+          <t>Move the RX decision to the start of checkout; RX skips the address; add Upload Prescription Photo (C15); optionally add delivery schedule and store credit.</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
@@ -8928,17 +8928,17 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Title page / cover (i)</t>
+          <t>Fig 2.11 diagram + text p.82-83</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
+          <t>Prescription approval/rejection before confirmation (C3, after it is built); RX skips courier steps (C17); resolved holds return to admin review (C18); stock shortage -&gt; Out of Stock hold (C19); overpayment approved with credit (C2); expired holds closed by the System lane, credit kept.</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -8951,7 +8951,11 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="H98" s="11" t="inlineStr"/>
+      <c r="H98" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I98" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -8975,12 +8979,12 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Title page / cover (i)</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
+          <t>Still labelled 'Capstone Project Proposal' dated May 16, 2026; update the label and date for the final manuscript.</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
@@ -8990,7 +8994,7 @@
       </c>
       <c r="F99" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G99" s="11" t="inlineStr">
@@ -9022,12 +9026,12 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Comparative Analysis (p.18)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
+          <t>About 100 'will ...' sentences are written as a proposal. Ask the adviser whether the final manuscript should switch to past/present tense, then convert.</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
@@ -9037,7 +9041,7 @@
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G100" s="11" t="inlineStr">
@@ -9069,12 +9073,12 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Conceptual Framework (Input) (p.25)</t>
+          <t>Comparative Analysis (p.18)</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
+          <t>The three compared systems are named but not cited in that section: J1TEK = Binag et al. (2024), Online Transporter = Llorente et al. (2022), Bandung FEFO = Malasari &amp; Sudrajat (2023). Binag and Llorente are in the reference list but cited nowhere in the text.</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
@@ -9093,9 +9097,9 @@
         </is>
       </c>
       <c r="H101" s="11" t="inlineStr"/>
-      <c r="I101" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J101" s="11" t="inlineStr"/>
@@ -9116,12 +9120,12 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.30-35)</t>
+          <t>Conceptual Framework (Input) (p.25)</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
+          <t>Says wholesale buyers' info is captured during account registration and that wholesale purchase orders are submitted through the platform. Wholesale buyers don't register or order online; staff record them.</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
@@ -9140,9 +9144,9 @@
         </is>
       </c>
       <c r="H102" s="11" t="inlineStr"/>
-      <c r="I102" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I102" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J102" s="11" t="inlineStr"/>
@@ -9163,12 +9167,12 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.96-98)</t>
+          <t>Methodology: sprint plan (p.30-35)</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
+          <t>Phases promise features that aren't built (device OTP, notifications by email, thermal printing, live chat, reports). Align with final decisions.</t>
         </is>
       </c>
       <c r="E103" s="11" t="inlineStr">
@@ -9215,7 +9219,7 @@
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
+          <t>Lists a 'Fifth Interview', but the appendices only have four transcripts (J-M). Add the transcript and proof, or remove the row.</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
@@ -9252,22 +9256,22 @@
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Price list</t>
+          <t>Calendar of Activities (p.96-98)</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Two price-list items have no price: Zardip Duo 40/5 (Telmisartan + Amlodipine) and Zincbos (Zinc Sulfate syrup)</t>
+          <t>Month header has no year. Update the bars to actual dates. The webapp branch history starts 2026-08-31 (earlier work isn't in this git history), so the team needs to fill earlier dates.</t>
         </is>
       </c>
       <c r="E105" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F105" s="11" t="inlineStr">
@@ -9277,17 +9281,13 @@
       </c>
       <c r="G105" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H105" s="11" t="inlineStr">
-        <is>
-          <t>Left out of the upload files; add by hand once priced.</t>
-        </is>
-      </c>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="H105" s="11" t="inlineStr"/>
       <c r="I105" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J105" s="11" t="inlineStr"/>
@@ -9303,27 +9303,27 @@
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>REQ088</t>
+          <t>Price list</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Hide costing/wholesale prices from public reads</t>
+          <t>Two price-list items have no price: Zardip Duo 40/5 (Telmisartan + Amlodipine) and Zincbos (Zinc Sulfate syrup)</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F106" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G106" s="11" t="inlineStr">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>DECIDED (revised): build it to avoid a removal letter.</t>
+          <t>Left out of the upload files; add by hand once priced.</t>
         </is>
       </c>
       <c r="I106" s="11" t="inlineStr">
@@ -9359,17 +9359,17 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Interview 1</t>
+          <t>REQ088</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
+          <t>Hide costing/wholesale prices from public reads</t>
         </is>
       </c>
       <c r="E107" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F107" s="11" t="inlineStr">
@@ -9384,18 +9384,18 @@
       </c>
       <c r="H107" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
+          <t>DECIDED (revised): build it to avoid a removal letter.</t>
         </is>
       </c>
       <c r="I107" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J107" s="11" t="inlineStr"/>
       <c r="K107" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9410,12 +9410,12 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (CREDIT terms)</t>
+          <t>Interview 1</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Credit sales follow-up (who owes what, mark as paid)</t>
+          <t>Park/hold a walk-in sale ('keep') while serving the next customer</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
+          <t>DECIDED: future work. Client's current POS practice; not in the paper.</t>
         </is>
       </c>
       <c r="I108" s="11" t="inlineStr">
@@ -9461,12 +9461,12 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Report Formats sheet (daily Sales section)</t>
+          <t>Report Formats sheet (CREDIT terms)</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
+          <t>Credit sales follow-up (who owes what, mark as paid)</t>
         </is>
       </c>
       <c r="E109" s="11" t="inlineStr">
@@ -9476,7 +9476,7 @@
       </c>
       <c r="F109" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G109" s="11" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="H109" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
+          <t>DECIDED: future work. Not in the paper; ask the client if the main office tracks collections instead.</t>
         </is>
       </c>
       <c r="I109" s="11" t="inlineStr">
@@ -9507,22 +9507,22 @@
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Report Formats sheet (daily Sales section)</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
+          <t>Pay-in / pay-out (cash drawer in and out) recorded per day</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F110" s="11" t="inlineStr">
@@ -9537,18 +9537,18 @@
       </c>
       <c r="H110" s="11" t="inlineStr">
         <is>
-          <t>DONE chat is built; keep the sentence.</t>
+          <t>DECIDED: future work. Both were 0.00 on the sample day; ask if it's used.</t>
         </is>
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr"/>
       <c r="K110" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -9558,22 +9558,22 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>REQ013, REQ068</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>Dosage/usage notes field on products</t>
+          <t>States the AI assistant won't give medical advice: keep only if chat is built.</t>
         </is>
       </c>
       <c r="E111" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F111" s="11" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="H111" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE chat is built; keep the sentence.</t>
         </is>
       </c>
       <c r="I111" s="11" t="inlineStr">
@@ -9614,17 +9614,17 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>REQ049</t>
+          <t>REQ013, REQ068</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Supplier column in the inventory batch table</t>
+          <t>Dosage/usage notes field on products</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F112" s="11" t="inlineStr">
@@ -9665,12 +9665,12 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>REQ103, REQ107</t>
+          <t>REQ049</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
+          <t>Supplier column in the inventory batch table</t>
         </is>
       </c>
       <c r="E113" s="11" t="inlineStr">
@@ -9690,7 +9690,7 @@
       </c>
       <c r="H113" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I113" s="11" t="inlineStr">
@@ -9716,12 +9716,12 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>REQ116</t>
+          <t>REQ103, REQ107</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>Customer Accounts: list of the customer's orders</t>
+          <t>Delivery: 'copy all' including preferred schedule + order no.; internal delivery notes</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="H114" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 06574da. Use the notes for rider name/plate/number, which staff currently screenshot privately (Interviews 2-3).</t>
         </is>
       </c>
       <c r="I114" s="11" t="inlineStr">
@@ -9767,17 +9767,17 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ116</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
+          <t>Customer Accounts: list of the customer's orders</t>
         </is>
       </c>
       <c r="E115" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F115" s="11" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="H115" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I115" s="11" t="inlineStr">
@@ -9818,17 +9818,17 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>REQ070</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Category rename: replace native prompt() with app dialog</t>
+          <t>Staff creation uses shared validators; stop silent Administrator -&gt; Branch Manager change</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>Polish</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F116" s="11" t="inlineStr">
@@ -9843,7 +9843,7 @@
       </c>
       <c r="H116" s="11" t="inlineStr">
         <is>
-          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
+          <t>DONE 847c877. From the first review.</t>
         </is>
       </c>
       <c r="I116" s="11" t="inlineStr">
@@ -9869,17 +9869,17 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>REQ033, REQ093</t>
+          <t>REQ070</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
+          <t>Category rename: replace native prompt() with app dialog</t>
         </is>
       </c>
       <c r="E117" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Polish</t>
         </is>
       </c>
       <c r="F117" s="11" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="H117" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92. From the first review.</t>
+          <t>DONE category tools commit: rename uses the app dialog; deleting a category can move its products. From the first review.</t>
         </is>
       </c>
       <c r="I117" s="11" t="inlineStr">
@@ -9920,12 +9920,12 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>REQ099</t>
+          <t>REQ033, REQ093</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>'Payment not received' as its own hold type</t>
+          <t>Receipt only after verification; show subtotal/credit applied on PDF</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
@@ -9945,7 +9945,7 @@
       </c>
       <c r="H118" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 082ec92. From the first review.</t>
         </is>
       </c>
       <c r="I118" s="11" t="inlineStr">
@@ -9971,12 +9971,12 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>REQ026</t>
+          <t>REQ099</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>Checkout pick-up notice mentions bringing the original prescription</t>
+          <t>'Payment not received' as its own hold type</t>
         </is>
       </c>
       <c r="E119" s="11" t="inlineStr">
@@ -9996,7 +9996,7 @@
       </c>
       <c r="H119" s="11" t="inlineStr">
         <is>
-          <t>DONE 082ec92.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I119" s="11" t="inlineStr">
@@ -10022,12 +10022,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>REQ009</t>
+          <t>REQ026</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>Show quantity in stock on catalog cards</t>
+          <t>Checkout pick-up notice mentions bringing the original prescription</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="H120" s="11" t="inlineStr">
         <is>
-          <t>DONE 06574da.</t>
+          <t>DONE 082ec92.</t>
         </is>
       </c>
       <c r="I120" s="11" t="inlineStr">
@@ -10073,17 +10073,17 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>REQ040</t>
+          <t>REQ009</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>Profile picture in Account Settings</t>
+          <t>Show quantity in stock on catalog cards</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F121" s="11" t="inlineStr">
@@ -10098,7 +10098,7 @@
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3.</t>
+          <t>DONE 06574da.</t>
         </is>
       </c>
       <c r="I121" s="11" t="inlineStr">
@@ -10124,17 +10124,17 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>REQNF028</t>
+          <t>REQ040</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
+          <t>Profile picture in Account Settings</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F122" s="11" t="inlineStr">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="H122" s="11" t="inlineStr">
         <is>
-          <t>DONE 847c877.</t>
+          <t>DONE 77336f3.</t>
         </is>
       </c>
       <c r="I122" s="11" t="inlineStr">
@@ -10175,17 +10175,17 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>REQ047</t>
+          <t>REQNF028</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
+          <t>One date formatter (MM/DD/YYYY, 12-hour) across all screens</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F123" s="11" t="inlineStr">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="H123" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
+          <t>DONE 847c877.</t>
         </is>
       </c>
       <c r="I123" s="11" t="inlineStr">
@@ -10226,17 +10226,17 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>REQNF017</t>
+          <t>REQ047</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>README with setup steps; fix the error message that points to it</t>
+          <t>Dashboard 'Active Online Orders' excludes delivered/closed</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F124" s="11" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="H124" s="11" t="inlineStr">
         <is>
-          <t>DONE 77336f3. From the first review.</t>
+          <t>DONE d9fc96b: counts verified + dispatched only. From the first review.</t>
         </is>
       </c>
       <c r="I124" s="11" t="inlineStr">
@@ -10277,17 +10277,17 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>REQ001</t>
+          <t>REQNF017</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>Normalize phone number at registration</t>
+          <t>README with setup steps; fix the error message that points to it</t>
         </is>
       </c>
       <c r="E125" s="11" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F125" s="11" t="inlineStr">
@@ -10302,7 +10302,7 @@
       </c>
       <c r="H125" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b. From the first review.</t>
+          <t>DONE 77336f3. From the first review.</t>
         </is>
       </c>
       <c r="I125" s="11" t="inlineStr">
@@ -10328,17 +10328,17 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>REQ008; Interview 1</t>
+          <t>REQ001</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
+          <t>Normalize phone number at registration</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="F126" s="11" t="inlineStr">
@@ -10353,7 +10353,7 @@
       </c>
       <c r="H126" s="11" t="inlineStr">
         <is>
-          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
+          <t>DONE d9fc96b. From the first review.</t>
         </is>
       </c>
       <c r="I126" s="11" t="inlineStr">
@@ -10379,17 +10379,17 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>REQ031</t>
+          <t>REQ008; Interview 1</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr">
         <is>
-          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
+          <t>Store announcements + promotions banner, editable by staff (e.g. closure days)</t>
         </is>
       </c>
       <c r="E127" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F127" s="11" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="H127" s="11" t="inlineStr">
         <is>
-          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
+          <t>DONE Settings -&gt; Store Announcement; shown under the header on shop pages.</t>
         </is>
       </c>
       <c r="I127" s="11" t="inlineStr">
@@ -10430,17 +10430,17 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37</t>
+          <t>REQ031</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
+          <t>Show invalid-payment holds to customers as 'Payment Rejected - re-upload needed'</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F128" s="11" t="inlineStr">
@@ -10455,18 +10455,18 @@
       </c>
       <c r="H128" s="11" t="inlineStr">
         <is>
-          <t>Built (stock in vs out), then removed at the team's request 2026-10-21 - see the Removals sheet. Keeps the Chart.js claim (no letter).</t>
+          <t>DONE d9fc96b: customer badges show Payment Rejected / Balance Due / Out of Stock / Prescription Rejected. Keeps the paper's status name (no letter).</t>
         </is>
       </c>
       <c r="I128" s="11" t="inlineStr">
         <is>
-          <t>None (not in paper)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J128" s="11" t="inlineStr"/>
       <c r="K128" s="11" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10481,12 +10481,12 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Modules p.42</t>
+          <t>Technical Background p.35-37</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">
         <is>
-          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
+          <t>Inventory movement chart on the dashboard (stock in/out over the period)</t>
         </is>
       </c>
       <c r="E129" s="11" t="inlineStr">
@@ -10506,18 +10506,18 @@
       </c>
       <c r="H129" s="11" t="inlineStr">
         <is>
-          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
+          <t>Built (stock in vs out), then removed at the team's request 2026-10-21 - see the Removals sheet. Keeps the Chart.js claim (no letter).</t>
         </is>
       </c>
       <c r="I129" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None (not in paper)</t>
         </is>
       </c>
       <c r="J129" s="11" t="inlineStr"/>
       <c r="K129" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -10532,12 +10532,12 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework p.23</t>
+          <t>Modules p.42</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
+          <t>Price lock/unlock toggle per product (Branch Manager only)</t>
         </is>
       </c>
       <c r="E130" s="11" t="inlineStr">
@@ -10557,7 +10557,7 @@
       </c>
       <c r="H130" s="11" t="inlineStr">
         <is>
-          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
+          <t>DONE Lock/Unlock prices button for the Branch Manager in Edit Product. Keeps 'price locking' (no letter).</t>
         </is>
       </c>
       <c r="I130" s="11" t="inlineStr">
@@ -10583,12 +10583,12 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>REQ039, Fig 2.10, C16</t>
+          <t>Theoretical Framework p.23</t>
         </is>
       </c>
       <c r="D131" s="11" t="inlineStr">
         <is>
-          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
+          <t>Browser notifications for staff alerts (new order, pending payment, expiry, low stock)</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="H131" s="11" t="inlineStr">
         <is>
-          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
+          <t>DONE Notifications -&gt; Turn on desktop alerts; each new alert pops up once. Keeps the 'push notifications' claim (no letter).</t>
         </is>
       </c>
       <c r="I131" s="11" t="inlineStr">
@@ -10634,17 +10634,17 @@
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>REQ004</t>
+          <t>REQ039, Fig 2.10, C16</t>
         </is>
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
+          <t>Order-placed notification in the customer's bell (no database rule change needed if derived from order status)</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F132" s="11" t="inlineStr">
@@ -10659,7 +10659,7 @@
       </c>
       <c r="H132" s="11" t="inlineStr">
         <is>
-          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
+          <t>DONE written at checkout (rule allows only the customer's own 'order_placed' notice).</t>
         </is>
       </c>
       <c r="I132" s="11" t="inlineStr">
@@ -10670,7 +10670,7 @@
       <c r="J132" s="11" t="inlineStr"/>
       <c r="K132" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -10685,17 +10685,17 @@
       </c>
       <c r="C133" s="11" t="inlineStr">
         <is>
-          <t>Inventory module</t>
+          <t>REQ004</t>
         </is>
       </c>
       <c r="D133" s="11" t="inlineStr">
         <is>
-          <t>Inventory list: drop the 'Never received' placeholder rows</t>
+          <t>Login lockout counter can be reset by anyone (public loginAttempts collection)</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F133" s="11" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="H133" s="11" t="inlineStr">
         <is>
-          <t>DONE 66b8b2e. Products never stocked no longer show as empty batch rows.</t>
+          <t>Lockout works for normal use; a determined attacker could clear it. Mention as a limitation if not fixed.</t>
         </is>
       </c>
       <c r="I133" s="11" t="inlineStr">
@@ -10721,7 +10721,7 @@
       <c r="J133" s="11" t="inlineStr"/>
       <c r="K133" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -10736,12 +10736,12 @@
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>REQ001 registration validation</t>
+          <t>Inventory module</t>
         </is>
       </c>
       <c r="D134" s="11" t="inlineStr">
         <is>
-          <t>Name fields allow periods and dashes (Ma. Clara, Juan P. Cruz, Jr., Anne-Marie)</t>
+          <t>Inventory list: drop the 'Never received' placeholder rows</t>
         </is>
       </c>
       <c r="E134" s="11" t="inlineStr">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="H134" s="11" t="inlineStr">
         <is>
-          <t>DONE 010449e, 8ce4aa0. Same rule on register, account settings, staff and admin settings.</t>
+          <t>DONE 66b8b2e. Products never stocked no longer show as empty batch rows.</t>
         </is>
       </c>
       <c r="I134" s="11" t="inlineStr">
@@ -10787,12 +10787,12 @@
       </c>
       <c r="C135" s="11" t="inlineStr">
         <is>
-          <t>Checkout module, REQ019</t>
+          <t>REQ001 registration validation</t>
         </is>
       </c>
       <c r="D135" s="11" t="inlineStr">
         <is>
-          <t>Checkout: Same Day Delivery wording and a notice that the Lalamove fee is paid to the rider</t>
+          <t>Name fields allow periods and dashes (Ma. Clara, Juan P. Cruz, Jr., Anne-Marie)</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="H135" s="11" t="inlineStr">
         <is>
-          <t>DONE 010449e.</t>
+          <t>DONE 010449e, 8ce4aa0. Same rule on register, account settings, staff and admin settings.</t>
         </is>
       </c>
       <c r="I135" s="11" t="inlineStr">
@@ -10838,12 +10838,12 @@
       </c>
       <c r="C136" s="11" t="inlineStr">
         <is>
-          <t>EmailJS (Technical Background)</t>
+          <t>Checkout module, REQ019</t>
         </is>
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>Settings: Email Test button that shows EmailJS's reply</t>
+          <t>Checkout: Same Day Delivery wording and a notice that the Lalamove fee is paid to the rider</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="H136" s="11" t="inlineStr">
         <is>
-          <t>DONE 4eca895. Found the order template was missing To Email {{to_email}} - set it in the EmailJS dashboard before go-live.</t>
+          <t>DONE 010449e.</t>
         </is>
       </c>
       <c r="I136" s="11" t="inlineStr">
@@ -10889,12 +10889,12 @@
       </c>
       <c r="C137" s="11" t="inlineStr">
         <is>
-          <t>Shopping cart module</t>
+          <t>EmailJS (Technical Background)</t>
         </is>
       </c>
       <c r="D137" s="11" t="inlineStr">
         <is>
-          <t>Cart page: 'You May Also Like' product suggestions under the cart items</t>
+          <t>Settings: Email Test button that shows EmailJS's reply</t>
         </is>
       </c>
       <c r="E137" s="11" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="H137" s="11" t="inlineStr">
         <is>
-          <t>DONE 1581610. Team request 2026-10-21 (like Shopee).</t>
+          <t>DONE 4eca895. Found the order template was missing To Email {{to_email}} - set it in the EmailJS dashboard before go-live.</t>
         </is>
       </c>
       <c r="I137" s="11" t="inlineStr">
@@ -10940,12 +10940,12 @@
       </c>
       <c r="C138" s="11" t="inlineStr">
         <is>
-          <t>Notification module</t>
+          <t>Shopping cart module</t>
         </is>
       </c>
       <c r="D138" s="11" t="inlineStr">
         <is>
-          <t>Notifications: filter by Orders / Stock / Live Chat, newest first, mark read per filter</t>
+          <t>Cart page: 'You May Also Like' product suggestions under the cart items</t>
         </is>
       </c>
       <c r="E138" s="11" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="H138" s="11" t="inlineStr">
         <is>
-          <t>DONE 1581610. Team request 2026-10-21.</t>
+          <t>DONE 1581610. Team request 2026-10-21 (like Shopee).</t>
         </is>
       </c>
       <c r="I138" s="11" t="inlineStr">
@@ -10991,12 +10991,12 @@
       </c>
       <c r="C139" s="11" t="inlineStr">
         <is>
-          <t>Inventory module</t>
+          <t>Notification module</t>
         </is>
       </c>
       <c r="D139" s="11" t="inlineStr">
         <is>
-          <t>Inventory: 'Quantity' renamed to 'Available Inventory' (table and export)</t>
+          <t>Notifications: filter by Orders / Stock / Live Chat, newest first, mark read per filter</t>
         </is>
       </c>
       <c r="E139" s="11" t="inlineStr">
@@ -11042,12 +11042,12 @@
       </c>
       <c r="C140" s="11" t="inlineStr">
         <is>
-          <t>All PDF exports</t>
+          <t>Inventory module</t>
         </is>
       </c>
       <c r="D140" s="11" t="inlineStr">
         <is>
-          <t>PDFs printed the peso sign as a broken character - now 'PHP'</t>
+          <t>Inventory: 'Quantity' renamed to 'Available Inventory' (table and export)</t>
         </is>
       </c>
       <c r="E140" s="11" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="H140" s="11" t="inlineStr">
         <is>
-          <t>DONE a3f410b. jsPDF's built-in fonts have no peso sign.</t>
+          <t>DONE 1581610. Team request 2026-10-21.</t>
         </is>
       </c>
       <c r="I140" s="11" t="inlineStr">
@@ -11093,12 +11093,12 @@
       </c>
       <c r="C141" s="11" t="inlineStr">
         <is>
-          <t>Online order module</t>
+          <t>All PDF exports</t>
         </is>
       </c>
       <c r="D141" s="11" t="inlineStr">
         <is>
-          <t>Online Orders: Reference No. and SI No. columns (searchable); order date and time shown in Payment Verification</t>
+          <t>PDFs printed the peso sign as a broken character - now 'PHP'</t>
         </is>
       </c>
       <c r="E141" s="11" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="H141" s="11" t="inlineStr">
         <is>
-          <t>DONE 2a52561, 8d5a42e. Team request 2026-10-21.</t>
+          <t>DONE a3f410b. jsPDF's built-in fonts have no peso sign.</t>
         </is>
       </c>
       <c r="I141" s="11" t="inlineStr">
@@ -11144,12 +11144,12 @@
       </c>
       <c r="C142" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module, Reports module</t>
+          <t>Online order module</t>
         </is>
       </c>
       <c r="D142" s="11" t="inlineStr">
         <is>
-          <t>Reports moved out of the Orders tab: all reports open from the dashboard Reports panel</t>
+          <t>Online Orders: Reference No. and SI No. columns (searchable); order date and time shown in Payment Verification</t>
         </is>
       </c>
       <c r="E142" s="11" t="inlineStr">
@@ -11169,7 +11169,7 @@
       </c>
       <c r="H142" s="11" t="inlineStr">
         <is>
-          <t>DONE 2a52561. Team request 2026-10-21. Paper: if the Orders module text mentions an export there, point it to Reports.</t>
+          <t>DONE 2a52561, 8d5a42e. Team request 2026-10-21.</t>
         </is>
       </c>
       <c r="I142" s="11" t="inlineStr">
@@ -11195,12 +11195,12 @@
       </c>
       <c r="C143" s="11" t="inlineStr">
         <is>
-          <t>Dashboard module, sequential SI</t>
+          <t>Dashboard module, Reports module</t>
         </is>
       </c>
       <c r="D143" s="11" t="inlineStr">
         <is>
-          <t>Dashboard: Find a Sale by SI No. (walk-in, online and wholesale)</t>
+          <t>Reports moved out of the Orders tab: all reports open from the dashboard Reports panel</t>
         </is>
       </c>
       <c r="E143" s="11" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="H143" s="11" t="inlineStr">
         <is>
-          <t>DONE 8d5a42e. Every sale gets an SI No.; online orders keep their order/reference numbers too.</t>
+          <t>DONE 2a52561. Team request 2026-10-21. Paper: if the Orders module text mentions an export there, point it to Reports.</t>
         </is>
       </c>
       <c r="I143" s="11" t="inlineStr">
@@ -11246,12 +11246,12 @@
       </c>
       <c r="C144" s="11" t="inlineStr">
         <is>
-          <t>Go-live</t>
+          <t>Dashboard module, sequential SI</t>
         </is>
       </c>
       <c r="D144" s="11" t="inlineStr">
         <is>
-          <t>Temporary Clear Test Data page (Branch Manager / Administrator) and its delete rule; both switch off 2026-11-15</t>
+          <t>Dashboard: Find a Sale by SI No. (walk-in, online and wholesale)</t>
         </is>
       </c>
       <c r="E144" s="11" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="H144" s="11" t="inlineStr">
         <is>
-          <t>DONE 77fdd25, 112ce91 (publish firestore.rules to use it). Remove the page, its Settings card and the TEMPORARY rule block after go-live; not part of the paper.</t>
+          <t>DONE 8d5a42e. Every sale gets an SI No.; online orders keep their order/reference numbers too.</t>
         </is>
       </c>
       <c r="I144" s="11" t="inlineStr">
@@ -11297,17 +11297,17 @@
       </c>
       <c r="C145" s="11" t="inlineStr">
         <is>
-          <t>Tech Stack (free plans), REQNF013</t>
+          <t>Go-live</t>
         </is>
       </c>
       <c r="D145" s="11" t="inlineStr">
         <is>
-          <t>Watch Firestore usage after go-live: Dashboard and Reports still read the full sales history on each visit</t>
+          <t>Temporary Clear Test Data page (Branch Manager / Administrator) and its delete rule; both switch off 2026-11-15</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F145" s="11" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="H145" s="11" t="inlineStr">
         <is>
-          <t>Fine at one branch's volume; if the 50,000 reads/day limit gets close, limit them to the chosen period.</t>
+          <t>DONE 77fdd25, 112ce91 (publish firestore.rules to use it). Remove the page, its Settings card and the TEMPORARY rule block after go-live; not part of the paper.</t>
         </is>
       </c>
       <c r="I145" s="11" t="inlineStr">
@@ -11333,7 +11333,7 @@
       <c r="J145" s="11" t="inlineStr"/>
       <c r="K145" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11348,17 +11348,17 @@
       </c>
       <c r="C146" s="11" t="inlineStr">
         <is>
-          <t>Report Formats (Supplier Purchases, Monthly Inventory), Scope p.6</t>
+          <t>Tech Stack (free plans), REQNF013</t>
         </is>
       </c>
       <c r="D146" s="11" t="inlineStr">
         <is>
-          <t>No grocery / non-medical items (client, 2026-10-22): Grocery removed from the default categories; Supplier Purchases is one sheet</t>
+          <t>Watch Firestore usage after go-live: Dashboard and Reports still read the full sales history on each visit</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Missing</t>
         </is>
       </c>
       <c r="F146" s="11" t="inlineStr">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="H146" s="11" t="inlineStr">
         <is>
-          <t>DONE 19118db. Delete a 'Grocery' category already in Firebase via Manage Categories.</t>
+          <t>Fine at one branch's volume; if the 50,000 reads/day limit gets close, limit them to the chosen period.</t>
         </is>
       </c>
       <c r="I146" s="11" t="inlineStr">
@@ -11384,7 +11384,7 @@
       <c r="J146" s="11" t="inlineStr"/>
       <c r="K146" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -11399,12 +11399,12 @@
       </c>
       <c r="C147" s="11" t="inlineStr">
         <is>
-          <t>Report Formats, Scope p.6</t>
+          <t>Report Formats (Supplier Purchases, Monthly Inventory), Scope p.6</t>
         </is>
       </c>
       <c r="D147" s="11" t="inlineStr">
         <is>
-          <t>Categories confirmed from Amson's own files: price list = Generics + Medical Supplies; month-end report also has Branded and Drugstore (Per Piece); no Grocery</t>
+          <t>No grocery / non-medical items (client, 2026-10-22): Grocery removed from the default categories; Supplier Purchases is one sheet</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="H147" s="11" t="inlineStr">
         <is>
-          <t>DONE no code change needed beyond 19118db. System defaults match; per-piece items in the price list are medical supplies and stay there.</t>
+          <t>DONE 19118db. Delete a 'Grocery' category already in Firebase via Manage Categories.</t>
         </is>
       </c>
       <c r="I147" s="11" t="inlineStr">
@@ -11450,12 +11450,12 @@
       </c>
       <c r="C148" s="11" t="inlineStr">
         <is>
-          <t>REQ064 batch upload, Product Management module</t>
+          <t>Report Formats, Scope p.6</t>
         </is>
       </c>
       <c r="D148" s="11" t="inlineStr">
         <is>
-          <t>Bulk photo upload (Products &gt; Upload Photos): pick many photos at once, each matched to a product by its file name (brand, strength, form, or SKU), staff check/change every match, then all are shrunk, uploaded to Cloudinary and saved together; audit-logged</t>
+          <t>Categories confirmed from Amson's own files: price list = Generics + Medical Supplies; month-end report also has Branded and Drugstore (Per Piece); no Grocery</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
@@ -11475,7 +11475,7 @@
       </c>
       <c r="H148" s="11" t="inlineStr">
         <is>
-          <t>DONE 17d8caa. Branch Manager and Technical Staff (not Sales Staff). Ambiguous names (e.g. 'cetirizine.jpg' when there's a tablet and a syrup) are left for staff to choose; two photos for one product are blocked. Paper (optional): one sentence under REQ064 / Product Management.</t>
+          <t>DONE no code change needed beyond 19118db. System defaults match; per-piece items in the price list are medical supplies and stay there.</t>
         </is>
       </c>
       <c r="I148" s="11" t="inlineStr">
@@ -11501,12 +11501,12 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>REQ064 batch upload, Product Management module, REQNF usability</t>
+          <t>REQ064 batch upload, Product Management module</t>
         </is>
       </c>
       <c r="D149" s="11" t="inlineStr">
         <is>
-          <t>Products page UI: Upload Photos is a two-step modal (choose/drop photos with naming tips, then check matches with filters and a searchable product picker); progress and result pop-ups for photo saving and batch import (import result offers Add photos, failed rows kept for retry); batch import audit-logged</t>
+          <t>Bulk photo upload (Products &gt; Upload Photos): pick many photos at once, each matched to a product by its file name (brand, strength, form, or SKU), staff check/change every match, then all are shrunk, uploaded to Cloudinary and saved together; audit-logged</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H149" s="11" t="inlineStr">
         <is>
-          <t>DONE 93635fd. Client/team feedback 2026-10-23: it was hard to tell when an import had finished.</t>
+          <t>DONE 17d8caa. Branch Manager and Technical Staff (not Sales Staff). Ambiguous names (e.g. 'cetirizine.jpg' when there's a tablet and a syrup) are left for staff to choose; two photos for one product are blocked. Paper (optional): one sentence under REQ064 / Product Management.</t>
         </is>
       </c>
       <c r="I149" s="11" t="inlineStr">
@@ -11552,17 +11552,17 @@
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ064 batch upload, Product Management module, REQNF usability</t>
         </is>
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>Products page UI: Upload Photos is a two-step modal (choose/drop photos with naming tips, then check matches with filters and a searchable product picker); progress and result pop-ups for photo saving and batch import (import result offers Add photos, failed rows kept for retry); batch import audit-logged</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F150" s="11" t="inlineStr">
@@ -11575,7 +11575,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H150" s="11" t="inlineStr"/>
+      <c r="H150" s="11" t="inlineStr">
+        <is>
+          <t>DONE 93635fd. Client/team feedback 2026-10-23: it was hard to tell when an import had finished.</t>
+        </is>
+      </c>
       <c r="I150" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -11584,7 +11588,7 @@
       <c r="J150" s="11" t="inlineStr"/>
       <c r="K150" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11594,17 +11598,17 @@
       </c>
       <c r="B151" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D151" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
@@ -11625,7 +11629,7 @@
       <c r="H151" s="11" t="inlineStr"/>
       <c r="I151" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J151" s="11" t="inlineStr"/>
@@ -11641,27 +11645,27 @@
       </c>
       <c r="B152" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F152" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G152" s="11" t="inlineStr">
@@ -11669,11 +11673,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H152" s="11" t="inlineStr">
-        <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
-        </is>
-      </c>
+      <c r="H152" s="11" t="inlineStr"/>
       <c r="I152" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -11697,12 +11697,12 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>REQ090</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D153" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G153" s="11" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Rare; same-second exchanges on one line.</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I153" s="11" t="inlineStr">
@@ -11748,12 +11748,12 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
@@ -11773,7 +11773,7 @@
       </c>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>Needs a server function to clean up; note in the user manual.</t>
+          <t>Rare; same-second exchanges on one line.</t>
         </is>
       </c>
       <c r="I154" s="11" t="inlineStr">
@@ -11799,17 +11799,17 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D155" s="11" t="inlineStr">
         <is>
-          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F155" s="11" t="inlineStr">
@@ -11824,12 +11824,12 @@
       </c>
       <c r="H155" s="11" t="inlineStr">
         <is>
-          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
-        </is>
-      </c>
-      <c r="I155" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Needs a server function to clean up; note in the user manual.</t>
+        </is>
+      </c>
+      <c r="I155" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J155" s="11" t="inlineStr"/>
@@ -11850,17 +11850,17 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F156" s="11" t="inlineStr">
@@ -11875,12 +11875,12 @@
       </c>
       <c r="H156" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I156" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
+        </is>
+      </c>
+      <c r="I156" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr"/>
@@ -11901,17 +11901,17 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>REQ059-061, Fig 2.2 / 2.5 'Month-End Stock Reconciliation', Modules (Inventory), Theoretical Framework p.24</t>
         </is>
       </c>
       <c r="D157" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>'Stock Reconciliation' renamed 'Stock Count' on every screen, message and audit entry (new count numbers SC-YYYY-NN)</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F157" s="11" t="inlineStr">
@@ -11926,12 +11926,12 @@
       </c>
       <c r="H157" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
-        </is>
-      </c>
-      <c r="I157" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>System done 2026-10-24. Paper: rename to 'Stock Count' (or 'Month-End Stock Count') in REQ059-061, Fig 2.2 and 2.5 and the Modules text, or write 'stock count (reconciliation)' once. Wording only - no letter.</t>
+        </is>
+      </c>
+      <c r="I157" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J157" s="11" t="inlineStr"/>
@@ -11952,12 +11952,12 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="I158" s="11" t="inlineStr">
         <is>
-          <t>Adds</t>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J158" s="11" t="inlineStr"/>
@@ -12003,12 +12003,12 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D159" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
@@ -12031,9 +12031,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I159" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I159" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J159" s="11" t="inlineStr"/>
@@ -12054,12 +12054,12 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
@@ -12079,12 +12079,12 @@
       </c>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I160" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J160" s="11" t="inlineStr"/>
@@ -12105,17 +12105,17 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D161" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F161" s="11" t="inlineStr">
@@ -12128,10 +12128,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H161" s="11" t="inlineStr"/>
+      <c r="H161" s="11" t="inlineStr">
+        <is>
+          <t>See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I161" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J161" s="11" t="inlineStr"/>
@@ -12152,17 +12156,17 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F162" s="11" t="inlineStr">
@@ -12175,10 +12179,14 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H162" s="11" t="inlineStr"/>
-      <c r="I162" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H162" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
+      <c r="I162" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J162" s="11" t="inlineStr"/>
@@ -12199,12 +12207,12 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D163" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
@@ -12222,20 +12230,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H163" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
-      <c r="I163" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H163" s="11" t="inlineStr"/>
+      <c r="I163" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J163" s="11" t="inlineStr"/>
       <c r="K163" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12250,12 +12254,12 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -12274,9 +12278,9 @@
         </is>
       </c>
       <c r="H164" s="11" t="inlineStr"/>
-      <c r="I164" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I164" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J164" s="11" t="inlineStr"/>
@@ -12297,12 +12301,12 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D165" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
@@ -12320,16 +12324,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H165" s="11" t="inlineStr"/>
-      <c r="I165" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H165" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I165" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J165" s="11" t="inlineStr"/>
       <c r="K165" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12344,12 +12352,12 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -12368,9 +12376,9 @@
         </is>
       </c>
       <c r="H166" s="11" t="inlineStr"/>
-      <c r="I166" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I166" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J166" s="11" t="inlineStr"/>
@@ -12391,12 +12399,12 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D167" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
@@ -12415,9 +12423,9 @@
         </is>
       </c>
       <c r="H167" s="11" t="inlineStr"/>
-      <c r="I167" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I167" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J167" s="11" t="inlineStr"/>
@@ -12438,12 +12446,12 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D168" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
@@ -12485,12 +12493,12 @@
       </c>
       <c r="C169" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D169" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
@@ -12509,9 +12517,9 @@
         </is>
       </c>
       <c r="H169" s="11" t="inlineStr"/>
-      <c r="I169" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I169" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J169" s="11" t="inlineStr"/>
@@ -12532,12 +12540,12 @@
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
@@ -12556,9 +12564,9 @@
         </is>
       </c>
       <c r="H170" s="11" t="inlineStr"/>
-      <c r="I170" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="I170" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J170" s="11" t="inlineStr"/>
@@ -12579,12 +12587,12 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D171" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
@@ -12602,20 +12610,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H171" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I171" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H171" s="11" t="inlineStr"/>
+      <c r="I171" s="11" t="inlineStr">
+        <is>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J171" s="11" t="inlineStr"/>
       <c r="K171" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12630,12 +12634,12 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
@@ -12677,12 +12681,12 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D173" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
@@ -12700,16 +12704,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H173" s="11" t="inlineStr"/>
-      <c r="I173" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H173" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I173" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J173" s="11" t="inlineStr"/>
       <c r="K173" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12724,12 +12732,12 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
@@ -12771,12 +12779,12 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D175" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
@@ -12818,12 +12826,12 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
@@ -12865,12 +12873,12 @@
       </c>
       <c r="C177" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D177" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
@@ -12912,12 +12920,12 @@
       </c>
       <c r="C178" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D178" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
@@ -12959,12 +12967,12 @@
       </c>
       <c r="C179" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D179" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E179" s="11" t="inlineStr">
@@ -13006,12 +13014,12 @@
       </c>
       <c r="C180" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D180" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E180" s="11" t="inlineStr">
@@ -13042,18 +13050,112 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C181" s="11" t="inlineStr">
+        <is>
+          <t>Appendices (p.124)</t>
+        </is>
+      </c>
+      <c r="D181" s="11" t="inlineStr">
+        <is>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+        </is>
+      </c>
+      <c r="E181" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F181" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G181" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H181" s="11" t="inlineStr"/>
+      <c r="I181" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J181" s="11" t="inlineStr"/>
+      <c r="K181" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="11" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C182" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D182" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E182" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F182" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G182" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H182" s="11" t="inlineStr"/>
+      <c r="I182" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J182" s="11" t="inlineStr"/>
+      <c r="K182" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K180"/>
-  <conditionalFormatting sqref="K2:K180">
+  <autoFilter ref="A1:K182"/>
+  <conditionalFormatting sqref="K2:K182">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: view past stock counts (161)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To-Do'!$A$1:$K$183</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements'!$A$1:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Use Cases'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Activity Diagrams'!$A$1:$G$46</definedName>
@@ -3972,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K182"/>
+  <dimension ref="A1:K183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11603,17 +11603,17 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>System roles (-)</t>
+          <t>REQ059-061 stock count, Inventory module</t>
         </is>
       </c>
       <c r="D151" s="11" t="inlineStr">
         <is>
-          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
+          <t>View past stock counts: each finished count opens with its month, who started/finalized it and when, totals (matched, differences, units short/over), the reason, every batch line, a Differences-only filter, search and PDF/Excel export</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
@@ -11626,7 +11626,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H151" s="11" t="inlineStr"/>
+      <c r="H151" s="11" t="inlineStr">
+        <is>
+          <t>DONE 2ceab34. Client request 2026-10-24.</t>
+        </is>
+      </c>
       <c r="I151" s="11" t="inlineStr">
         <is>
           <t>None</t>
@@ -11635,7 +11639,7 @@
       <c r="J151" s="11" t="inlineStr"/>
       <c r="K151" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11645,17 +11649,17 @@
       </c>
       <c r="B152" s="11" t="inlineStr">
         <is>
-          <t>System + paper</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>Whole paper + system (-)</t>
+          <t>System roles (-)</t>
         </is>
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
+          <t>The system also has a legacy 'Administrator' role that the paper never mentions. Hide it from the UI or document it.</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
@@ -11676,7 +11680,7 @@
       <c r="H152" s="11" t="inlineStr"/>
       <c r="I152" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J152" s="11" t="inlineStr"/>
@@ -11692,27 +11696,27 @@
       </c>
       <c r="B153" s="11" t="inlineStr">
         <is>
-          <t>Paper</t>
+          <t>System + paper</t>
         </is>
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>REQ005, REQ044</t>
+          <t>Whole paper + system (-)</t>
         </is>
       </c>
       <c r="D153" s="11" t="inlineStr">
         <is>
-          <t>New-device code is checked in the browser, not by the database rules</t>
+          <t>'QR PH' in the paper and most screens, 'QR Ph' on the payment page image text. The official name is 'QR Ph'; pick one everywhere.</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>Limitation</t>
+          <t>Manuscript pass</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G153" s="11" t="inlineStr">
@@ -11720,11 +11724,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H153" s="11" t="inlineStr">
-        <is>
-          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
-        </is>
-      </c>
+      <c r="H153" s="11" t="inlineStr"/>
       <c r="I153" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -11748,12 +11748,12 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>REQ090</t>
+          <t>REQ005, REQ044</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
+          <t>New-device code is checked in the browser, not by the database rules</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="F154" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G154" s="11" t="inlineStr">
@@ -11773,7 +11773,7 @@
       </c>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>Rare; same-second exchanges on one line.</t>
+          <t>Stops normal use of a stolen password; a technical attacker could skip it. State this in Limitations.</t>
         </is>
       </c>
       <c r="I154" s="11" t="inlineStr">
@@ -11799,12 +11799,12 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>REQ118</t>
+          <t>REQ090</t>
         </is>
       </c>
       <c r="D155" s="11" t="inlineStr">
         <is>
-          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
+          <t>Known, not fixed: two wholesale exchanges on the same order line at the same second can mix up which batch a later return goes back to (stock totals stay right)</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="H155" s="11" t="inlineStr">
         <is>
-          <t>Needs a server function to clean up; note in the user manual.</t>
+          <t>Rare; same-second exchanges on one line.</t>
         </is>
       </c>
       <c r="I155" s="11" t="inlineStr">
@@ -11850,17 +11850,17 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
+          <t>REQ118</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
+          <t>Known, not fixed: if creating a staff account fails after the login is made, the email can't be reused until the login is removed in the Firebase console</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="F156" s="11" t="inlineStr">
@@ -11875,12 +11875,12 @@
       </c>
       <c r="H156" s="11" t="inlineStr">
         <is>
-          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
-        </is>
-      </c>
-      <c r="I156" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+          <t>Needs a server function to clean up; note in the user manual.</t>
+        </is>
+      </c>
+      <c r="I156" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr"/>
@@ -11901,17 +11901,17 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>REQ059-061, Fig 2.2 / 2.5 'Month-End Stock Reconciliation', Modules (Inventory), Theoretical Framework p.24</t>
+          <t>Technical Background (Chart.js 'inventory movement data'), Dashboard module</t>
         </is>
       </c>
       <c r="D157" s="11" t="inlineStr">
         <is>
-          <t>'Stock Reconciliation' renamed 'Stock Count' on every screen, message and audit entry (new count numbers SC-YYYY-NN)</t>
+          <t>Inventory Movement chart removed from the dashboard at the team's request (2026-10-21)</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="F157" s="11" t="inlineStr">
@@ -11926,12 +11926,12 @@
       </c>
       <c r="H157" s="11" t="inlineStr">
         <is>
-          <t>System done 2026-10-24. Paper: rename to 'Stock Count' (or 'Month-End Stock Count') in REQ059-061, Fig 2.2 and 2.5 and the Modules text, or write 'stock count (reconciliation)' once. Wording only - no letter.</t>
-        </is>
-      </c>
-      <c r="I157" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+          <t>Paper: drop 'inventory movement data' from the Chart.js line, or note it in the panel letter; stock in/out is still in the Inventory page and reports.</t>
+        </is>
+      </c>
+      <c r="I157" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J157" s="11" t="inlineStr"/>
@@ -11952,17 +11952,17 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Modules FEFO p.41</t>
+          <t>REQ059-061, Fig 2.2 / 2.5 'Month-End Stock Reconciliation', Modules (Inventory), Theoretical Framework p.24</t>
         </is>
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>Add the 2-month Bad Order step (C7).</t>
+          <t>'Stock Reconciliation' renamed 'Stock Count' on every screen, message and audit entry (new count numbers SC-YYYY-NN)</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
         <is>
-          <t>Paper edit</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F158" s="11" t="inlineStr">
@@ -11977,7 +11977,7 @@
       </c>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>See Contradictions / Paper Edits</t>
+          <t>System done 2026-10-24. Paper: rename to 'Stock Count' (or 'Month-End Stock Count') in REQ059-061, Fig 2.2 and 2.5 and the Modules text, or write 'stock count (reconciliation)' once. Wording only - no letter.</t>
         </is>
       </c>
       <c r="I158" s="11" t="inlineStr">
@@ -12003,12 +12003,12 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Technical Background p.35-37; Budget p.99</t>
+          <t>Modules FEFO p.41</t>
         </is>
       </c>
       <c r="D159" s="11" t="inlineStr">
         <is>
-          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
+          <t>Add the 2-month Bad Order step (C7).</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
@@ -12031,9 +12031,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I159" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I159" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J159" s="11" t="inlineStr"/>
@@ -12054,12 +12054,12 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Scope p.6; Product Browsing REQ009</t>
+          <t>Technical Background p.35-37; Budget p.99</t>
         </is>
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
+          <t>Cloudinary instead of Firebase Storage; Choices.js added; DataTable removed; hosting per decision (Tech Stack sheet).</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
@@ -12082,9 +12082,9 @@
           <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
-      <c r="I160" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I160" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J160" s="11" t="inlineStr"/>
@@ -12105,12 +12105,12 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Scope and Limitations p.7</t>
+          <t>Scope p.6; Product Browsing REQ009</t>
         </is>
       </c>
       <c r="D161" s="11" t="inlineStr">
         <is>
-          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
+          <t>The client also sells medical supplies (grocery items are dropped, client 2026-10-22); the paper only mentions OTC/prescription medicines. Mention medical supplies.</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
@@ -12156,12 +12156,12 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Decision-dependent</t>
+          <t>Scope and Limitations p.7</t>
         </is>
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
+          <t>Add: system receipts/invoices are internal records, not BIR-registered official receipts; BIR/VAT receipts stay manual on request; no BIR or government integration (client policy, Interview 1).</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
@@ -12181,12 +12181,12 @@
       </c>
       <c r="H162" s="11" t="inlineStr">
         <is>
-          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+          <t>See Contradictions / Paper Edits</t>
         </is>
       </c>
       <c r="I162" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J162" s="11" t="inlineStr"/>
@@ -12207,17 +12207,17 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Whole paper (-)</t>
+          <t>Decision-dependent</t>
         </is>
       </c>
       <c r="D163" s="11" t="inlineStr">
         <is>
-          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
+          <t>Live chat/AI (Obj. 1, Scope, Framework, REQ035-038, REQ108-110, NF008, NF012); real-time refresh (NF005); hosting (NF013); wholesale price visibility (REQ088).</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
         <is>
-          <t>Manuscript pass</t>
+          <t>Paper edit</t>
         </is>
       </c>
       <c r="F163" s="11" t="inlineStr">
@@ -12230,7 +12230,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H163" s="11" t="inlineStr"/>
+      <c r="H163" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: build it on Gemini via Firebase AI Logic (free tier), swappable to Groq; FAQ answers without AI calls; staff handoff when the free limit is hit. Verify the project's limit in AI Studio first. See Contradictions / Paper Edits</t>
+        </is>
+      </c>
       <c r="I163" s="11" t="inlineStr">
         <is>
           <t>Corrects / rewords</t>
@@ -12254,12 +12258,12 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Scope (p.6)</t>
+          <t>Whole paper (-)</t>
         </is>
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
+          <t>Spelling consistency: 'Fulfilment' on the cover vs 'fulfillment' elsewhere.</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -12278,9 +12282,9 @@
         </is>
       </c>
       <c r="H164" s="11" t="inlineStr"/>
-      <c r="I164" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I164" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J164" s="11" t="inlineStr"/>
@@ -12301,12 +12305,12 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Theoretical Framework (p.22-23)</t>
+          <t>Scope (p.6)</t>
         </is>
       </c>
       <c r="D165" s="11" t="inlineStr">
         <is>
-          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
+          <t>'Intended to serve retail customers, wholesale clients, branch staff, and main office management': wholesale clients and the main office never log in. Reword to 'staff record wholesale transactions; reports are submitted to the main office'.</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
@@ -12324,11 +12328,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H165" s="11" t="inlineStr">
-        <is>
-          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
-        </is>
-      </c>
+      <c r="H165" s="11" t="inlineStr"/>
       <c r="I165" s="12" t="inlineStr">
         <is>
           <t>REMOVES / narrows - see Removals (Letter)</t>
@@ -12337,7 +12337,7 @@
       <c r="J165" s="11" t="inlineStr"/>
       <c r="K165" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12352,12 +12352,12 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Methodology: sprint plan (p.32)</t>
+          <t>Theoretical Framework (p.22-23)</t>
         </is>
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
+          <t>Mentions 'instantaneous push notifications for near-expiry supplies'; the system has an in-app notification bell, not push notifications. Reword.</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -12375,16 +12375,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H166" s="11" t="inlineStr"/>
-      <c r="I166" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H166" s="11" t="inlineStr">
+        <is>
+          <t>DONE Desktop alerts now built; wording can stay (or say 'desktop alerts').</t>
+        </is>
+      </c>
+      <c r="I166" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J166" s="11" t="inlineStr"/>
       <c r="K166" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12399,12 +12403,12 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35)</t>
+          <t>Methodology: sprint plan (p.32)</t>
         </is>
       </c>
       <c r="D167" s="11" t="inlineStr">
         <is>
-          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
+          <t>Phase 4 (customer side) lists the 'one-click copy feature for delivery details' under My Orders; that's an admin Delivery feature (also listed in Phase 6). Remove it from Phase 4.</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
@@ -12446,12 +12450,12 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35-36)</t>
+          <t>Technical Background (p.35)</t>
         </is>
       </c>
       <c r="D168" s="11" t="inlineStr">
         <is>
-          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
+          <t>Say 'Cloud Firestore' instead of 'real-time database', and Cloudinary instead of Firebase cloud storage for images.</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
@@ -12470,9 +12474,9 @@
         </is>
       </c>
       <c r="H168" s="11" t="inlineStr"/>
-      <c r="I168" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="I168" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J168" s="11" t="inlineStr"/>
@@ -12498,7 +12502,7 @@
       </c>
       <c r="D169" s="11" t="inlineStr">
         <is>
-          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
+          <t>EmailJS listed for order confirmations and password reset links: password reset is Firebase Auth; order emails depend on REQ039.</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
@@ -12540,12 +12544,12 @@
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Technical Background (p.35, 37)</t>
+          <t>Technical Background (p.35-36)</t>
         </is>
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
+          <t>Chart.js listed for 'inventory movement data': dashboard charts are sales only (inventory uses count tiles). Reword or add an inventory chart.</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
@@ -12587,12 +12591,12 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.36-38)</t>
+          <t>Technical Background (p.35, 37)</t>
         </is>
       </c>
       <c r="D171" s="11" t="inlineStr">
         <is>
-          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
+          <t>DataTable listed; tables are custom-built. Remove or reword.</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
@@ -12611,9 +12615,9 @@
         </is>
       </c>
       <c r="H171" s="11" t="inlineStr"/>
-      <c r="I171" s="11" t="inlineStr">
-        <is>
-          <t>Adds</t>
+      <c r="I171" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J171" s="11" t="inlineStr"/>
@@ -12634,12 +12638,12 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Technical Background: Software (p.38)</t>
+          <t>Technical Background: Software (p.36-38)</t>
         </is>
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
+          <t>Missing tools actually used: Cloudinary (images), Choices.js (searchable dropdowns), Bootstrap Icons, Google Fonts (Roboto), Git/GitHub (version control), Node.js http-server (local serving).</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
@@ -12660,7 +12664,7 @@
       <c r="H172" s="11" t="inlineStr"/>
       <c r="I172" s="11" t="inlineStr">
         <is>
-          <t>Corrects / rewords</t>
+          <t>Adds</t>
         </is>
       </c>
       <c r="J172" s="11" t="inlineStr"/>
@@ -12681,12 +12685,12 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Modules: Price Management (p.42)</t>
+          <t>Technical Background: Software (p.38)</t>
         </is>
       </c>
       <c r="D173" s="11" t="inlineStr">
         <is>
-          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
+          <t>Canva is listed for mockups, but the Gantt chart says 'Creation of Figma'. Use one tool name.</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
@@ -12704,20 +12708,16 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H173" s="11" t="inlineStr">
-        <is>
-          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
-        </is>
-      </c>
-      <c r="I173" s="12" t="inlineStr">
-        <is>
-          <t>REMOVES / narrows - see Removals (Letter)</t>
+      <c r="H173" s="11" t="inlineStr"/>
+      <c r="I173" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
         </is>
       </c>
       <c r="J173" s="11" t="inlineStr"/>
       <c r="K173" s="11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -12732,12 +12732,12 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
+          <t>Modules: Price Management (p.42)</t>
         </is>
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
+          <t>'Allows price locking': the lock is the Branch Manager-only rule (no separate lock switch). Reword, or add a lock toggle.</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
@@ -12755,16 +12755,20 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H174" s="11" t="inlineStr"/>
-      <c r="I174" s="11" t="inlineStr">
-        <is>
-          <t>Corrects / rewords</t>
+      <c r="H174" s="11" t="inlineStr">
+        <is>
+          <t>DONE No paper change needed: the Branch Manager has a Lock/Unlock prices toggle per product.</t>
+        </is>
+      </c>
+      <c r="I174" s="12" t="inlineStr">
+        <is>
+          <t>REMOVES / narrows - see Removals (Letter)</t>
         </is>
       </c>
       <c r="J174" s="11" t="inlineStr"/>
       <c r="K174" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12779,12 +12783,12 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>Calendar of Activities (p.97-98)</t>
+          <t>Wireframes (Figs 2.16-2.21) (p.92-95)</t>
         </is>
       </c>
       <c r="D175" s="11" t="inlineStr">
         <is>
-          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
+          <t>Not compared yet. Replace with real screenshots, or keep them labelled as early wireframes.</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
@@ -12826,12 +12830,12 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>Budgetary Estimate (p.99)</t>
+          <t>Calendar of Activities (p.97-98)</t>
         </is>
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
+          <t>Add rows for work actually done (POS, inventory, payment verification, wholesale, reports, testing) and mark 'System Deployment' per the hosting decision.</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
@@ -12878,7 +12882,7 @@
       </c>
       <c r="D177" s="11" t="inlineStr">
         <is>
-          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
+          <t>Total ₱31,790.08 checks out. Missing: Cloudinary (free), OpenAI API (pay-per-use, if chat is built), thermal printer (if printing is in scope).</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
@@ -12920,12 +12924,12 @@
       </c>
       <c r="C178" s="11" t="inlineStr">
         <is>
-          <t>References (p.100)</t>
+          <t>Budgetary Estimate (p.99)</t>
         </is>
       </c>
       <c r="D178" s="11" t="inlineStr">
         <is>
-          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
+          <t>Domain name ₱841.08 and Firebase Blaze ₱200: keep only if actually bought/used. Netlify is listed as free, but deployment was blocked by billing; make these consistent.</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
@@ -12967,12 +12971,12 @@
       </c>
       <c r="C179" s="11" t="inlineStr">
         <is>
-          <t>References (p.10 / refs)</t>
+          <t>References (p.100)</t>
         </is>
       </c>
       <c r="D179" s="11" t="inlineStr">
         <is>
-          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
+          <t>Davis reference is written 'Fred D. Davis. (1989)'; APA is 'Davis, F. D. (1989).'</t>
         </is>
       </c>
       <c r="E179" s="11" t="inlineStr">
@@ -13014,12 +13018,12 @@
       </c>
       <c r="C180" s="11" t="inlineStr">
         <is>
-          <t>References (p.17 / refs)</t>
+          <t>References (p.10 / refs)</t>
         </is>
       </c>
       <c r="D180" s="11" t="inlineStr">
         <is>
-          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
+          <t>'The Generics Pharmacy (TGP) Sumulong Case Study (2024)' is cited without an author; check the APA author/organization format.</t>
         </is>
       </c>
       <c r="E180" s="11" t="inlineStr">
@@ -13061,12 +13065,12 @@
       </c>
       <c r="C181" s="11" t="inlineStr">
         <is>
-          <t>Appendices (p.124)</t>
+          <t>References (p.17 / refs)</t>
         </is>
       </c>
       <c r="D181" s="11" t="inlineStr">
         <is>
-          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
+          <t>Sardjono et al. (2023) is described as an Agile-based study, but its listed title is about Track and Trace in Pharma 4.0. Verify the source matches the summary.</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
@@ -13108,12 +13112,12 @@
       </c>
       <c r="C182" s="11" t="inlineStr">
         <is>
-          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+          <t>Appendices (p.124)</t>
         </is>
       </c>
       <c r="D182" s="11" t="inlineStr">
         <is>
-          <t>Regenerate page numbers after all edits.</t>
+          <t>List of Appendices says 'PayMongo Pricing' / 'Lalamove API Instruction'; the appendix pages say 'PayMongo Pricing Limitation' / 'Lalamove API Limitation'. Match titles.</t>
         </is>
       </c>
       <c r="E182" s="11" t="inlineStr">
@@ -13144,18 +13148,65 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="11" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="11" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C183" s="11" t="inlineStr">
+        <is>
+          <t>Table of Contents / List of Figures (p.iv-vi)</t>
+        </is>
+      </c>
+      <c r="D183" s="11" t="inlineStr">
+        <is>
+          <t>Regenerate page numbers after all edits.</t>
+        </is>
+      </c>
+      <c r="E183" s="11" t="inlineStr">
+        <is>
+          <t>Manuscript pass</t>
+        </is>
+      </c>
+      <c r="F183" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G183" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H183" s="11" t="inlineStr"/>
+      <c r="I183" s="11" t="inlineStr">
+        <is>
+          <t>Corrects / rewords</t>
+        </is>
+      </c>
+      <c r="J183" s="11" t="inlineStr"/>
+      <c r="K183" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K182"/>
-  <conditionalFormatting sqref="K2:K182">
+  <autoFilter ref="A1:K183"/>
+  <conditionalFormatting sqref="K2:K183">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Client,Decision,System,System + paper,Paper"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Register: Sales Staff database rules done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hFpAbHof1mVo4HNKESie6
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -4995,7 +4995,7 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Pages already block Sales Staff; someone with technical know-how could still write other collections directly.</t>
+          <t>DONE 5223385: Sales Staff limited to POS, stock, counters, audit entries, catalog and own account in the rules. Pages already block Sales Staff; someone with technical know-how could still write other collections directly.</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
@@ -5006,7 +5006,7 @@
       <c r="J20" s="11" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register + test plan: REQ047 and REQ098 were already fixed in 72e7361
Dashboard 'Active Online Orders' counts only payment confirmed and
dispatched orders (on load and live), and approving a resubmitted order
clears the old hold and notifies the customer. Notes and the expected
results of T11-02 and T13-19 now say so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBZf6oKSsJ7KuyzUF78Kfz
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -2415,7 +2415,7 @@
     <t xml:space="preserve">js/admin-dashboard.js:129</t>
   </si>
   <si>
-    <t xml:space="preserve">Exceeds paper (charts, period filter, out-of-stock). 'Active Online Orders' wrongly counts delivered and closed orders.</t>
+    <t xml:space="preserve">Exceeds paper (charts, period filter, out-of-stock). Fixed 72e7361: 'Active Online Orders' counts only payment confirmed + dispatched orders (on load and live). (was: also counted delivered and closed orders.)</t>
   </si>
   <si>
     <t xml:space="preserve">Count fix is one line.</t>
@@ -3036,7 +3036,7 @@
     <t xml:space="preserve">js/admin-online-orders.js:638</t>
   </si>
   <si>
-    <t xml:space="preserve">System approves overpaid orders immediately and adds the excess to store credit (no hold). Bug: on a resubmitted order the old hold is never cleared, so it gets stuck On Hold, and no 'Payment confirmed' notification is sent.</t>
+    <t xml:space="preserve">System approves overpaid orders immediately and adds the excess to store credit (no hold). Fixed 72e7361: approving a resubmitted order clears the old hold and sends the Payment confirmed notice. (was: old hold never cleared, order stuck On Hold, no notification.)</t>
   </si>
   <si>
     <t xml:space="preserve">The paper says hold everywhere (REQ095, REQ098, Fig 2.6 text, Fig 2.11 text and diagram); approve-and-credit is what the client agreed to in the Interview 4 walkthrough. Fix the bug and reword the paper (C2).</t>

</xml_diff>

<commit_message>
Daily Sales: show dates as MM/DD/YYYY; register: two stale rows
- The Daily Sales day column printed 10-24-2026; every other date uses
  MM/DD/YYYY (REQNF028).
- Register: Use Case 2.2 Login now Matches (device OTP built in 7ede9d4);
  Activity 2.12 six-month flag runs on every load, not only Inventory.

Checked against the Auth + Firestore emulators with the published rules:
every page per role, role redirects, POS sales (FEFO, cash, reference,
RX Verified, no out-of-stock or near-expiry sales), online order through
approval, underpayment hold -> resubmit -> approve, price and void rules,
dashboard tiles, 6-month and 2-month expiry rules, Daily Sales PDF/Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBZf6oKSsJ7KuyzUF78Kfz
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -3804,7 +3804,7 @@
     <t xml:space="preserve">REQ004-005, 043-045</t>
   </si>
   <si>
-    <t xml:space="preserve">No unrecognized-device OTP.</t>
+    <t xml:space="preserve">Device OTP built (7ede9d4). (was: No unrecognized-device OTP.)</t>
   </si>
   <si>
     <t xml:space="preserve">Update Account Settings</t>
@@ -4500,7 +4500,7 @@
     <t xml:space="preserve">Flag for pull-out -&gt; expiration alert -&gt; admin chooses Write Off or Reserve for Free-of-Cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Flagged automatically as Wholesale Only (only when Inventory opens) + alert; no pull-out action choice</t>
+    <t xml:space="preserve">Flagged automatically as Wholesale Only on every Inventory, Dashboard, POS and shop load (REQ066) + alert; no pull-out action choice</t>
   </si>
   <si>
     <t xml:space="preserve">REQ066 timing fix; 'Reserve for free-of-cost' could just be the Wholesale Only flag + REQ091.</t>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">COUNTIF('Use Cases'!D:D,"Matches")</f>
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">COUNTIF('Use Cases'!D:D,"Partial")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20767,7 +20767,7 @@
         <v>1250</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>1251</v>

</xml_diff>

<commit_message>
Netlify: publish only the website files
netlify.toml copies the pages, admin/, shop/, js/, css/, assets/ and
_headers into dist/ and publishes that, so docs/ (register, test plan),
README, firestore.rules and the .bat helpers are not downloadable from
the live site. Register: #34 hosting decided (Netlify), #42 email
verification kept as a code and moved to Limitations.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBZf6oKSsJ7KuyzUF78Kfz
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -522,7 +522,7 @@
     <t xml:space="preserve">Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
   </si>
   <si>
-    <t xml:space="preserve">DECIDED: Netlify (already set up).</t>
+    <t xml:space="preserve">DECIDED: Netlify. netlify.toml publishes only the site files (docs/ etc. stay private); connect repo branch webapp in Netlify, then add the Netlify domain to Firebase Authorized domains (#190).</t>
   </si>
   <si>
     <t xml:space="preserve">Report Formats sheet (Discount/Deductions columns); Interview 2</t>
@@ -591,7 +591,7 @@
     <t xml:space="preserve">Close the email-verification bypass (code readable by customer; customer can set emailVerified)</t>
   </si>
   <si>
-    <t xml:space="preserve">From the first review.</t>
+    <t xml:space="preserve">DECIDED 2026-10-25: keep the 6-digit code (a fix needs a server function or switching to a Firebase link). Add to Limitations: email verification is checked in the browser; a technically skilled user could bypass it. Orders still require staff-verified payment.</t>
   </si>
   <si>
     <t xml:space="preserve">REQ005, REQ044, Fig 2.3, Fig 2.8</t>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="B20" s="1" t="n">
         <f aca="false">COUNTIF('To-Do'!K:K,"Open")</f>
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="J43" s="12"/>
       <c r="K43" s="13" t="s">
-        <v>45</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Register: new-device codes turned off (REQ005, REQ044)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBZf6oKSsJ7KuyzUF78Kfz
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -1884,7 +1884,7 @@
     <t xml:space="preserve">js/device-trust.js; js/auth.js</t>
   </si>
   <si>
-    <t xml:space="preserve">Built (7ede9d4): new browser gets an emailed 6-digit code (10 min, 5 tries, resend after 60 s); recognized devices in Account Settings. Checked in the browser, not by database rules.</t>
+    <t xml:space="preserve">Built (7ede9d4) but turned off 2026-10-25 (team decision): REQUIRE_DEVICE_CODE = false in js/device-trust.js. Set to true to require the code again. Built (7ede9d4): new browser gets an emailed 6-digit code (10 min, 5 tries, resend after 60 s); recognized devices in Account Settings. Checked in the browser, not by database rules.</t>
   </si>
   <si>
     <t xml:space="preserve">Paper may add: the device check runs in the browser.</t>
@@ -2421,7 +2421,7 @@
     <t xml:space="preserve">js/device-trust.js; js/admin-header.js</t>
   </si>
   <si>
-    <t xml:space="preserve">Built with REQ005 (7ede9d4); admin pages send an unconfirmed device back to login.</t>
+    <t xml:space="preserve">Built (7ede9d4) but turned off 2026-10-25 (team decision): REQUIRE_DEVICE_CODE = false in js/device-trust.js. Set to true to require the code again. Built with REQ005 (7ede9d4); admin pages send an unconfirmed device back to login.</t>
   </si>
   <si>
     <t xml:space="preserve">p.51; Fig 2.8</t>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">COUNTIF(Requirements!D:D,"Matches")</f>
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">COUNTIF('Use Cases'!D:D,"Matches")</f>
@@ -6723,7 +6723,7 @@
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">COUNTIF(Requirements!D:D,"Partial")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">COUNTIF('Use Cases'!D:D,"Partial")</f>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="B19" s="1" t="n">
         <f aca="false">COUNTIF(Requirements!G:G,"Decision needed")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15632,7 +15632,7 @@
         <v>610</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>611</v>
@@ -15641,7 +15641,7 @@
         <v>612</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>613</v>
@@ -16967,7 +16967,7 @@
         <v>789</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>790</v>
@@ -16976,7 +16976,7 @@
         <v>791</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="H45" s="12"/>
       <c r="I45" s="12" t="s">

</xml_diff>

<commit_message>
Register: main address amsonpharma.web.app
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBZf6oKSsJ7KuyzUF78Kfz
</commit_message>
<xml_diff>
--- a/docs/AMSON-Deviation-Register.xlsx
+++ b/docs/AMSON-Deviation-Register.xlsx
@@ -522,7 +522,7 @@
     <t xml:space="preserve">Deployment: Firebase Hosting (HTTPS) or move hosting to Limitations</t>
   </si>
   <si>
-    <t xml:space="preserve">DECIDED 2026-10-25: Firebase Hosting (free, no per-deploy cost, same project). Netlify dropped: its free plan spends 15 of 300 monthly credits per auto-deploy and paused the site. Deploy: npx firebase-tools deploy --only hosting (README).</t>
+    <t xml:space="preserve">DECIDED 2026-10-25: Firebase Hosting (free, no per-deploy cost, same project). Netlify dropped: its free plan spends 15 of 300 monthly credits per auto-deploy and paused the site. Deploy: npx firebase-tools deploy --only hosting (README). 2026-10-25: main address https://amsonpharma.web.app; the old amson-web-app.web.app gets the same files on each deploy. Both are authorized login domains; add amsonpharma.web.app to the reCAPTCHA checkbox key's domains.</t>
   </si>
   <si>
     <t xml:space="preserve">Report Formats sheet (Discount/Deductions columns); Interview 2</t>
@@ -3531,7 +3531,7 @@
     <t xml:space="preserve">start-server.bat (http-server)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hosted on Firebase Hosting over HTTPS (https://amson-web-app.web.app), 2026-10-25. (was: plain HTTP locally, no hosted deployment.)</t>
+    <t xml:space="preserve">Hosted on Firebase Hosting over HTTPS (https://amsonpharma.web.app), 2026-10-25. (was: plain HTTP locally, no hosted deployment.)</t>
   </si>
   <si>
     <t xml:space="preserve">Resolved by deploying (see REQNF013).</t>

</xml_diff>